<commit_message>
Use 幼稚部 / 小学部 for ELC and Primary in Japanese
Renames the audience labels and updates all Japanese event titles,
descriptions, page text and feeds for consistency. English unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/admin/EIS-Compass-events.xlsx
+++ b/admin/EIS-Compass-events.xlsx
@@ -2007,7 +2007,7 @@
       </c>
       <c r="J24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ELC・初等部カリキュラム説明会</t>
+          <t xml:space="preserve">幼稚部・小学部カリキュラム説明会</t>
         </is>
       </c>
       <c r="K24" t="inlineStr" s="2">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="J33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ELC運動会リハーサル #1</t>
+          <t xml:space="preserve">幼稚部運動会リハーサル #1</t>
         </is>
       </c>
       <c r="K33" t="inlineStr" s="2">
@@ -3155,7 +3155,7 @@
       </c>
       <c r="J38" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ELC運動会リハーサル #2</t>
+          <t xml:space="preserve">幼稚部運動会リハーサル #2</t>
         </is>
       </c>
       <c r="K38" t="inlineStr" s="2">
@@ -3237,7 +3237,7 @@
       </c>
       <c r="J39" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ELC運動会</t>
+          <t xml:space="preserve">幼稚部運動会</t>
         </is>
       </c>
       <c r="K39" t="inlineStr" s="2">
@@ -3657,7 +3657,7 @@
       </c>
       <c r="L44" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ELC・初等部の保護者の皆様をお招きし、朝の授業をご参観いただき、お子様と一緒に朝の日課を体験していただきます。</t>
+          <t xml:space="preserve">幼稚部・小学部の保護者の皆様をお招きし、朝の授業をご参観いただき、お子様と一緒に朝の日課を体験していただきます。</t>
         </is>
       </c>
       <c r="M44" t="inlineStr" s="2">
@@ -4149,7 +4149,7 @@
       </c>
       <c r="L50" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ご家族や地域の皆様が寄付された品物や体験に入札し、初等部生徒会が選んだ取り組みを支援します。</t>
+          <t xml:space="preserve">ご家族や地域の皆様が寄付された品物や体験に入札し、小学部生徒会が選んだ取り組みを支援します。</t>
         </is>
       </c>
       <c r="M50" t="inlineStr" s="2">
@@ -4313,7 +4313,7 @@
       </c>
       <c r="L52" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">イーグルネストごとに、楽しい活動やゲームを通して仲間と交流し、季節を祝います。初等部生徒会が主催します。</t>
+          <t xml:space="preserve">イーグルネストごとに、楽しい活動やゲームを通して仲間と交流し、季節を祝います。小学部生徒会が主催します。</t>
         </is>
       </c>
       <c r="M52" t="inlineStr" s="2">
@@ -5697,7 +5697,7 @@
       </c>
       <c r="J69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">初等部運動会リハーサル #1</t>
+          <t xml:space="preserve">小学部運動会リハーサル #1</t>
         </is>
       </c>
       <c r="K69" t="inlineStr" s="2">
@@ -5789,7 +5789,7 @@
       </c>
       <c r="L70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ELC・初等部の保護者の皆様をお招きし、朝の授業をご参観いただき、お子様と一緒に朝の日課を体験していただきます。</t>
+          <t xml:space="preserve">幼稚部・小学部の保護者の皆様をお招きし、朝の授業をご参観いただき、お子様と一緒に朝の日課を体験していただきます。</t>
         </is>
       </c>
       <c r="M70" t="inlineStr" s="2">
@@ -6189,7 +6189,7 @@
       </c>
       <c r="J75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">初等部運動会リハーサル #2</t>
+          <t xml:space="preserve">小学部運動会リハーサル #2</t>
         </is>
       </c>
       <c r="K75" t="inlineStr" s="2">
@@ -6927,7 +6927,7 @@
       </c>
       <c r="J84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">初等部運動会リハーサル #3</t>
+          <t xml:space="preserve">小学部運動会リハーサル #3</t>
         </is>
       </c>
       <c r="K84" t="inlineStr" s="2">
@@ -7091,7 +7091,7 @@
       </c>
       <c r="J86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">初等部運動会 2027</t>
+          <t xml:space="preserve">小学部運動会 2027</t>
         </is>
       </c>
       <c r="K86" t="inlineStr" s="2">
@@ -8813,7 +8813,7 @@
       </c>
       <c r="J107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">初等部・ELC 年度末発表会</t>
+          <t xml:space="preserve">小学部・幼稚部 年度末発表会</t>
         </is>
       </c>
       <c r="K107" t="inlineStr" s="2">

</xml_diff>

<commit_message>
Polish Japanese event titles
More natural school Japanese for 30 event titles (e.g. 第2回キャリア座談会
instead of セカンドキャリア, 宿泊プログラム, 国際理解フェスティバル,
校内○○大会, 朝の授業参観), stray spaces removed, and matching wording
in the related descriptions. Feeds and spreadsheet regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/admin/EIS-Compass-events.xlsx
+++ b/admin/EIS-Compass-events.xlsx
@@ -367,7 +367,7 @@
       </c>
       <c r="J4" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">オリエンテーション週間・生活指導説明会</t>
+          <t xml:space="preserve">オリエンテーション週間・学校生活説明会</t>
         </is>
       </c>
       <c r="K4" t="inlineStr" s="2">
@@ -777,7 +777,7 @@
       </c>
       <c r="J9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">お気に入りの本を持ってくる日</t>
+          <t xml:space="preserve">お気に入りの本を持ってこよう！</t>
         </is>
       </c>
       <c r="K9" t="inlineStr" s="2">
@@ -951,7 +951,7 @@
       </c>
       <c r="L11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">キーボード操作のスキル、正確さ、自信を高めることを目的とした、親善タイピング大会に参加します。</t>
+          <t xml:space="preserve">キーボード操作のスキル、正確さ、自信を高めることを目的とした、校内タイピング大会に参加します。</t>
         </is>
       </c>
       <c r="M11" t="inlineStr" s="2">
@@ -1105,7 +1105,7 @@
       </c>
       <c r="J13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">校内バスケットボール親善大会</t>
+          <t xml:space="preserve">校内バスケットボール大会</t>
         </is>
       </c>
       <c r="K13" t="inlineStr" s="2">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="L13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">校内でのバスケットボール親善大会に参加し、チームワーク、スポーツマンシップ、愛校心を育みます。</t>
+          <t xml:space="preserve">校内バスケットボール大会に参加し、チームワーク、スポーツマンシップ、愛校心を育みます。</t>
         </is>
       </c>
       <c r="M13" t="inlineStr" s="2">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="J14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">コンセプト・コン（グローバルな視野）</t>
+          <t xml:space="preserve">コンセプト・コン（国際的な視野）</t>
         </is>
       </c>
       <c r="K14" t="inlineStr" s="2">
@@ -1679,7 +1679,7 @@
       </c>
       <c r="J20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">DPラフティング</t>
+          <t xml:space="preserve">DPラフティング体験</t>
         </is>
       </c>
       <c r="K20" t="inlineStr" s="2">
@@ -1761,7 +1761,7 @@
       </c>
       <c r="J21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">進路支援・メンタルヘルス座談会</t>
+          <t xml:space="preserve">進路・メンタルヘルス座談会</t>
         </is>
       </c>
       <c r="K21" t="inlineStr" s="2">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="J27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">大学フェア</t>
+          <t xml:space="preserve">大学進学フェア</t>
         </is>
       </c>
       <c r="K27" t="inlineStr" s="2">
@@ -2499,7 +2499,7 @@
       </c>
       <c r="J30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">豊田高専 見学</t>
+          <t xml:space="preserve">豊田高専見学</t>
         </is>
       </c>
       <c r="K30" t="inlineStr" s="2">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="J32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">インターナショナル・マインドネス・フェスティバル</t>
+          <t xml:space="preserve">国際理解フェスティバル</t>
         </is>
       </c>
       <c r="K32" t="inlineStr" s="2">
@@ -2827,7 +2827,7 @@
       </c>
       <c r="J34" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">トヨタ博物館 校外学習</t>
+          <t xml:space="preserve">トヨタ博物館校外学習</t>
         </is>
       </c>
       <c r="K34" t="inlineStr" s="2">
@@ -2909,7 +2909,7 @@
       </c>
       <c r="J35" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">課外活動：秋のCAS・プロジェクト支援フェア</t>
+          <t xml:space="preserve">課外活動：秋のCAS・プロジェクトサポートフェア</t>
         </is>
       </c>
       <c r="K35" t="inlineStr" s="2">
@@ -3319,7 +3319,7 @@
       </c>
       <c r="J40" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">校内サッカー親善大会</t>
+          <t xml:space="preserve">校内サッカー大会</t>
         </is>
       </c>
       <c r="K40" t="inlineStr" s="2">
@@ -3329,7 +3329,7 @@
       </c>
       <c r="L40" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">校内でのサッカー親善大会に参加し、チームワーク、スポーツマンシップ、愛校心を育みます。</t>
+          <t xml:space="preserve">校内サッカー大会に参加し、チームワーク、スポーツマンシップ、愛校心を育みます。</t>
         </is>
       </c>
       <c r="M40" t="inlineStr" s="2">
@@ -3647,7 +3647,7 @@
       </c>
       <c r="J44" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">保護者モーニング参観 #1</t>
+          <t xml:space="preserve">朝の授業参観 #1</t>
         </is>
       </c>
       <c r="K44" t="inlineStr" s="2">
@@ -3729,7 +3729,7 @@
       </c>
       <c r="J45" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">教員感謝デー</t>
+          <t xml:space="preserve">教職員感謝デー</t>
         </is>
       </c>
       <c r="K45" t="inlineStr" s="2">
@@ -4467,7 +4467,7 @@
       </c>
       <c r="J54" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ティーパーティー／PTA（どなたでも）</t>
+          <t xml:space="preserve">PTAティーパーティー（どなたでも参加できます）</t>
         </is>
       </c>
       <c r="K54" t="inlineStr" s="2">
@@ -4631,7 +4631,7 @@
       </c>
       <c r="J56" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">第1学期末行事 お泊まりプログラム：G6–10</t>
+          <t xml:space="preserve">第1学期末行事：宿泊プログラム（G6–10）</t>
         </is>
       </c>
       <c r="K56" t="inlineStr" s="2">
@@ -4641,7 +4641,7 @@
       </c>
       <c r="L56" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">6～10年生が学校でのお泊まりプログラムに参加し、共に活動しながら仲間づくりを行い、第1学期の終わりを祝います。</t>
+          <t xml:space="preserve">6～10年生が校内での宿泊プログラムに参加し、共に活動しながら仲間づくりを行い、第1学期の終わりを祝います。</t>
         </is>
       </c>
       <c r="M56" t="inlineStr" s="2">
@@ -4795,7 +4795,7 @@
       </c>
       <c r="J58" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">G10保護者説明会（高等部の科目選択）</t>
+          <t xml:space="preserve">G10保護者向け説明会（高等部科目選択）</t>
         </is>
       </c>
       <c r="K58" t="inlineStr" s="2">
@@ -4959,7 +4959,7 @@
       </c>
       <c r="J60" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">卒業生講話</t>
+          <t xml:space="preserve">卒業生トーク</t>
         </is>
       </c>
       <c r="K60" t="inlineStr" s="2">
@@ -5205,7 +5205,7 @@
       </c>
       <c r="J63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">校内バレーボール親善大会</t>
+          <t xml:space="preserve">校内バレーボール大会</t>
         </is>
       </c>
       <c r="K63" t="inlineStr" s="2">
@@ -5215,7 +5215,7 @@
       </c>
       <c r="L63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">校内でのバレーボール親善大会に参加し、チームワーク、スポーツマンシップ、愛校心を育みます。</t>
+          <t xml:space="preserve">校内バレーボール大会に参加し、チームワーク、スポーツマンシップ、愛校心を育みます。</t>
         </is>
       </c>
       <c r="M63" t="inlineStr" s="2">
@@ -5369,7 +5369,7 @@
       </c>
       <c r="J65" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">進路支援：セカンドキャリア座談会・キャリアフェア</t>
+          <t xml:space="preserve">進路支援：第2回キャリア座談会・キャリアフェア</t>
         </is>
       </c>
       <c r="K65" t="inlineStr" s="2">
@@ -5779,7 +5779,7 @@
       </c>
       <c r="J70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">保護者モーニング参観 #2</t>
+          <t xml:space="preserve">朝の授業参観 #2</t>
         </is>
       </c>
       <c r="K70" t="inlineStr" s="2">
@@ -6517,7 +6517,7 @@
       </c>
       <c r="J79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ティーパーティー／PTA（どなたでも）</t>
+          <t xml:space="preserve">PTAティーパーティー（どなたでも参加できます）</t>
         </is>
       </c>
       <c r="K79" t="inlineStr" s="2">
@@ -7419,7 +7419,7 @@
       </c>
       <c r="J90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">生物IA準備 校外学習：海岸の生態系</t>
+          <t xml:space="preserve">生物IA準備校外学習：海岸生態系調査</t>
         </is>
       </c>
       <c r="K90" t="inlineStr" s="2">
@@ -7501,7 +7501,7 @@
       </c>
       <c r="J91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">G12お祝い行事</t>
+          <t xml:space="preserve">G12修了記念イベント</t>
         </is>
       </c>
       <c r="K91" t="inlineStr" s="2">
@@ -7829,7 +7829,7 @@
       </c>
       <c r="J95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">校内バスケットボール親善大会</t>
+          <t xml:space="preserve">校内バスケットボール大会</t>
         </is>
       </c>
       <c r="K95" t="inlineStr" s="2">
@@ -7839,7 +7839,7 @@
       </c>
       <c r="L95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">校内でのバスケットボール親善大会に参加し、チームワーク、スポーツマンシップ、愛校心を育みます。</t>
+          <t xml:space="preserve">校内バスケットボール大会に参加し、チームワーク、スポーツマンシップ、愛校心を育みます。</t>
         </is>
       </c>
       <c r="M95" t="inlineStr" s="2">
@@ -7911,7 +7911,7 @@
       </c>
       <c r="J96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">起業家デー</t>
+          <t xml:space="preserve">アントレプレナーシップ・デー</t>
         </is>
       </c>
       <c r="K96" t="inlineStr" s="2">
@@ -8075,7 +8075,7 @@
       </c>
       <c r="J98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">土曜校 最終日イベント</t>
+          <t xml:space="preserve">土曜校最終日イベント</t>
         </is>
       </c>
       <c r="K98" t="inlineStr" s="2">
@@ -8157,7 +8157,7 @@
       </c>
       <c r="J99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">コンセプト・コン（未来への視点）</t>
+          <t xml:space="preserve">コンセプト・コン（未来を考える）</t>
         </is>
       </c>
       <c r="K99" t="inlineStr" s="2">
@@ -8239,7 +8239,7 @@
       </c>
       <c r="J100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">G12卒業式（パフォーマンス付き）</t>
+          <t xml:space="preserve">G12卒業式・記念パフォーマンス</t>
         </is>
       </c>
       <c r="K100" t="inlineStr" s="2">
@@ -8321,7 +8321,7 @@
       </c>
       <c r="J101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">学びの発表会 準備</t>
+          <t xml:space="preserve">学びの発表会準備</t>
         </is>
       </c>
       <c r="K101" t="inlineStr" s="2">
@@ -8731,7 +8731,7 @@
       </c>
       <c r="J106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">幼稚部・5年生 卒業式</t>
+          <t xml:space="preserve">幼稚部・5年生卒業式</t>
         </is>
       </c>
       <c r="K106" t="inlineStr" s="2">
@@ -8813,7 +8813,7 @@
       </c>
       <c r="J107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">小学部・幼稚部 年度末発表会</t>
+          <t xml:space="preserve">小学部・幼稚部年度末発表会</t>
         </is>
       </c>
       <c r="K107" t="inlineStr" s="2">

</xml_diff>

<commit_message>
Support event times from Excel
- Import converts Excel time values (e.g. 0.625 -> 15:00) and tidies
  9:30, 15:00 - 17:00, 15:00〜17:00 and full-width digits
- Downloaded spreadsheet formats date/time columns as text so Excel
  keeps what is typed; clearer Guide sheet text for the time column
- Upcoming banner no longer repeats "today" on a day off

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/admin/EIS-Compass-events.xlsx
+++ b/admin/EIS-Compass-events.xlsx
@@ -42,11 +42,14 @@
   <cellStyleXfs count="1">
     <xf/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf/>
     <xf fontId="1" fillId="2" applyFont="1" applyFill="1"/>
     <xf applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
 </styleSheet>
@@ -56,9 +59,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="11" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1" style="3"/>
+    <col min="3" max="3" width="12" customWidth="1" style="3"/>
+    <col min="4" max="4" width="13" customWidth="1" style="3"/>
     <col min="5" max="5" width="24" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
@@ -161,17 +164,17 @@
           <t xml:space="preserve">2026-08-12-book-drive</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr" s="2">
+      <c r="B2" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-08-12</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr" s="2">
+      <c r="C2" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-08-12</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr" s="2">
+      <c r="D2" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -243,17 +246,17 @@
           <t xml:space="preserve">2026-08-17-student-orientation-program</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr" s="2">
+      <c r="B3" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-08-17</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr" s="2">
+      <c r="C3" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-08-17</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr" s="2">
+      <c r="D3" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -325,17 +328,17 @@
           <t xml:space="preserve">2026-08-17-orientation-week-welfare-briefing</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr" s="2">
+      <c r="B4" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-08-17</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr" s="2">
+      <c r="C4" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-08-21</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr" s="2">
+      <c r="D4" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -407,17 +410,17 @@
           <t xml:space="preserve">2026-08-22-sat-test-1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr" s="2">
+      <c r="B5" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-08-22</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr" s="2">
+      <c r="C5" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-08-22</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr" s="2">
+      <c r="D5" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -489,17 +492,17 @@
           <t xml:space="preserve">2026-08-24-book-drive</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr" s="2">
+      <c r="B6" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-08-24</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr" s="2">
+      <c r="C6" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-08-24</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr" s="2">
+      <c r="D6" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -571,17 +574,17 @@
           <t xml:space="preserve">2026-08-24-jigsaw-competition</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr" s="2">
+      <c r="B7" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-08-24</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr" s="2">
+      <c r="C7" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-08-24</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr" s="2">
+      <c r="D7" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -653,17 +656,17 @@
           <t xml:space="preserve">2026-08-28-movie-night</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr" s="2">
+      <c r="B8" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-08-28</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr" s="2">
+      <c r="C8" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-08-28</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr" s="2">
+      <c r="D8" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -735,17 +738,17 @@
           <t xml:space="preserve">2026-09-01-bring-your-favourite-book-day</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr" s="2">
+      <c r="B9" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-09-01</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr" s="2">
+      <c r="C9" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-09-01</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr" s="2">
+      <c r="D9" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -817,17 +820,17 @@
           <t xml:space="preserve">2026-09-04-art-workshop</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr" s="2">
+      <c r="B10" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-09-04</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr" s="2">
+      <c r="C10" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-09-04</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr" s="2">
+      <c r="D10" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -899,17 +902,17 @@
           <t xml:space="preserve">2026-09-09-speed-typing-competition</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr" s="2">
+      <c r="B11" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr" s="2">
+      <c r="C11" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr" s="2">
+      <c r="D11" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -981,17 +984,17 @@
           <t xml:space="preserve">2026-09-12-sat-test-2</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr" s="2">
+      <c r="B12" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-09-12</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr" s="2">
+      <c r="C12" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-09-12</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr" s="2">
+      <c r="D12" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1063,17 +1066,17 @@
           <t xml:space="preserve">2026-09-14-friendly-basketball-tournament-internal</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr" s="2">
+      <c r="B13" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-09-14</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr" s="2">
+      <c r="C13" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-09-18</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr" s="2">
+      <c r="D13" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1145,17 +1148,17 @@
           <t xml:space="preserve">2026-09-14-concept-con-global-mindedness</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr" s="2">
+      <c r="B14" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-09-14</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr" s="2">
+      <c r="C14" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-09-18</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr" s="2">
+      <c r="D14" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1227,17 +1230,17 @@
           <t xml:space="preserve">2026-09-18-coffee-hour</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr" s="2">
+      <c r="B15" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-09-18</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr" s="2">
+      <c r="C15" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-09-18</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr" s="2">
+      <c r="D15" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1309,17 +1312,17 @@
           <t xml:space="preserve">2026-09-25-open-campus</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr" s="2">
+      <c r="B16" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-09-25</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr" s="2">
+      <c r="C16" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-09-25</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr" s="2">
+      <c r="D16" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1391,17 +1394,17 @@
           <t xml:space="preserve">2026-09-28-spirit-week</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr" s="2">
+      <c r="B17" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-09-28</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr" s="2">
+      <c r="C17" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-09-30</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr" s="2">
+      <c r="D17" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1473,17 +1476,17 @@
           <t xml:space="preserve">2026-10-03-world-tea-party</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr" s="2">
+      <c r="B18" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-03</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr" s="2">
+      <c r="C18" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-03</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr" s="2">
+      <c r="D18" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1555,17 +1558,17 @@
           <t xml:space="preserve">2026-10-03-sat-test-3</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr" s="2">
+      <c r="B19" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-03</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr" s="2">
+      <c r="C19" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-03</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr" s="2">
+      <c r="D19" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1637,17 +1640,17 @@
           <t xml:space="preserve">2026-10-03-dp-rafting-trip</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr" s="2">
+      <c r="B20" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-03</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr" s="2">
+      <c r="C20" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-03</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr" s="2">
+      <c r="D20" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1719,17 +1722,17 @@
           <t xml:space="preserve">2026-10-07-career-support-and-mental-health-round-table</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr" s="2">
+      <c r="B21" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-07</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr" s="2">
+      <c r="C21" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-07</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr" s="2">
+      <c r="D21" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1801,17 +1804,17 @@
           <t xml:space="preserve">2026-10-09-high-school-curriculum-night</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr" s="2">
+      <c r="B22" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr" s="2">
+      <c r="C22" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr" s="2">
+      <c r="D22" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1883,17 +1886,17 @@
           <t xml:space="preserve">2026-10-09-eagle-bucks-store</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr" s="2">
+      <c r="B23" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr" s="2">
+      <c r="C23" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr" s="2">
+      <c r="D23" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1965,17 +1968,17 @@
           <t xml:space="preserve">2026-10-19-elc-primary-curriculum-night</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr" s="2">
+      <c r="B24" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-19</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr" s="2">
+      <c r="C24" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-19</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr" s="2">
+      <c r="D24" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -2047,17 +2050,17 @@
           <t xml:space="preserve">2026-10-19-parent-teacher-conferences</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr" s="2">
+      <c r="B25" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-19</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr" s="2">
+      <c r="C25" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-19</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr" s="2">
+      <c r="D25" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -2129,17 +2132,17 @@
           <t xml:space="preserve">2026-10-20-secondary-curriculum-night</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr" s="2">
+      <c r="B26" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-20</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr" s="2">
+      <c r="C26" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-20</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr" s="2">
+      <c r="D26" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -2211,17 +2214,17 @@
           <t xml:space="preserve">2026-10-21-college-fair</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr" s="2">
+      <c r="B27" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-21</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr" s="2">
+      <c r="C27" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-21</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr" s="2">
+      <c r="D27" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -2293,17 +2296,17 @@
           <t xml:space="preserve">2026-10-23-nagoya-university-biology-laboratory-visit</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr" s="2">
+      <c r="B28" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-23</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr" s="2">
+      <c r="C28" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-23</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr" s="2">
+      <c r="D28" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -2375,17 +2378,17 @@
           <t xml:space="preserve">2026-10-25-pta-picnic</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr" s="2">
+      <c r="B29" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-25</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr" s="2">
+      <c r="C29" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-25</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr" s="2">
+      <c r="D29" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -2457,17 +2460,17 @@
           <t xml:space="preserve">2026-10-26-toyota-college-trip</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr" s="2">
+      <c r="B30" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-26</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr" s="2">
+      <c r="C30" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-26</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr" s="2">
+      <c r="D30" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -2539,17 +2542,17 @@
           <t xml:space="preserve">2026-10-30-sensory-wonderland</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr" s="2">
+      <c r="B31" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-30</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr" s="2">
+      <c r="C31" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-30</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr" s="2">
+      <c r="D31" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -2621,17 +2624,17 @@
           <t xml:space="preserve">2026-10-31-international-mindedness-festival</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr" s="2">
+      <c r="B32" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-31</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr" s="2">
+      <c r="C32" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-31</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr" s="2">
+      <c r="D32" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -2703,17 +2706,17 @@
           <t xml:space="preserve">2026-11-04-elc-sports-day-rehearsal-1</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr" s="2">
+      <c r="B33" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-04</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr" s="2">
+      <c r="C33" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-04</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr" s="2">
+      <c r="D33" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -2785,17 +2788,17 @@
           <t xml:space="preserve">2026-11-05-toyota-museum-field-trip</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr" s="2">
+      <c r="B34" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-05</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr" s="2">
+      <c r="C34" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-05</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr" s="2">
+      <c r="D34" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -2867,17 +2870,17 @@
           <t xml:space="preserve">2026-11-06-extracurricular-activities-autumn-cas-project-su</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr" s="2">
+      <c r="B35" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-06</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr" s="2">
+      <c r="C35" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-06</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr" s="2">
+      <c r="D35" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -2949,17 +2952,17 @@
           <t xml:space="preserve">2026-11-07-sat-test-4</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr" s="2">
+      <c r="B36" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-07</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr" s="2">
+      <c r="C36" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-07</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr" s="2">
+      <c r="D36" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -3031,17 +3034,17 @@
           <t xml:space="preserve">2026-11-09-wellbeing-week</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr" s="2">
+      <c r="B37" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-09</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr" s="2">
+      <c r="C37" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-13</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr" s="2">
+      <c r="D37" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -3113,17 +3116,17 @@
           <t xml:space="preserve">2026-11-11-elc-sports-day-rehearsal-2</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr" s="2">
+      <c r="B38" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-11</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr" s="2">
+      <c r="C38" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-11</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr" s="2">
+      <c r="D38" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -3195,17 +3198,17 @@
           <t xml:space="preserve">2026-11-14-elc-sports-day</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr" s="2">
+      <c r="B39" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-14</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr" s="2">
+      <c r="C39" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-14</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr" s="2">
+      <c r="D39" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -3277,17 +3280,17 @@
           <t xml:space="preserve">2026-11-16-friendly-soccer-tournament-internal</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr" s="2">
+      <c r="B40" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-16</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr" s="2">
+      <c r="C40" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-20</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr" s="2">
+      <c r="D40" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -3359,17 +3362,17 @@
           <t xml:space="preserve">2026-11-17-foundation-field-trip</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr" s="2">
+      <c r="B41" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-17</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr" s="2">
+      <c r="C41" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-17</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr" s="2">
+      <c r="D41" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -3441,17 +3444,17 @@
           <t xml:space="preserve">2026-11-20-gifu-kakamigahara-air-and-space-museum</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr" s="2">
+      <c r="B42" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-20</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr" s="2">
+      <c r="C42" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-20</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr" s="2">
+      <c r="D42" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -3523,17 +3526,17 @@
           <t xml:space="preserve">2026-11-24-winter-art-contest</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr" s="2">
+      <c r="B43" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-24</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr" s="2">
+      <c r="C43" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-25</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr" s="2">
+      <c r="D43" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -3605,17 +3608,17 @@
           <t xml:space="preserve">2026-11-27-parents-morning-1</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr" s="2">
+      <c r="B44" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-27</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr" s="2">
+      <c r="C44" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-27</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr" s="2">
+      <c r="D44" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -3687,17 +3690,17 @@
           <t xml:space="preserve">2026-11-27-teacher-appreciation-day</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr" s="2">
+      <c r="B45" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-27</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr" s="2">
+      <c r="C45" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-27</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr" s="2">
+      <c r="D45" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -3769,17 +3772,17 @@
           <t xml:space="preserve">2026-11-28-2026-enishi-futsal-tournament</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr" s="2">
+      <c r="B46" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-28</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr" s="2">
+      <c r="C46" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-28</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr" s="2">
+      <c r="D46" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -3851,17 +3854,17 @@
           <t xml:space="preserve">2026-12-03-grade-3-4-musical</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr" s="2">
+      <c r="B47" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-12-03</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr" s="2">
+      <c r="C47" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-12-04</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr" s="2">
+      <c r="D47" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -3933,17 +3936,17 @@
           <t xml:space="preserve">2026-12-05-sat-test-5</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr" s="2">
+      <c r="B48" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-12-05</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr" s="2">
+      <c r="C48" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-12-05</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr" s="2">
+      <c r="D48" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -4015,17 +4018,17 @@
           <t xml:space="preserve">2026-12-10-choir-and-orchestra-concert</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr" s="2">
+      <c r="B49" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-12-10</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr" s="2">
+      <c r="C49" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-12-10</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr" s="2">
+      <c r="D49" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -4097,17 +4100,17 @@
           <t xml:space="preserve">2026-12-11-silent-auction</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr" s="2">
+      <c r="B50" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-12-11</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr" s="2">
+      <c r="C50" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-12-11</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr" s="2">
+      <c r="D50" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -4179,17 +4182,17 @@
           <t xml:space="preserve">2026-12-16-industry-visit-tech-company</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr" s="2">
+      <c r="B51" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-12-16</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr" s="2">
+      <c r="C51" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-12-16</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr" s="2">
+      <c r="D51" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -4261,17 +4264,17 @@
           <t xml:space="preserve">2026-12-16-winter-party-eagle-nest</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr" s="2">
+      <c r="B52" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-12-16</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr" s="2">
+      <c r="C52" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-12-16</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr" s="2">
+      <c r="D52" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -4343,17 +4346,17 @@
           <t xml:space="preserve">2026-12-17-talent-day</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr" s="2">
+      <c r="B53" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-12-17</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr" s="2">
+      <c r="C53" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-12-17</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr" s="2">
+      <c r="D53" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -4425,17 +4428,17 @@
           <t xml:space="preserve">2026-12-18-tea-party-pta-for-all</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr" s="2">
+      <c r="B54" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-12-18</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr" s="2">
+      <c r="C54" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-12-18</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr" s="2">
+      <c r="D54" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -4507,17 +4510,17 @@
           <t xml:space="preserve">2026-12-18-eagle-bucks-store</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr" s="2">
+      <c r="B55" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-12-18</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr" s="2">
+      <c r="C55" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-12-18</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr" s="2">
+      <c r="D55" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -4589,17 +4592,17 @@
           <t xml:space="preserve">2026-12-19-end-of-term-1-activity-sleep-over-program-g6-10</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr" s="2">
+      <c r="B56" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-12-19</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr" s="2">
+      <c r="C56" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-12-19</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr" s="2">
+      <c r="D56" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -4671,17 +4674,17 @@
           <t xml:space="preserve">2026-12-21-winter-study-camp-g11-12</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr" s="2">
+      <c r="B57" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-12-21</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr" s="2">
+      <c r="C57" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-12-23</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr" s="2">
+      <c r="D57" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -4753,17 +4756,17 @@
           <t xml:space="preserve">2027-01-14-g10-parent-info-session-high-school-subject-choi</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr" s="2">
+      <c r="B58" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-01-14</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr" s="2">
+      <c r="C58" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-01-14</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr" s="2">
+      <c r="D58" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -4835,17 +4838,17 @@
           <t xml:space="preserve">2027-01-22-open-campus</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr" s="2">
+      <c r="B59" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-01-22</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr" s="2">
+      <c r="C59" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-01-22</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr" s="2">
+      <c r="D59" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -4917,17 +4920,17 @@
           <t xml:space="preserve">2027-01-23-alumni-talk</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr" s="2">
+      <c r="B60" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-01-23</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr" s="2">
+      <c r="C60" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-01-23</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr" s="2">
+      <c r="D60" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -4999,17 +5002,17 @@
           <t xml:space="preserve">2027-01-27-natural-disaster-field-trip</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr" s="2">
+      <c r="B61" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-01-27</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr" s="2">
+      <c r="C61" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-01-27</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr" s="2">
+      <c r="D61" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5081,17 +5084,17 @@
           <t xml:space="preserve">2027-01-30-model-united-nations-event-mun</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr" s="2">
+      <c r="B62" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-01-30</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr" s="2">
+      <c r="C62" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-01-30</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr" s="2">
+      <c r="D62" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5163,17 +5166,17 @@
           <t xml:space="preserve">2027-02-01-friendly-volleyball-tournament-internal</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr" s="2">
+      <c r="B63" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-02-01</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr" s="2">
+      <c r="C63" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-02-05</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr" s="2">
+      <c r="D63" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5245,17 +5248,17 @@
           <t xml:space="preserve">2027-02-01-concept-con-language</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr" s="2">
+      <c r="B64" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-02-01</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr" s="2">
+      <c r="C64" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-02-05</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr" s="2">
+      <c r="D64" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5327,17 +5330,17 @@
           <t xml:space="preserve">2027-02-18-career-support-second-career-roundtable-and-care</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr" s="2">
+      <c r="B65" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-02-18</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr" s="2">
+      <c r="C65" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-02-18</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr" s="2">
+      <c r="D65" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5409,17 +5412,17 @@
           <t xml:space="preserve">2027-02-19-collective-field-trip</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr" s="2">
+      <c r="B66" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-02-19</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr" s="2">
+      <c r="C66" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-02-19</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr" s="2">
+      <c r="D66" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5491,17 +5494,17 @@
           <t xml:space="preserve">2027-02-22-world-thinking-day</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr" s="2">
+      <c r="B67" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-02-22</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr" s="2">
+      <c r="C67" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-02-22</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr" s="2">
+      <c r="D67" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5573,17 +5576,17 @@
           <t xml:space="preserve">2027-02-22-secondary-sports-day-rehearsal-1</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr" s="2">
+      <c r="B68" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-02-22</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr" s="2">
+      <c r="C68" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-02-22</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr" s="2">
+      <c r="D68" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5655,17 +5658,17 @@
           <t xml:space="preserve">2027-02-25-primary-sports-day-rehearsal-1</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr" s="2">
+      <c r="B69" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-02-25</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr" s="2">
+      <c r="C69" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-02-25</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr" s="2">
+      <c r="D69" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5737,17 +5740,17 @@
           <t xml:space="preserve">2027-02-26-parents-morning-2</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr" s="2">
+      <c r="B70" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-02-26</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr" s="2">
+      <c r="C70" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-02-26</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr" s="2">
+      <c r="D70" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5819,17 +5822,17 @@
           <t xml:space="preserve">2027-02-26-eagle-talks</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr" s="2">
+      <c r="B71" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-02-26</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr" s="2">
+      <c r="C71" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-02-26</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr" s="2">
+      <c r="D71" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5901,17 +5904,17 @@
           <t xml:space="preserve">2027-03-04-grade-1-2-musical</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr" s="2">
+      <c r="B72" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-04</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr" s="2">
+      <c r="C72" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-05</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr" s="2">
+      <c r="D72" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -5983,17 +5986,17 @@
           <t xml:space="preserve">2027-03-05-higashiyama-zoo-botanical-garden</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr" s="2">
+      <c r="B73" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-05</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr" s="2">
+      <c r="C73" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-05</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr" s="2">
+      <c r="D73" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6065,17 +6068,17 @@
           <t xml:space="preserve">2027-03-06-sat-test-6</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr" s="2">
+      <c r="B74" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-06</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr" s="2">
+      <c r="C74" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-06</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr" s="2">
+      <c r="D74" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6147,17 +6150,17 @@
           <t xml:space="preserve">2027-03-09-primary-sports-day-rehearsal-2</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr" s="2">
+      <c r="B75" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-09</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr" s="2">
+      <c r="C75" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-09</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr" s="2">
+      <c r="D75" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6229,17 +6232,17 @@
           <t xml:space="preserve">2027-03-12-secondary-sports-day-rehearsal-2</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr" s="2">
+      <c r="B76" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-12</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr" s="2">
+      <c r="C76" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-12</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr" s="2">
+      <c r="D76" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6311,17 +6314,17 @@
           <t xml:space="preserve">2027-03-18-japanese-culture-day</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr" s="2">
+      <c r="B77" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-18</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr" s="2">
+      <c r="C77" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-18</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr" s="2">
+      <c r="D77" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6393,17 +6396,17 @@
           <t xml:space="preserve">2027-03-19-eagle-bucks-store</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr" s="2">
+      <c r="B78" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-19</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr" s="2">
+      <c r="C78" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-19</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr" s="2">
+      <c r="D78" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6475,17 +6478,17 @@
           <t xml:space="preserve">2027-03-19-tea-party-pta-for-all</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr" s="2">
+      <c r="B79" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-19</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr" s="2">
+      <c r="C79" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-19</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr" s="2">
+      <c r="D79" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6557,17 +6560,17 @@
           <t xml:space="preserve">2027-03-19-end-of-term-2-activity-g9-12</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr" s="2">
+      <c r="B80" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-19</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr" s="2">
+      <c r="C80" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-20</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr" s="2">
+      <c r="D80" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6639,17 +6642,17 @@
           <t xml:space="preserve">2027-03-20-end-of-term-2-activity-g6-8</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr" s="2">
+      <c r="B81" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-20</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr" s="2">
+      <c r="C81" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-21</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr" s="2">
+      <c r="D81" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6721,17 +6724,17 @@
           <t xml:space="preserve">2027-03-30-parent-teacher-conferences</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr" s="2">
+      <c r="B82" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-30</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr" s="2">
+      <c r="C82" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-30</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr" s="2">
+      <c r="D82" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6803,17 +6806,17 @@
           <t xml:space="preserve">2027-03-31-secondary-sports-day-rehearsal-3</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr" s="2">
+      <c r="B83" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-31</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr" s="2">
+      <c r="C83" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-31</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr" s="2">
+      <c r="D83" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6885,17 +6888,17 @@
           <t xml:space="preserve">2027-04-01-primary-sports-day-rehearsal-3</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr" s="2">
+      <c r="B84" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-04-01</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr" s="2">
+      <c r="C84" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-04-01</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr" s="2">
+      <c r="D84" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6967,17 +6970,17 @@
           <t xml:space="preserve">2027-04-03-sports-day</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr" s="2">
+      <c r="B85" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-04-03</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr" s="2">
+      <c r="C85" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-04-03</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr" s="2">
+      <c r="D85" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -7049,17 +7052,17 @@
           <t xml:space="preserve">2027-04-03-primary-sports-day-2027</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr" s="2">
+      <c r="B86" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-04-03</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr" s="2">
+      <c r="C86" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-04-03</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr" s="2">
+      <c r="D86" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -7131,17 +7134,17 @@
           <t xml:space="preserve">2027-04-15-world-art-day</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr" s="2">
+      <c r="B87" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-04-15</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr" s="2">
+      <c r="C87" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-04-15</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr" s="2">
+      <c r="D87" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -7213,17 +7216,17 @@
           <t xml:space="preserve">2027-04-16-foundation-field-trip</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr" s="2">
+      <c r="B88" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-04-16</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr" s="2">
+      <c r="C88" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-04-16</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr" s="2">
+      <c r="D88" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -7295,17 +7298,17 @@
           <t xml:space="preserve">2027-04-21-hackathon-hour-of-code</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr" s="2">
+      <c r="B89" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-04-21</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr" s="2">
+      <c r="C89" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-04-21</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr" s="2">
+      <c r="D89" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -7377,17 +7380,17 @@
           <t xml:space="preserve">2027-04-22-biology-ia-prep-field-trip-shore-ecosystem</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr" s="2">
+      <c r="B90" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-04-22</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr" s="2">
+      <c r="C90" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-04-22</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr" s="2">
+      <c r="D90" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -7459,17 +7462,17 @@
           <t xml:space="preserve">2027-04-23-g12-celebration</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr" s="2">
+      <c r="B91" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-04-23</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr" s="2">
+      <c r="C91" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-04-23</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr" s="2">
+      <c r="D91" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -7541,17 +7544,17 @@
           <t xml:space="preserve">2027-04-26-grade-4-5-camping-trip</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr" s="2">
+      <c r="B92" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-04-26</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr" s="2">
+      <c r="C92" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-04-27</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr" s="2">
+      <c r="D92" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -7623,17 +7626,17 @@
           <t xml:space="preserve">2027-04-27-choir-and-orchestra-concert</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr" s="2">
+      <c r="B93" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-04-27</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr" s="2">
+      <c r="C93" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-04-27</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr" s="2">
+      <c r="D93" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -7705,17 +7708,17 @@
           <t xml:space="preserve">2027-04-30-science-fair</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr" s="2">
+      <c r="B94" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-04-30</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr" s="2">
+      <c r="C94" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-04-30</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr" s="2">
+      <c r="D94" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -7787,17 +7790,17 @@
           <t xml:space="preserve">2027-05-17-friendly-basketball-tournament-internal</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr" s="2">
+      <c r="B95" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-05-17</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr" s="2">
+      <c r="C95" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-05-21</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr" s="2">
+      <c r="D95" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -7869,17 +7872,17 @@
           <t xml:space="preserve">2027-05-19-entrepreneurs-day</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr" s="2">
+      <c r="B96" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-05-19</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr" s="2">
+      <c r="C96" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-05-20</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr" s="2">
+      <c r="D96" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -7951,17 +7954,17 @@
           <t xml:space="preserve">2027-05-21-collective-field-trip</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr" s="2">
+      <c r="B97" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-05-21</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr" s="2">
+      <c r="C97" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-05-21</t>
         </is>
       </c>
-      <c r="D97" t="inlineStr" s="2">
+      <c r="D97" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -8033,17 +8036,17 @@
           <t xml:space="preserve">2027-05-22-saturday-school-last-day-event</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr" s="2">
+      <c r="B98" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-05-22</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr" s="2">
+      <c r="C98" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-05-22</t>
         </is>
       </c>
-      <c r="D98" t="inlineStr" s="2">
+      <c r="D98" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -8115,17 +8118,17 @@
           <t xml:space="preserve">2027-05-24-concept-con-future-focus</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr" s="2">
+      <c r="B99" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-05-24</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr" s="2">
+      <c r="C99" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-05-28</t>
         </is>
       </c>
-      <c r="D99" t="inlineStr" s="2">
+      <c r="D99" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -8197,17 +8200,17 @@
           <t xml:space="preserve">2027-05-28-g12-graduation-with-performances</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr" s="2">
+      <c r="B100" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-05-28</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr" s="2">
+      <c r="C100" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-05-28</t>
         </is>
       </c>
-      <c r="D100" t="inlineStr" s="2">
+      <c r="D100" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -8279,17 +8282,17 @@
           <t xml:space="preserve">2027-06-03-celebration-of-learning-prep</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr" s="2">
+      <c r="B101" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-06-03</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr" s="2">
+      <c r="C101" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-06-03</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr" s="2">
+      <c r="D101" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -8361,17 +8364,17 @@
           <t xml:space="preserve">2027-06-03-ukulele-concert</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr" s="2">
+      <c r="B102" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-06-03</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr" s="2">
+      <c r="C102" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-06-04</t>
         </is>
       </c>
-      <c r="D102" t="inlineStr" s="2">
+      <c r="D102" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -8443,17 +8446,17 @@
           <t xml:space="preserve">2027-06-04-celebration-of-learning</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr" s="2">
+      <c r="B103" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-06-04</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr" s="2">
+      <c r="C103" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-06-04</t>
         </is>
       </c>
-      <c r="D103" t="inlineStr" s="2">
+      <c r="D103" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -8525,17 +8528,17 @@
           <t xml:space="preserve">2027-06-05-sat-test-7</t>
         </is>
       </c>
-      <c r="B104" t="inlineStr" s="2">
+      <c r="B104" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-06-05</t>
         </is>
       </c>
-      <c r="C104" t="inlineStr" s="2">
+      <c r="C104" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-06-05</t>
         </is>
       </c>
-      <c r="D104" t="inlineStr" s="2">
+      <c r="D104" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -8607,17 +8610,17 @@
           <t xml:space="preserve">2027-06-17-eagle-bucks-store</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr" s="2">
+      <c r="B105" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-06-17</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr" s="2">
+      <c r="C105" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-06-17</t>
         </is>
       </c>
-      <c r="D105" t="inlineStr" s="2">
+      <c r="D105" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -8689,17 +8692,17 @@
           <t xml:space="preserve">2027-06-18-kindergarten-and-grade-5-graduation</t>
         </is>
       </c>
-      <c r="B106" t="inlineStr" s="2">
+      <c r="B106" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-06-18</t>
         </is>
       </c>
-      <c r="C106" t="inlineStr" s="2">
+      <c r="C106" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-06-18</t>
         </is>
       </c>
-      <c r="D106" t="inlineStr" s="2">
+      <c r="D106" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -8771,17 +8774,17 @@
           <t xml:space="preserve">2027-06-18-primary-elc-year-end-performance</t>
         </is>
       </c>
-      <c r="B107" t="inlineStr" s="2">
+      <c r="B107" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-06-18</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr" s="2">
+      <c r="C107" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-06-18</t>
         </is>
       </c>
-      <c r="D107" t="inlineStr" s="2">
+      <c r="D107" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -8853,17 +8856,17 @@
           <t xml:space="preserve">2027-06-19-end-of-term-3-activity-g6-10</t>
         </is>
       </c>
-      <c r="B108" t="inlineStr" s="2">
+      <c r="B108" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-06-19</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr" s="2">
+      <c r="C108" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-06-19</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr" s="2">
+      <c r="D108" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -8935,17 +8938,17 @@
           <t xml:space="preserve">2027-06-22-parent-teacher-conferences</t>
         </is>
       </c>
-      <c r="B109" t="inlineStr" s="2">
+      <c r="B109" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-06-22</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr" s="2">
+      <c r="C109" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-06-23</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr" s="2">
+      <c r="D109" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -9017,17 +9020,17 @@
           <t xml:space="preserve">2027-06-28-summer-school</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr" s="2">
+      <c r="B110" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-06-28</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr" s="2">
+      <c r="C110" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-07-24</t>
         </is>
       </c>
-      <c r="D110" t="inlineStr" s="2">
+      <c r="D110" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -9100,8 +9103,8 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="1" max="1" width="12" customWidth="1" style="3"/>
+    <col min="2" max="2" width="12" customWidth="1" style="3"/>
     <col min="3" max="3" width="10" customWidth="1"/>
     <col min="4" max="4" width="32" customWidth="1"/>
     <col min="5" max="5" width="24" customWidth="1"/>
@@ -9135,12 +9138,12 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr" s="2">
+      <c r="A2" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-09-21</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr" s="2">
+      <c r="B2" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-09-21</t>
         </is>
@@ -9162,12 +9165,12 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr" s="2">
+      <c r="A3" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-09-22</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr" s="2">
+      <c r="B3" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-09-22</t>
         </is>
@@ -9189,12 +9192,12 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr" s="2">
+      <c r="A4" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr" s="2">
+      <c r="B4" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-12</t>
         </is>
@@ -9216,12 +9219,12 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr" s="2">
+      <c r="A5" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-13</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr" s="2">
+      <c r="B5" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-10-16</t>
         </is>
@@ -9243,12 +9246,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr" s="2">
+      <c r="A6" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-03</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr" s="2">
+      <c r="B6" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-03</t>
         </is>
@@ -9270,12 +9273,12 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr" s="2">
+      <c r="A7" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-23</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr" s="2">
+      <c r="B7" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-11-23</t>
         </is>
@@ -9297,12 +9300,12 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr" s="2">
+      <c r="A8" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-12-21</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr" s="2">
+      <c r="B8" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-12-25</t>
         </is>
@@ -9324,12 +9327,12 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr" s="2">
+      <c r="A9" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-12-28</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr" s="2">
+      <c r="B9" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2026-12-31</t>
         </is>
@@ -9351,12 +9354,12 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr" s="2">
+      <c r="A10" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-01-01</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr" s="2">
+      <c r="B10" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-01-01</t>
         </is>
@@ -9378,12 +9381,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr" s="2">
+      <c r="A11" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-01-04</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr" s="2">
+      <c r="B11" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-01-06</t>
         </is>
@@ -9405,12 +9408,12 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr" s="2">
+      <c r="A12" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-02-11</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr" s="2">
+      <c r="B12" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-02-11</t>
         </is>
@@ -9432,12 +9435,12 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr" s="2">
+      <c r="A13" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-02-23</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr" s="2">
+      <c r="B13" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-02-23</t>
         </is>
@@ -9459,12 +9462,12 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr" s="2">
+      <c r="A14" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-21</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr" s="2">
+      <c r="B14" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-21</t>
         </is>
@@ -9486,12 +9489,12 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr" s="2">
+      <c r="A15" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-22</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr" s="2">
+      <c r="B15" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-26</t>
         </is>
@@ -9513,12 +9516,12 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr" s="2">
+      <c r="A16" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-29</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr" s="2">
+      <c r="B16" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-03-29</t>
         </is>
@@ -9540,12 +9543,12 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr" s="2">
+      <c r="A17" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-05-03</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr" s="2">
+      <c r="B17" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-05-03</t>
         </is>
@@ -9567,12 +9570,12 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr" s="2">
+      <c r="A18" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-05-04</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr" s="2">
+      <c r="B18" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-05-04</t>
         </is>
@@ -9594,12 +9597,12 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr" s="2">
+      <c r="A19" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-05-05</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr" s="2">
+      <c r="B19" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-05-05</t>
         </is>
@@ -9621,12 +9624,12 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr" s="2">
+      <c r="A20" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-05-06</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr" s="2">
+      <c r="B20" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-05-07</t>
         </is>
@@ -9648,12 +9651,12 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr" s="2">
+      <c r="A21" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-06-06</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr" s="2">
+      <c r="B21" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-06-07</t>
         </is>
@@ -9675,12 +9678,12 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr" s="2">
+      <c r="A22" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-06-21</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr" s="2">
+      <c r="B22" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-06-21</t>
         </is>
@@ -9702,12 +9705,12 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr" s="2">
+      <c r="A23" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-06-24</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr" s="2">
+      <c r="B23" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-06-25</t>
         </is>
@@ -9729,12 +9732,12 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr" s="2">
+      <c r="A24" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-07-19</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr" s="2">
+      <c r="B24" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-07-19</t>
         </is>
@@ -9756,12 +9759,12 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr" s="2">
+      <c r="A25" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-07-26</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr" s="2">
+      <c r="B25" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-07-30</t>
         </is>
@@ -9837,7 +9840,7 @@
       </c>
       <c r="B4" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Optional, e.g. 15:00 or 15:00-17:00. Empty = all day.</t>
+          <t xml:space="preserve">Optional. 24-hour time: 15:00 for a start time, or 15:00-17:00 for start and end. Leave empty for all-day events (most events). Shown on the website and in subscribed calendars.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add up to three links per event (flyers, forms, extra info)
- Spreadsheet: link_1, link_2, link_3 columns; "URL", "Label | URL" or
  "English | 日本語 | URL"; Excel hyperlinks and HYPERLINK() formulas
  are read; older spreadsheets without link columns keep existing links
- Event window: "More information" buttons with automatic bilingual
  names for PDFs, forms, documents, videos and email
- Admin: link fields in the edit form, checks for invalid addresses,
  links included in feeds and Add to Google Calendar details

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/admin/EIS-Compass-events.xlsx
+++ b/admin/EIS-Compass-events.xlsx
@@ -73,7 +73,10 @@
     <col min="13" max="13" width="20" customWidth="1"/>
     <col min="14" max="14" width="20" customWidth="1"/>
     <col min="15" max="15" width="30" customWidth="1"/>
-    <col min="16" max="16" width="8" customWidth="1"/>
+    <col min="16" max="16" width="40" customWidth="1"/>
+    <col min="17" max="17" width="40" customWidth="1"/>
+    <col min="18" max="18" width="40" customWidth="1"/>
+    <col min="19" max="19" width="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -154,6 +157,21 @@
       </c>
       <c r="P1" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">link_1</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">link_2</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">link_3</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">hidden</t>
         </is>
       </c>
@@ -239,6 +257,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr" s="2">
@@ -321,6 +354,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr" s="2">
@@ -403,6 +451,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q4" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr" s="2">
@@ -485,6 +548,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr" s="2">
@@ -567,6 +645,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr" s="2">
@@ -649,6 +742,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr" s="2">
@@ -731,6 +839,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr" s="2">
@@ -813,6 +936,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr" s="2">
@@ -895,6 +1033,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr" s="2">
@@ -977,6 +1130,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr" s="2">
@@ -1059,6 +1227,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr" s="2">
@@ -1141,6 +1324,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr" s="2">
@@ -1223,6 +1421,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr" s="2">
@@ -1305,6 +1518,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr" s="2">
@@ -1387,6 +1615,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr" s="2">
@@ -1469,6 +1712,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q17" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr" s="2">
@@ -1551,6 +1809,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q18" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr" s="2">
@@ -1633,6 +1906,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q19" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr" s="2">
@@ -1715,6 +2003,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q20" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr" s="2">
@@ -1797,6 +2100,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q21" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr" s="2">
@@ -1879,6 +2197,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q22" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr" s="2">
@@ -1961,6 +2294,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q23" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr" s="2">
@@ -2043,6 +2391,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q24" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr" s="2">
@@ -2125,6 +2488,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q25" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr" s="2">
@@ -2207,6 +2585,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q26" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr" s="2">
@@ -2289,6 +2682,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q27" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr" s="2">
@@ -2371,6 +2779,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q28" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr" s="2">
@@ -2453,6 +2876,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q29" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr" s="2">
@@ -2535,6 +2973,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q30" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr" s="2">
@@ -2617,6 +3070,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q31" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr" s="2">
@@ -2699,6 +3167,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q32" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr" s="2">
@@ -2781,6 +3264,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q33" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr" s="2">
@@ -2863,6 +3361,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q34" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr" s="2">
@@ -2945,6 +3458,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q35" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr" s="2">
@@ -3027,6 +3555,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q36" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr" s="2">
@@ -3109,6 +3652,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q37" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr" s="2">
@@ -3191,6 +3749,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q38" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr" s="2">
@@ -3273,6 +3846,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q39" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr" s="2">
@@ -3355,6 +3943,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q40" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr" s="2">
@@ -3437,6 +4040,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr" s="2">
@@ -3519,6 +4137,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr" s="2">
@@ -3601,6 +4234,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr" s="2">
@@ -3683,6 +4331,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr" s="2">
@@ -3765,6 +4428,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr" s="2">
@@ -3847,6 +4525,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr" s="2">
@@ -3929,6 +4622,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr" s="2">
@@ -4011,6 +4719,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr" s="2">
@@ -4093,6 +4816,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr" s="2">
@@ -4175,6 +4913,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr" s="2">
@@ -4257,6 +5010,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr" s="2">
@@ -4339,6 +5107,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q52" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr" s="2">
@@ -4421,6 +5204,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr" s="2">
@@ -4503,6 +5301,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr" s="2">
@@ -4585,6 +5398,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr" s="2">
@@ -4667,6 +5495,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr" s="2">
@@ -4749,6 +5592,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr" s="2">
@@ -4831,6 +5689,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr" s="2">
@@ -4913,6 +5786,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr" s="2">
@@ -4995,6 +5883,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr" s="2">
@@ -5077,6 +5980,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr" s="2">
@@ -5159,6 +6077,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr" s="2">
@@ -5241,6 +6174,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr" s="2">
@@ -5323,6 +6271,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr" s="2">
@@ -5405,6 +6368,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr" s="2">
@@ -5487,6 +6465,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr" s="2">
@@ -5569,6 +6562,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr" s="2">
@@ -5651,6 +6659,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr" s="2">
@@ -5733,6 +6756,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr" s="2">
@@ -5815,6 +6853,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr" s="2">
@@ -5897,6 +6950,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr" s="2">
@@ -5979,6 +7047,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr" s="2">
@@ -6061,6 +7144,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr" s="2">
@@ -6143,6 +7241,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr" s="2">
@@ -6225,6 +7338,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr" s="2">
@@ -6307,6 +7435,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr" s="2">
@@ -6389,6 +7532,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr" s="2">
@@ -6471,6 +7629,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr" s="2">
@@ -6553,6 +7726,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr" s="2">
@@ -6635,6 +7823,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr" s="2">
@@ -6717,6 +7920,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr" s="2">
@@ -6799,6 +8017,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr" s="2">
@@ -6881,6 +8114,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr" s="2">
@@ -6963,6 +8211,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr" s="2">
@@ -7045,6 +8308,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr" s="2">
@@ -7127,6 +8405,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr" s="2">
@@ -7209,6 +8502,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr" s="2">
@@ -7291,6 +8599,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr" s="2">
@@ -7373,6 +8696,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr" s="2">
@@ -7455,6 +8793,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr" s="2">
@@ -7537,6 +8890,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr" s="2">
@@ -7619,6 +8987,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr" s="2">
@@ -7701,6 +9084,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr" s="2">
@@ -7783,6 +9181,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr" s="2">
@@ -7865,6 +9278,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr" s="2">
@@ -7947,6 +9375,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr" s="2">
@@ -8029,6 +9472,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr" s="2">
@@ -8111,6 +9569,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr" s="2">
@@ -8193,6 +9666,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr" s="2">
@@ -8275,6 +9763,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q100" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R100" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S100" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr" s="2">
@@ -8357,6 +9860,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q101" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R101" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S101" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr" s="2">
@@ -8439,6 +9957,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q102" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R102" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S102" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr" s="2">
@@ -8521,6 +10054,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q103" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R103" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S103" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr" s="2">
@@ -8603,6 +10151,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q104" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R104" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S104" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr" s="2">
@@ -8685,6 +10248,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q105" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R105" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S105" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr" s="2">
@@ -8767,6 +10345,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q106" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R106" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S106" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr" s="2">
@@ -8849,6 +10442,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q107" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R107" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S107" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr" s="2">
@@ -8931,6 +10539,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q108" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R108" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S108" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr" s="2">
@@ -9013,6 +10636,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Q109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr" s="2">
@@ -9091,6 +10729,21 @@
         </is>
       </c>
       <c r="P110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="Q110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S110" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -9919,10 +11572,22 @@
     <row r="11">
       <c r="A11" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">link_1 / link_2 / link_3</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Optional links shown as buttons in the event window (flyers, sign-up forms, more information). Enter just the address (https://…), or add a label: Flyer | https://…  or  Flyer | チラシ | https://…  Without a label the button is named automatically (PDF flyer, Sign-up form, View document…). Excel hyperlinks (Insert &gt; Link) also work. Flyers uploaded to the website can use a path such as compass/files/sports-day.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Holidays sheet: type</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr" s="2">
+      <c r="B12" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">national, school or noclass</t>
         </is>

</xml_diff>

<commit_message>
Calendar updates from coordinators (8 Oct)
- Remove Career Support & Mental Health Round Table (7 Oct, postponed)
- ELC & Primary Curriculum Night: 17:30-20:30, Community Room, parents
  invited, fuller EN/JA description
- Sensory Wonderland: ELC (not Primary)
- IMF: Saturday 10:00-14:00, theme, no school buses; Japanese title
  インターナショナル・マインデッドネス・フェスティバル
- Add Concept Con (Wellbeing) for Primary, 9-13 Nov
- Winter Art Contest -> Gallery Day: ELC & Primary Art Showcase,
  24 Nov only, 13:10-14:55, Gym
- Grade 3, 4 Musical: 3 Dec only, 17:30
- Last updated 8 Oct 2026

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/admin/EIS-Compass-events.xlsx
+++ b/admin/EIS-Compass-events.xlsx
@@ -2022,17 +2022,17 @@
     <row r="21">
       <c r="A21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2026-10-07-career-support-and-mental-health-round-table</t>
+          <t xml:space="preserve">2026-10-09-high-school-curriculum-night</t>
         </is>
       </c>
       <c r="B21" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-10-07</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-10-07</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="D21" t="inlineStr" s="3">
@@ -2047,7 +2047,7 @@
       </c>
       <c r="F21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G21" t="inlineStr" s="2">
@@ -2062,22 +2062,22 @@
       </c>
       <c r="I21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Career Support and Mental Health Round Table</t>
+          <t xml:space="preserve">High School Curriculum Night</t>
         </is>
       </c>
       <c r="J21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">進路・メンタルヘルス座談会</t>
+          <t xml:space="preserve">高等部カリキュラム説明会</t>
         </is>
       </c>
       <c r="K21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">An informative event where students can learn about IB university admissions, holistic admissions strategies in Japan and abroad, and explore future academic and career opportunities through discussions with experts and representatives.</t>
+          <t xml:space="preserve">An information session for students to learn about the IB Diploma Programme, course choices, academic expectations, and pathways to university.</t>
         </is>
       </c>
       <c r="L21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">専門家や関係者との対話を通して、IBでの大学入試、国内外の総合型選抜の戦略について学び、将来の進学やキャリアの可能性を探る説明会です。</t>
+          <t xml:space="preserve">IBディプロマ・プログラム、科目選択、学業面で求められること、大学への進路について学ぶ説明会です。</t>
         </is>
       </c>
       <c r="M21" t="inlineStr" s="2">
@@ -2092,7 +2092,7 @@
       </c>
       <c r="O21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2026-10-07-career-support-and-mental-health-round-table.webp</t>
+          <t xml:space="preserve">compass/images/events/2026-10-09-high-school-curriculum-night.webp</t>
         </is>
       </c>
       <c r="P21" t="inlineStr" s="2">
@@ -2119,7 +2119,7 @@
     <row r="22">
       <c r="A22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2026-10-09-high-school-curriculum-night</t>
+          <t xml:space="preserve">2026-10-09-eagle-bucks-store</t>
         </is>
       </c>
       <c r="B22" t="inlineStr" s="3">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="E22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">High School</t>
+          <t xml:space="preserve">Primary</t>
         </is>
       </c>
       <c r="F22" t="inlineStr" s="2">
@@ -2159,22 +2159,22 @@
       </c>
       <c r="I22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">High School Curriculum Night</t>
+          <t xml:space="preserve">Eagle Bucks Store</t>
         </is>
       </c>
       <c r="J22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">高等部カリキュラム説明会</t>
+          <t xml:space="preserve">イーグルバックス・ストア</t>
         </is>
       </c>
       <c r="K22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">An information session for students to learn about the IB Diploma Programme, course choices, academic expectations, and pathways to university.</t>
+          <t xml:space="preserve">Students can use their earned Eagle Bucks to purchase rewards and special items. The store reinforces positive behavior, responsibility, and goal-setting.</t>
         </is>
       </c>
       <c r="L22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">IBディプロマ・プログラム、科目選択、学業面で求められること、大学への進路について学ぶ説明会です。</t>
+          <t xml:space="preserve">獲得したイーグルバックスを使って、ごほうびや特別なアイテムと交換できます。前向きな行動、責任感、目標設定を後押しする取り組みです。</t>
         </is>
       </c>
       <c r="M22" t="inlineStr" s="2">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="O22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2026-10-09-high-school-curriculum-night.webp</t>
+          <t xml:space="preserve">compass/images/events/2026-10-09-eagle-bucks-store.webp</t>
         </is>
       </c>
       <c r="P22" t="inlineStr" s="2">
@@ -2216,32 +2216,32 @@
     <row r="23">
       <c r="A23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2026-10-09-eagle-bucks-store</t>
+          <t xml:space="preserve">2026-10-19-elc-primary-curriculum-night</t>
         </is>
       </c>
       <c r="B23" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-10-09</t>
+          <t xml:space="preserve">2026-10-19</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-10-09</t>
+          <t xml:space="preserve">2026-10-19</t>
         </is>
       </c>
       <c r="D23" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">17:30-20:30</t>
         </is>
       </c>
       <c r="E23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary</t>
+          <t xml:space="preserve">Primary, ELC</t>
         </is>
       </c>
       <c r="F23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="G23" t="inlineStr" s="2">
@@ -2256,37 +2256,37 @@
       </c>
       <c r="I23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Eagle Bucks Store</t>
+          <t xml:space="preserve">ELC &amp; Primary Curriculum Night</t>
         </is>
       </c>
       <c r="J23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">イーグルバックス・ストア</t>
+          <t xml:space="preserve">幼稚部・小学部カリキュラム説明会</t>
         </is>
       </c>
       <c r="K23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students can use their earned Eagle Bucks to purchase rewards and special items. The store reinforces positive behavior, responsibility, and goal-setting.</t>
+          <t xml:space="preserve">An evening to help families understand what children learn, how they learn, how progress is assessed, and how learning can be supported at home. Families will experience classroom activities, explore topics of interest, and ask questions. The evening begins with a welcome in the Community Room, followed by two breakout sessions and a panel Q&amp;A. Please complete the attendance and session selection form; sessions with limited interest may be cancelled.</t>
         </is>
       </c>
       <c r="L23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">獲得したイーグルバックスを使って、ごほうびや特別なアイテムと交換できます。前向きな行動、責任感、目標設定を後押しする取り組みです。</t>
+          <t xml:space="preserve">お子さまが何を、どのように学んでいるのか、学習の進歩をどのように評価しているのか、ご家庭でどのように学びを支えられるのかについて理解を深めていただく会です。教室での活動を体験し、関心のあるテーマについて学び、質問していただけます。コミュニティルームでの開会の後、2つの分科会とパネル質疑応答を行います。参加確認・セッション選択フォームへのご回答をお願いいたします（参加希望者が少ないセッションは中止となる場合があります）。</t>
         </is>
       </c>
       <c r="M23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Community Room</t>
         </is>
       </c>
       <c r="N23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">コミュニティルーム</t>
         </is>
       </c>
       <c r="O23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2026-10-09-eagle-bucks-store.webp</t>
+          <t xml:space="preserve">compass/images/events/2026-10-19-elc-primary-curriculum-night.webp</t>
         </is>
       </c>
       <c r="P23" t="inlineStr" s="2">
@@ -2313,7 +2313,7 @@
     <row r="24">
       <c r="A24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2026-10-19-elc-primary-curriculum-night</t>
+          <t xml:space="preserve">2026-10-19-parent-teacher-conferences</t>
         </is>
       </c>
       <c r="B24" t="inlineStr" s="3">
@@ -2333,17 +2333,17 @@
       </c>
       <c r="E24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary, ELC</t>
+          <t xml:space="preserve">Whole School</t>
         </is>
       </c>
       <c r="F24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="G24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="H24" t="inlineStr" s="2">
@@ -2353,22 +2353,22 @@
       </c>
       <c r="I24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ELC &amp; Primary Curriculum Night</t>
+          <t xml:space="preserve">Parent Teacher Conferences</t>
         </is>
       </c>
       <c r="J24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">幼稚部・小学部カリキュラム説明会</t>
+          <t xml:space="preserve">保護者面談</t>
         </is>
       </c>
       <c r="K24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Families are invited to learn about the curriculum, classroom routines, and learning goals for the year. This event helps strengthen the home-school partnership.</t>
+          <t xml:space="preserve">Parents meet one-on-one with each teacher to discuss their child's progress, strengths, and next steps. The school campus is closed to students on this day.</t>
         </is>
       </c>
       <c r="L24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">カリキュラム、教室での日課、今年度の学習目標についてご紹介します。家庭と学校の連携を深める行事です。</t>
+          <t xml:space="preserve">保護者の皆様が各担当教員と個別に面談し、お子様の成長、強み、今後の課題についてお話しします。当日、生徒は登校しません。</t>
         </is>
       </c>
       <c r="M24" t="inlineStr" s="2">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="O24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2026-10-19-elc-primary-curriculum-night.webp</t>
+          <t xml:space="preserve">compass/images/events/2026-10-19-parent-teacher-conferences.webp</t>
         </is>
       </c>
       <c r="P24" t="inlineStr" s="2">
@@ -2410,17 +2410,17 @@
     <row r="25">
       <c r="A25" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2026-10-19-parent-teacher-conferences</t>
+          <t xml:space="preserve">2026-10-20-secondary-curriculum-night</t>
         </is>
       </c>
       <c r="B25" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-10-19</t>
+          <t xml:space="preserve">2026-10-20</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-10-19</t>
+          <t xml:space="preserve">2026-10-20</t>
         </is>
       </c>
       <c r="D25" t="inlineStr" s="3">
@@ -2430,17 +2430,17 @@
       </c>
       <c r="E25" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Whole School</t>
+          <t xml:space="preserve">Secondary</t>
         </is>
       </c>
       <c r="F25" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G25" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H25" t="inlineStr" s="2">
@@ -2450,22 +2450,22 @@
       </c>
       <c r="I25" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Parent Teacher Conferences</t>
+          <t xml:space="preserve">Secondary Curriculum Night</t>
         </is>
       </c>
       <c r="J25" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">保護者面談</t>
+          <t xml:space="preserve">中等部カリキュラム説明会</t>
         </is>
       </c>
       <c r="K25" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Parents meet one-on-one with each teacher to discuss their child's progress, strengths, and next steps. The school campus is closed to students on this day.</t>
+          <t xml:space="preserve">Secondary parents are invited to Curriculum Night to learn more about subject expectations, learning goals, assessment, and support for students in Grades 6 to 10.</t>
         </is>
       </c>
       <c r="L25" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">保護者の皆様が各担当教員と個別に面談し、お子様の成長、強み、今後の課題についてお話しします。当日、生徒は登校しません。</t>
+          <t xml:space="preserve">中等部の保護者の皆様を対象に、6～10年生の各教科で求められること、学習目標、評価、生徒への支援についてご説明します。</t>
         </is>
       </c>
       <c r="M25" t="inlineStr" s="2">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="O25" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2026-10-19-parent-teacher-conferences.webp</t>
+          <t xml:space="preserve">compass/images/events/2026-10-20-secondary-curriculum-night.webp</t>
         </is>
       </c>
       <c r="P25" t="inlineStr" s="2">
@@ -2507,17 +2507,17 @@
     <row r="26">
       <c r="A26" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2026-10-20-secondary-curriculum-night</t>
+          <t xml:space="preserve">2026-10-21-college-fair</t>
         </is>
       </c>
       <c r="B26" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-10-20</t>
+          <t xml:space="preserve">2026-10-21</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-10-20</t>
+          <t xml:space="preserve">2026-10-21</t>
         </is>
       </c>
       <c r="D26" t="inlineStr" s="3">
@@ -2527,12 +2527,12 @@
       </c>
       <c r="E26" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary</t>
+          <t xml:space="preserve">High School</t>
         </is>
       </c>
       <c r="F26" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="G26" t="inlineStr" s="2">
@@ -2547,22 +2547,22 @@
       </c>
       <c r="I26" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary Curriculum Night</t>
+          <t xml:space="preserve">College Fair</t>
         </is>
       </c>
       <c r="J26" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">中等部カリキュラム説明会</t>
+          <t xml:space="preserve">大学進学フェア</t>
         </is>
       </c>
       <c r="K26" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary parents are invited to Curriculum Night to learn more about subject expectations, learning goals, assessment, and support for students in Grades 6 to 10.</t>
+          <t xml:space="preserve">A special event where representatives from several international and Japanese universities visit our school to introduce their programs and admission opportunities. The fair is open to all students and parents, and students from other international schools in the area are also invited to attend.</t>
         </is>
       </c>
       <c r="L26" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">中等部の保護者の皆様を対象に、6～10年生の各教科で求められること、学習目標、評価、生徒への支援についてご説明します。</t>
+          <t xml:space="preserve">国内外の複数の大学の担当者が来校し、各大学のプログラムや入学機会を紹介する特別イベントです。全生徒・保護者が参加でき、近隣のインターナショナルスクールの生徒もご招待しています。</t>
         </is>
       </c>
       <c r="M26" t="inlineStr" s="2">
@@ -2577,7 +2577,7 @@
       </c>
       <c r="O26" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2026-10-20-secondary-curriculum-night.webp</t>
+          <t xml:space="preserve">compass/images/events/2026-10-21-college-fair.webp</t>
         </is>
       </c>
       <c r="P26" t="inlineStr" s="2">
@@ -2604,17 +2604,17 @@
     <row r="27">
       <c r="A27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2026-10-21-college-fair</t>
+          <t xml:space="preserve">2026-10-23-nagoya-university-biology-laboratory-visit</t>
         </is>
       </c>
       <c r="B27" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-10-21</t>
+          <t xml:space="preserve">2026-10-23</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-10-21</t>
+          <t xml:space="preserve">2026-10-23</t>
         </is>
       </c>
       <c r="D27" t="inlineStr" s="3">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="F27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G27" t="inlineStr" s="2">
@@ -2644,22 +2644,22 @@
       </c>
       <c r="I27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">College Fair</t>
+          <t xml:space="preserve">Nagoya University Biology Laboratory Visit</t>
         </is>
       </c>
       <c r="J27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">大学進学フェア</t>
+          <t xml:space="preserve">名古屋大学 生物学研究室訪問</t>
         </is>
       </c>
       <c r="K27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">A special event where representatives from several international and Japanese universities visit our school to introduce their programs and admission opportunities. The fair is open to all students and parents, and students from other international schools in the area are also invited to attend.</t>
+          <t xml:space="preserve">Grade 11 and 12 Biology students will visit Nagoya University for a guided laboratory experience, connecting classroom learning with real-world scientific research.</t>
         </is>
       </c>
       <c r="L27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">国内外の複数の大学の担当者が来校し、各大学のプログラムや入学機会を紹介する特別イベントです。全生徒・保護者が参加でき、近隣のインターナショナルスクールの生徒もご招待しています。</t>
+          <t xml:space="preserve">11・12年生の生物履修者が名古屋大学を訪問し、研究室での体験を通して授業での学びと実際の科学研究を結びつけます。</t>
         </is>
       </c>
       <c r="M27" t="inlineStr" s="2">
@@ -2674,7 +2674,7 @@
       </c>
       <c r="O27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2026-10-21-college-fair.webp</t>
+          <t xml:space="preserve">compass/images/events/2026-10-23-nagoya-university-biology-laboratory-visit.webp</t>
         </is>
       </c>
       <c r="P27" t="inlineStr" s="2">
@@ -2701,17 +2701,17 @@
     <row r="28">
       <c r="A28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2026-10-23-nagoya-university-biology-laboratory-visit</t>
+          <t xml:space="preserve">2026-10-25-pta-picnic</t>
         </is>
       </c>
       <c r="B28" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-10-23</t>
+          <t xml:space="preserve">2026-10-25</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-10-23</t>
+          <t xml:space="preserve">2026-10-25</t>
         </is>
       </c>
       <c r="D28" t="inlineStr" s="3">
@@ -2721,7 +2721,7 @@
       </c>
       <c r="E28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">High School</t>
+          <t xml:space="preserve">PTA</t>
         </is>
       </c>
       <c r="F28" t="inlineStr" s="2">
@@ -2741,22 +2741,22 @@
       </c>
       <c r="I28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Nagoya University Biology Laboratory Visit</t>
+          <t xml:space="preserve">PTA Picnic</t>
         </is>
       </c>
       <c r="J28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">名古屋大学 生物学研究室訪問</t>
+          <t xml:space="preserve">PTAピクニック</t>
         </is>
       </c>
       <c r="K28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Grade 11 and 12 Biology students will visit Nagoya University for a guided laboratory experience, connecting classroom learning with real-world scientific research.</t>
+          <t xml:space="preserve">Families, students, and staff come together for a fun outdoor gathering that strengthens relationships and builds school community.</t>
         </is>
       </c>
       <c r="L28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">11・12年生の生物履修者が名古屋大学を訪問し、研究室での体験を通して授業での学びと実際の科学研究を結びつけます。</t>
+          <t xml:space="preserve">ご家族、生徒、教職員が集まり、屋外で楽しく交流しながら絆を深め、学校コミュニティを育みます。</t>
         </is>
       </c>
       <c r="M28" t="inlineStr" s="2">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="O28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2026-10-23-nagoya-university-biology-laboratory-visit.webp</t>
+          <t xml:space="preserve">compass/images/events/2026-10-25-pta-picnic.webp</t>
         </is>
       </c>
       <c r="P28" t="inlineStr" s="2">
@@ -2798,17 +2798,17 @@
     <row r="29">
       <c r="A29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2026-10-25-pta-picnic</t>
+          <t xml:space="preserve">2026-10-26-toyota-college-trip</t>
         </is>
       </c>
       <c r="B29" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-10-25</t>
+          <t xml:space="preserve">2026-10-26</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-10-25</t>
+          <t xml:space="preserve">2026-10-26</t>
         </is>
       </c>
       <c r="D29" t="inlineStr" s="3">
@@ -2818,7 +2818,7 @@
       </c>
       <c r="E29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PTA</t>
+          <t xml:space="preserve">Secondary</t>
         </is>
       </c>
       <c r="F29" t="inlineStr" s="2">
@@ -2838,22 +2838,22 @@
       </c>
       <c r="I29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PTA Picnic</t>
+          <t xml:space="preserve">Toyota College Trip</t>
         </is>
       </c>
       <c r="J29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PTAピクニック</t>
+          <t xml:space="preserve">豊田高専見学</t>
         </is>
       </c>
       <c r="K29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Families, students, and staff come together for a fun outdoor gathering that strengthens relationships and builds school community.</t>
+          <t xml:space="preserve">Grade 8 Science students will visit Toyota College for a curriculum-based learning experience connected to their science studies.</t>
         </is>
       </c>
       <c r="L29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ご家族、生徒、教職員が集まり、屋外で楽しく交流しながら絆を深め、学校コミュニティを育みます。</t>
+          <t xml:space="preserve">8年生が理科の授業と関連したカリキュラムに基づく学習として、豊田高専を訪問します。</t>
         </is>
       </c>
       <c r="M29" t="inlineStr" s="2">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="O29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2026-10-25-pta-picnic.webp</t>
+          <t xml:space="preserve">compass/images/events/2026-10-26-toyota-college-trip.webp</t>
         </is>
       </c>
       <c r="P29" t="inlineStr" s="2">
@@ -2895,17 +2895,17 @@
     <row r="30">
       <c r="A30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2026-10-26-toyota-college-trip</t>
+          <t xml:space="preserve">2026-10-30-sensory-wonderland</t>
         </is>
       </c>
       <c r="B30" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-10-26</t>
+          <t xml:space="preserve">2026-10-30</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-10-26</t>
+          <t xml:space="preserve">2026-10-30</t>
         </is>
       </c>
       <c r="D30" t="inlineStr" s="3">
@@ -2915,7 +2915,7 @@
       </c>
       <c r="E30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary</t>
+          <t xml:space="preserve">ELC</t>
         </is>
       </c>
       <c r="F30" t="inlineStr" s="2">
@@ -2935,22 +2935,22 @@
       </c>
       <c r="I30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Toyota College Trip</t>
+          <t xml:space="preserve">Sensory Wonderland</t>
         </is>
       </c>
       <c r="J30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">豊田高専見学</t>
+          <t xml:space="preserve">センサリー・ワンダーランド</t>
         </is>
       </c>
       <c r="K30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Grade 8 Science students will visit Toyota College for a curriculum-based learning experience connected to their science studies.</t>
+          <t xml:space="preserve">Students explore a variety of interactive sensory experiences designed to engage curiosity, creativity, and learning through play.</t>
         </is>
       </c>
       <c r="L30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">8年生が理科の授業と関連したカリキュラムに基づく学習として、豊田高専を訪問します。</t>
+          <t xml:space="preserve">好奇心と創造性を刺激し、遊びを通して学ぶ、さまざまな体験型の感覚活動を楽しみます。</t>
         </is>
       </c>
       <c r="M30" t="inlineStr" s="2">
@@ -2965,7 +2965,7 @@
       </c>
       <c r="O30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2026-10-26-toyota-college-trip.webp</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="P30" t="inlineStr" s="2">
@@ -2992,32 +2992,32 @@
     <row r="31">
       <c r="A31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2026-10-30-sensory-wonderland</t>
+          <t xml:space="preserve">2026-10-31-international-mindedness-festival</t>
         </is>
       </c>
       <c r="B31" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-10-30</t>
+          <t xml:space="preserve">2026-10-31</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-10-30</t>
+          <t xml:space="preserve">2026-10-31</t>
         </is>
       </c>
       <c r="D31" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">10:00-14:00</t>
         </is>
       </c>
       <c r="E31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary</t>
+          <t xml:space="preserve">Whole School</t>
         </is>
       </c>
       <c r="F31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="G31" t="inlineStr" s="2">
@@ -3032,22 +3032,22 @@
       </c>
       <c r="I31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sensory Wonderland</t>
+          <t xml:space="preserve">International Mindedness Festival</t>
         </is>
       </c>
       <c r="J31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">センサリー・ワンダーランド</t>
+          <t xml:space="preserve">インターナショナル・マインデッドネス・フェスティバル</t>
         </is>
       </c>
       <c r="K31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students explore a variety of interactive sensory experiences designed to engage curiosity, creativity, and learning through play.</t>
+          <t xml:space="preserve">This year’s theme is “Festivals and Holidays Around the World”. A Saturday family event celebrating traditions, cultures, stories, arts, music and celebrations from around the world, with student activities, cultural displays, performances, arts and crafts, and interactive booths. Clean-up runs from 14:00 to 15:00, and community members are welcome to help. ELC and Primary students must attend with a parent or guardian and may not be dropped off. School buses will not operate. More details will be shared soon.</t>
         </is>
       </c>
       <c r="L31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">好奇心と創造性を刺激し、遊びを通して学ぶ、さまざまな体験型の感覚活動を楽しみます。</t>
+          <t xml:space="preserve">今年のテーマは「世界の祭りと祝日」です。世界各地の伝統、文化、物語、芸術、音楽、お祝いを紹介する、土曜日のご家族参加型イベントです。児童・生徒の活動、文化展示、パフォーマンス、工作、体験型ブースをお楽しみいただけます。午後2時～3時に片付けを行います（学校コミュニティの皆さまのご協力も歓迎します）。幼稚部・小学部の児童は必ず保護者同伴でご参加ください（お子さまだけを送り届けることはできません）。当日はスクールバスの運行はありません。詳細は近日中にお知らせします。</t>
         </is>
       </c>
       <c r="M31" t="inlineStr" s="2">
@@ -3062,7 +3062,7 @@
       </c>
       <c r="O31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">compass/images/events/2026-10-31-international-mindedness-festival.webp</t>
         </is>
       </c>
       <c r="P31" t="inlineStr" s="2">
@@ -3089,17 +3089,17 @@
     <row r="32">
       <c r="A32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2026-10-31-international-mindedness-festival</t>
+          <t xml:space="preserve">2026-11-04-elc-sports-day-rehearsal-1</t>
         </is>
       </c>
       <c r="B32" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-10-31</t>
+          <t xml:space="preserve">2026-11-04</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-10-31</t>
+          <t xml:space="preserve">2026-11-04</t>
         </is>
       </c>
       <c r="D32" t="inlineStr" s="3">
@@ -3109,12 +3109,12 @@
       </c>
       <c r="E32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Whole School</t>
+          <t xml:space="preserve">ELC</t>
         </is>
       </c>
       <c r="F32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G32" t="inlineStr" s="2">
@@ -3129,22 +3129,22 @@
       </c>
       <c r="I32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">International Mindedness Festival</t>
+          <t xml:space="preserve">ELC Sports Day Rehearsal #1</t>
         </is>
       </c>
       <c r="J32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">国際理解フェスティバル</t>
+          <t xml:space="preserve">幼稚部運動会リハーサル #1</t>
         </is>
       </c>
       <c r="K32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">The whole school community, including parents, will take part in IMF, a full-day event celebrating community, culture, and shared school experiences.</t>
+          <t xml:space="preserve">During Sports Day practice, students participate in a variety of physical activities, team games, relays, and event rehearsals in preparation for Sports Day. They develop teamwork, cooperation, sportsmanship, and physical fitness while learning event procedures, safety expectations, and cheering routines. Practice sessions help students build confidence and ensure they are prepared to participate successfully in the Sports Day celebration.</t>
         </is>
       </c>
       <c r="L32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">保護者の皆様を含む学校コミュニティ全体で、コミュニティと文化、そして共に過ごす学校生活を祝う終日行事「IMF」に参加します。</t>
+          <t xml:space="preserve">運動会に向けた練習では、さまざまな運動、チームゲーム、リレー、種目のリハーサルに取り組みます。進行の流れ、安全面のルール、応援の仕方を学びながら、チームワーク、協調性、スポーツマンシップ、体力を養います。練習を通して自信をつけ、運動会当日に力を発揮できるよう準備します。</t>
         </is>
       </c>
       <c r="M32" t="inlineStr" s="2">
@@ -3159,7 +3159,7 @@
       </c>
       <c r="O32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2026-10-31-international-mindedness-festival.webp</t>
+          <t xml:space="preserve">compass/images/events/2026-11-04-elc-sports-day-rehearsal-1.webp</t>
         </is>
       </c>
       <c r="P32" t="inlineStr" s="2">
@@ -3186,17 +3186,17 @@
     <row r="33">
       <c r="A33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2026-11-04-elc-sports-day-rehearsal-1</t>
+          <t xml:space="preserve">2026-11-05-toyota-museum-field-trip</t>
         </is>
       </c>
       <c r="B33" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-11-04</t>
+          <t xml:space="preserve">2026-11-05</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-11-04</t>
+          <t xml:space="preserve">2026-11-05</t>
         </is>
       </c>
       <c r="D33" t="inlineStr" s="3">
@@ -3206,7 +3206,7 @@
       </c>
       <c r="E33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ELC</t>
+          <t xml:space="preserve">Secondary</t>
         </is>
       </c>
       <c r="F33" t="inlineStr" s="2">
@@ -3226,22 +3226,22 @@
       </c>
       <c r="I33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ELC Sports Day Rehearsal #1</t>
+          <t xml:space="preserve">Toyota Museum Field Trip</t>
         </is>
       </c>
       <c r="J33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">幼稚部運動会リハーサル #1</t>
+          <t xml:space="preserve">トヨタ博物館校外学習</t>
         </is>
       </c>
       <c r="K33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">During Sports Day practice, students participate in a variety of physical activities, team games, relays, and event rehearsals in preparation for Sports Day. They develop teamwork, cooperation, sportsmanship, and physical fitness while learning event procedures, safety expectations, and cheering routines. Practice sessions help students build confidence and ensure they are prepared to participate successfully in the Sports Day celebration.</t>
+          <t xml:space="preserve">Grade 9 students go to the Toyota museum down the road and view the exhibits taking some notes on machines they learned about.</t>
         </is>
       </c>
       <c r="L33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">運動会に向けた練習では、さまざまな運動、チームゲーム、リレー、種目のリハーサルに取り組みます。進行の流れ、安全面のルール、応援の仕方を学びながら、チームワーク、協調性、スポーツマンシップ、体力を養います。練習を通して自信をつけ、運動会当日に力を発揮できるよう準備します。</t>
+          <t xml:space="preserve">9年生が近くのトヨタの博物館を訪れ、授業で学んだ機械について展示を見学しながらメモを取ります。</t>
         </is>
       </c>
       <c r="M33" t="inlineStr" s="2">
@@ -3256,7 +3256,7 @@
       </c>
       <c r="O33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2026-11-04-elc-sports-day-rehearsal-1.webp</t>
+          <t xml:space="preserve">compass/images/events/2026-11-05-toyota-museum-field-trip.webp</t>
         </is>
       </c>
       <c r="P33" t="inlineStr" s="2">
@@ -3283,17 +3283,17 @@
     <row r="34">
       <c r="A34" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2026-11-05-toyota-museum-field-trip</t>
+          <t xml:space="preserve">2026-11-06-extracurricular-activities-autumn-cas-project-su</t>
         </is>
       </c>
       <c r="B34" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-11-05</t>
+          <t xml:space="preserve">2026-11-06</t>
         </is>
       </c>
       <c r="C34" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-11-05</t>
+          <t xml:space="preserve">2026-11-06</t>
         </is>
       </c>
       <c r="D34" t="inlineStr" s="3">
@@ -3308,7 +3308,7 @@
       </c>
       <c r="F34" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="G34" t="inlineStr" s="2">
@@ -3323,22 +3323,22 @@
       </c>
       <c r="I34" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Toyota Museum Field Trip</t>
+          <t xml:space="preserve">Extracurricular Activities: Autumn CAS &amp; Project Support Fair</t>
         </is>
       </c>
       <c r="J34" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">トヨタ博物館校外学習</t>
+          <t xml:space="preserve">課外活動：秋のCAS・プロジェクトサポートフェア</t>
         </is>
       </c>
       <c r="K34" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Grade 9 students go to the Toyota museum down the road and view the exhibits taking some notes on machines they learned about.</t>
+          <t xml:space="preserve">Secondary PTA Supported Event to help students understand various volunteering and CAS project opportunities in the community. Open to MYP and DP Students.</t>
         </is>
       </c>
       <c r="L34" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">9年生が近くのトヨタの博物館を訪れ、授業で学んだ機械について展示を見学しながらメモを取ります。</t>
+          <t xml:space="preserve">中等部PTAの支援による行事で、地域でのさまざまなボランティアやCASプロジェクトの機会について知ることができます。MYP・DP生徒が対象です。</t>
         </is>
       </c>
       <c r="M34" t="inlineStr" s="2">
@@ -3353,7 +3353,7 @@
       </c>
       <c r="O34" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2026-11-05-toyota-museum-field-trip.webp</t>
+          <t xml:space="preserve">compass/images/events/2026-11-06-extracurricular-activities-autumn-cas-project-su.webp</t>
         </is>
       </c>
       <c r="P34" t="inlineStr" s="2">
@@ -3380,17 +3380,17 @@
     <row r="35">
       <c r="A35" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2026-11-06-extracurricular-activities-autumn-cas-project-su</t>
+          <t xml:space="preserve">2026-11-07-sat-test-4</t>
         </is>
       </c>
       <c r="B35" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-11-06</t>
+          <t xml:space="preserve">2026-11-07</t>
         </is>
       </c>
       <c r="C35" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-11-06</t>
+          <t xml:space="preserve">2026-11-07</t>
         </is>
       </c>
       <c r="D35" t="inlineStr" s="3">
@@ -3400,12 +3400,12 @@
       </c>
       <c r="E35" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary</t>
+          <t xml:space="preserve">High School</t>
         </is>
       </c>
       <c r="F35" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G35" t="inlineStr" s="2">
@@ -3420,22 +3420,22 @@
       </c>
       <c r="I35" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Extracurricular Activities: Autumn CAS &amp; Project Support Fair</t>
+          <t xml:space="preserve">SAT Test #4</t>
         </is>
       </c>
       <c r="J35" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">課外活動：秋のCAS・プロジェクトサポートフェア</t>
+          <t xml:space="preserve">SAT試験 第4回</t>
         </is>
       </c>
       <c r="K35" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary PTA Supported Event to help students understand various volunteering and CAS project opportunities in the community. Open to MYP and DP Students.</t>
+          <t xml:space="preserve">An internationally recognized university entrance exam. Our school is an official SAT test center, and both Enishi students and external students are welcome to take the test on campus.</t>
         </is>
       </c>
       <c r="L35" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">中等部PTAの支援による行事で、地域でのさまざまなボランティアやCASプロジェクトの機会について知ることができます。MYP・DP生徒が対象です。</t>
+          <t xml:space="preserve">国際的に認められた大学入学試験です。本校はSAT公式試験会場であり、本校生徒・外部生徒ともに校内で受験できます。</t>
         </is>
       </c>
       <c r="M35" t="inlineStr" s="2">
@@ -3450,7 +3450,7 @@
       </c>
       <c r="O35" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2026-11-06-extracurricular-activities-autumn-cas-project-su.webp</t>
+          <t xml:space="preserve">compass/images/events/2026-11-07-sat-test-4.webp</t>
         </is>
       </c>
       <c r="P35" t="inlineStr" s="2">
@@ -3477,17 +3477,17 @@
     <row r="36">
       <c r="A36" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2026-11-07-sat-test-4</t>
+          <t xml:space="preserve">2026-11-09-wellbeing-week</t>
         </is>
       </c>
       <c r="B36" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-11-07</t>
+          <t xml:space="preserve">2026-11-09</t>
         </is>
       </c>
       <c r="C36" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-11-07</t>
+          <t xml:space="preserve">2026-11-13</t>
         </is>
       </c>
       <c r="D36" t="inlineStr" s="3">
@@ -3497,7 +3497,7 @@
       </c>
       <c r="E36" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">High School</t>
+          <t xml:space="preserve">Whole School</t>
         </is>
       </c>
       <c r="F36" t="inlineStr" s="2">
@@ -3517,22 +3517,22 @@
       </c>
       <c r="I36" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SAT Test #4</t>
+          <t xml:space="preserve">Wellbeing Week</t>
         </is>
       </c>
       <c r="J36" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SAT試験 第4回</t>
+          <t xml:space="preserve">ウェルビーイング週間</t>
         </is>
       </c>
       <c r="K36" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">An internationally recognized university entrance exam. Our school is an official SAT test center, and both Enishi students and external students are welcome to take the test on campus.</t>
+          <t xml:space="preserve">A school wide event focused on raising awareness for wellbeing.</t>
         </is>
       </c>
       <c r="L36" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">国際的に認められた大学入学試験です。本校はSAT公式試験会場であり、本校生徒・外部生徒ともに校内で受験できます。</t>
+          <t xml:space="preserve">ウェルビーイング（心身の健康）への意識を高めることを目的とした全校行事です。</t>
         </is>
       </c>
       <c r="M36" t="inlineStr" s="2">
@@ -3547,7 +3547,7 @@
       </c>
       <c r="O36" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2026-11-07-sat-test-4.webp</t>
+          <t xml:space="preserve">compass/images/events/2026-11-09-wellbeing-week.webp</t>
         </is>
       </c>
       <c r="P36" t="inlineStr" s="2">
@@ -3574,7 +3574,7 @@
     <row r="37">
       <c r="A37" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2026-11-09-wellbeing-week</t>
+          <t xml:space="preserve">2026-11-09-concept-con-wellbeing</t>
         </is>
       </c>
       <c r="B37" t="inlineStr" s="3">
@@ -3594,7 +3594,7 @@
       </c>
       <c r="E37" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Whole School</t>
+          <t xml:space="preserve">Primary</t>
         </is>
       </c>
       <c r="F37" t="inlineStr" s="2">
@@ -3614,22 +3614,22 @@
       </c>
       <c r="I37" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Wellbeing Week</t>
+          <t xml:space="preserve">Concept Con (Wellbeing)</t>
         </is>
       </c>
       <c r="J37" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ウェルビーイング週間</t>
+          <t xml:space="preserve">コンセプト・コン（ウェルビーイング）</t>
         </is>
       </c>
       <c r="K37" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">A school wide event focused on raising awareness for wellbeing.</t>
+          <t xml:space="preserve">The Primary Concept Conference on the theme of wellbeing, held during Wellbeing Week.</t>
         </is>
       </c>
       <c r="L37" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ウェルビーイング（心身の健康）への意識を高めることを目的とした全校行事です。</t>
+          <t xml:space="preserve">ウェルビーイング週間に合わせて行う、小学部のコンセプト・カンファレンス（テーマ：ウェルビーイング）です。</t>
         </is>
       </c>
       <c r="M37" t="inlineStr" s="2">
@@ -3644,7 +3644,7 @@
       </c>
       <c r="O37" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2026-11-09-wellbeing-week.webp</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="P37" t="inlineStr" s="2">
@@ -4166,12 +4166,12 @@
       </c>
       <c r="C43" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-11-25</t>
+          <t xml:space="preserve">2026-11-24</t>
         </is>
       </c>
       <c r="D43" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">13:10-14:55</t>
         </is>
       </c>
       <c r="E43" t="inlineStr" s="2">
@@ -4196,32 +4196,32 @@
       </c>
       <c r="I43" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Winter Art Contest</t>
+          <t xml:space="preserve">Gallery Day: ELC &amp; Primary Art Showcase</t>
         </is>
       </c>
       <c r="J43" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">冬のアートコンテスト</t>
+          <t xml:space="preserve">ギャラリーデー：幼稚部・小学部アート展</t>
         </is>
       </c>
       <c r="K43" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students showcase their art that they have been working on with the visual arts teacher at an art showcase. Selected pieces will be displayed and celebrated within the school community.</t>
+          <t xml:space="preserve">ELC and Primary students display the artwork they have created with the visual arts teacher. Parents are welcome to view the gallery from 13:10 to 14:55. Students vote for their favourite artworks, and the winners for each grade are announced.</t>
         </is>
       </c>
       <c r="L43" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">美術の先生と取り組んできた作品を作品展で発表します。選ばれた作品は校内に展示され、学校コミュニティで共に称えます。</t>
+          <t xml:space="preserve">幼稚部・小学部の児童が美術の授業で制作した作品を展示します。保護者の皆さまは13:10～14:55にご鑑賞いただけます。児童による投票を行い、学年ごとの受賞作品を発表します。</t>
         </is>
       </c>
       <c r="M43" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Gym</t>
         </is>
       </c>
       <c r="N43" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">体育館</t>
         </is>
       </c>
       <c r="O43" t="inlineStr" s="2">
@@ -4554,12 +4554,12 @@
       </c>
       <c r="C47" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-12-04</t>
+          <t xml:space="preserve">2026-12-03</t>
         </is>
       </c>
       <c r="D47" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">17:30</t>
         </is>
       </c>
       <c r="E47" t="inlineStr" s="2">

</xml_diff>

<commit_message>
Calendar corrections: Jan 7-8, graduation, June holiday, Summer School
- 7-8 Jan 2027: no classes
- G12 Graduation moved 28 May -> 29 May 2027 (Date changed label)
- Remove incorrect school holiday 6-7 June 2027
- Summer School split around Marine Day: 28 Jun-18 Jul and 20-24 Jul

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/admin/EIS-Compass-events.xlsx
+++ b/admin/EIS-Compass-events.xlsx
@@ -9593,12 +9593,12 @@
       </c>
       <c r="B99" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-05-28</t>
+          <t xml:space="preserve">2027-05-29</t>
         </is>
       </c>
       <c r="C99" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-05-28</t>
+          <t xml:space="preserve">2027-05-29</t>
         </is>
       </c>
       <c r="D99" t="inlineStr" s="3">
@@ -9623,7 +9623,7 @@
       </c>
       <c r="H99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">changed</t>
         </is>
       </c>
       <c r="I99" t="inlineStr" s="2">
@@ -10568,85 +10568,182 @@
       </c>
       <c r="C109" t="inlineStr" s="3">
         <is>
+          <t xml:space="preserve">2027-07-18</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Whole School</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Summer School</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">サマースクール</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Participate in fun English style summer camps that challenge students and help foster friendships and connections with others.</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">英語で楽しく過ごすサマーキャンプに参加し、新たなことに挑戦しながら友情や人とのつながりを育みます。</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">compass/images/events/2027-06-28-summer-school.webp</t>
+        </is>
+      </c>
+      <c r="P109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="Q109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">2027-07-20-summer-school</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">2027-07-20</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr" s="3">
+        <is>
           <t xml:space="preserve">2027-07-24</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E109" t="inlineStr" s="2">
+      <c r="D110" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Whole School</t>
         </is>
       </c>
-      <c r="F109" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G109" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H109" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="I109" t="inlineStr" s="2">
+      <c r="F110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Summer School</t>
         </is>
       </c>
-      <c r="J109" t="inlineStr" s="2">
+      <c r="J110" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">サマースクール</t>
         </is>
       </c>
-      <c r="K109" t="inlineStr" s="2">
+      <c r="K110" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Participate in fun English style summer camps that challenge students and help foster friendships and connections with others.</t>
         </is>
       </c>
-      <c r="L109" t="inlineStr" s="2">
+      <c r="L110" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">英語で楽しく過ごすサマーキャンプに参加し、新たなことに挑戦しながら友情や人とのつながりを育みます。</t>
         </is>
       </c>
-      <c r="M109" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N109" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="O109" t="inlineStr" s="2">
+      <c r="M110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O110" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">compass/images/events/2027-06-28-summer-school.webp</t>
         </is>
       </c>
-      <c r="P109" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="Q109" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="R109" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="S109" t="inlineStr" s="2">
+      <c r="P110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="Q110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S110" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -10966,39 +11063,39 @@
     <row r="12">
       <c r="A12" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-02-11</t>
+          <t xml:space="preserve">2027-01-07</t>
         </is>
       </c>
       <c r="B12" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-02-11</t>
+          <t xml:space="preserve">2027-01-08</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">national</t>
+          <t xml:space="preserve">noclass</t>
         </is>
       </c>
       <c r="D12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">National Foundation Day</t>
+          <t xml:space="preserve">No classes</t>
         </is>
       </c>
       <c r="E12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">建国記念の日</t>
+          <t xml:space="preserve">授業なし</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-02-23</t>
+          <t xml:space="preserve">2027-02-11</t>
         </is>
       </c>
       <c r="B13" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-02-23</t>
+          <t xml:space="preserve">2027-02-11</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="2">
@@ -11008,24 +11105,24 @@
       </c>
       <c r="D13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Emperor's Birthday</t>
+          <t xml:space="preserve">National Foundation Day</t>
         </is>
       </c>
       <c r="E13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">天皇誕生日</t>
+          <t xml:space="preserve">建国記念の日</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-03-21</t>
+          <t xml:space="preserve">2027-02-23</t>
         </is>
       </c>
       <c r="B14" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-03-21</t>
+          <t xml:space="preserve">2027-02-23</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="2">
@@ -11035,105 +11132,105 @@
       </c>
       <c r="D14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Vernal Equinox Day</t>
+          <t xml:space="preserve">Emperor's Birthday</t>
         </is>
       </c>
       <c r="E14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">春分の日</t>
+          <t xml:space="preserve">天皇誕生日</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-03-22</t>
+          <t xml:space="preserve">2027-03-21</t>
         </is>
       </c>
       <c r="B15" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-03-26</t>
+          <t xml:space="preserve">2027-03-21</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">school</t>
+          <t xml:space="preserve">national</t>
         </is>
       </c>
       <c r="D15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">School Holiday</t>
+          <t xml:space="preserve">Vernal Equinox Day</t>
         </is>
       </c>
       <c r="E15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">学校休日</t>
+          <t xml:space="preserve">春分の日</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-03-29</t>
+          <t xml:space="preserve">2027-03-22</t>
         </is>
       </c>
       <c r="B16" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-03-29</t>
+          <t xml:space="preserve">2027-03-26</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">noclass</t>
+          <t xml:space="preserve">school</t>
         </is>
       </c>
       <c r="D16" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Staff Prep Day (no classes)</t>
+          <t xml:space="preserve">School Holiday</t>
         </is>
       </c>
       <c r="E16" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">教職員準備日（授業なし）</t>
+          <t xml:space="preserve">学校休日</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-05-03</t>
+          <t xml:space="preserve">2027-03-29</t>
         </is>
       </c>
       <c r="B17" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-05-03</t>
+          <t xml:space="preserve">2027-03-29</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">national</t>
+          <t xml:space="preserve">noclass</t>
         </is>
       </c>
       <c r="D17" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Constitution Memorial Day</t>
+          <t xml:space="preserve">Staff Prep Day (no classes)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">憲法記念日</t>
+          <t xml:space="preserve">教職員準備日（授業なし）</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-05-04</t>
+          <t xml:space="preserve">2027-05-03</t>
         </is>
       </c>
       <c r="B18" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-05-04</t>
+          <t xml:space="preserve">2027-05-03</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="2">
@@ -11143,24 +11240,24 @@
       </c>
       <c r="D18" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Greenery Day</t>
+          <t xml:space="preserve">Constitution Memorial Day</t>
         </is>
       </c>
       <c r="E18" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">みどりの日</t>
+          <t xml:space="preserve">憲法記念日</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-05-05</t>
+          <t xml:space="preserve">2027-05-04</t>
         </is>
       </c>
       <c r="B19" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-05-05</t>
+          <t xml:space="preserve">2027-05-04</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="2">
@@ -11170,51 +11267,51 @@
       </c>
       <c r="D19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Children's Day</t>
+          <t xml:space="preserve">Greenery Day</t>
         </is>
       </c>
       <c r="E19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">こどもの日</t>
+          <t xml:space="preserve">みどりの日</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-05-06</t>
+          <t xml:space="preserve">2027-05-05</t>
         </is>
       </c>
       <c r="B20" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-05-07</t>
+          <t xml:space="preserve">2027-05-05</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">school</t>
+          <t xml:space="preserve">national</t>
         </is>
       </c>
       <c r="D20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">School Holiday</t>
+          <t xml:space="preserve">Children's Day</t>
         </is>
       </c>
       <c r="E20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">学校休日</t>
+          <t xml:space="preserve">こどもの日</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-06-06</t>
+          <t xml:space="preserve">2027-05-06</t>
         </is>
       </c>
       <c r="B21" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-06-07</t>
+          <t xml:space="preserve">2027-05-07</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="2">

</xml_diff>

<commit_message>
Add Parent Teacher Conferences on 8 Jan 2027
Whole school, parents invited, no classes. The separate "No classes"
entry now covers 7 Jan only, as on other conference days.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/admin/EIS-Compass-events.xlsx
+++ b/admin/EIS-Compass-events.xlsx
@@ -5514,17 +5514,17 @@
     <row r="57">
       <c r="A57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-01-14-g10-parent-info-session-high-school-subject-choi</t>
+          <t xml:space="preserve">2027-01-08-parent-teacher-conferences</t>
         </is>
       </c>
       <c r="B57" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-01-14</t>
+          <t xml:space="preserve">2027-01-08</t>
         </is>
       </c>
       <c r="C57" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-01-14</t>
+          <t xml:space="preserve">2027-01-08</t>
         </is>
       </c>
       <c r="D57" t="inlineStr" s="3">
@@ -5534,7 +5534,7 @@
       </c>
       <c r="E57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary</t>
+          <t xml:space="preserve">Whole School</t>
         </is>
       </c>
       <c r="F57" t="inlineStr" s="2">
@@ -5544,7 +5544,7 @@
       </c>
       <c r="G57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="H57" t="inlineStr" s="2">
@@ -5554,22 +5554,22 @@
       </c>
       <c r="I57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">G10 Parent info Session (High School Subject Choice)</t>
+          <t xml:space="preserve">Parent Teacher Conferences</t>
         </is>
       </c>
       <c r="J57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">G10保護者向け説明会（高等部科目選択）</t>
+          <t xml:space="preserve">保護者面談</t>
         </is>
       </c>
       <c r="K57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Grade 10 parents are invited to an information session about DP subject choices and guidance for planning the next stage of their child’s learning.</t>
+          <t xml:space="preserve">Parents meet one-on-one with each teacher to discuss their child's progress, strengths, and next steps. The school campus is closed to students on this day.</t>
         </is>
       </c>
       <c r="L57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">10年生の保護者の皆様を対象に、DPの科目選択と、お子様の次のステージの学びを計画するためのガイダンスを行います。</t>
+          <t xml:space="preserve">保護者の皆様が各担当教員と個別に面談し、お子様の成長、強み、今後の課題についてお話しします。当日、生徒は登校しません。</t>
         </is>
       </c>
       <c r="M57" t="inlineStr" s="2">
@@ -5584,7 +5584,7 @@
       </c>
       <c r="O57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-01-14-g10-parent-info-session-high-school-subject-choi.webp</t>
+          <t xml:space="preserve">compass/images/events/2026-10-19-parent-teacher-conferences.webp</t>
         </is>
       </c>
       <c r="P57" t="inlineStr" s="2">
@@ -5611,17 +5611,17 @@
     <row r="58">
       <c r="A58" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-01-22-open-campus</t>
+          <t xml:space="preserve">2027-01-14-g10-parent-info-session-high-school-subject-choi</t>
         </is>
       </c>
       <c r="B58" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-01-22</t>
+          <t xml:space="preserve">2027-01-14</t>
         </is>
       </c>
       <c r="C58" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-01-22</t>
+          <t xml:space="preserve">2027-01-14</t>
         </is>
       </c>
       <c r="D58" t="inlineStr" s="3">
@@ -5631,12 +5631,12 @@
       </c>
       <c r="E58" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Whole School</t>
+          <t xml:space="preserve">Secondary</t>
         </is>
       </c>
       <c r="F58" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="G58" t="inlineStr" s="2">
@@ -5651,22 +5651,22 @@
       </c>
       <c r="I58" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Open Campus</t>
+          <t xml:space="preserve">G10 Parent info Session (High School Subject Choice)</t>
         </is>
       </c>
       <c r="J58" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">オープンキャンパス</t>
+          <t xml:space="preserve">G10保護者向け説明会（高等部科目選択）</t>
         </is>
       </c>
       <c r="K58" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Any person interested in seeing the daily operation of the school is invited to join a tour of the school during its regular hours.</t>
+          <t xml:space="preserve">Grade 10 parents are invited to an information session about DP subject choices and guidance for planning the next stage of their child’s learning.</t>
         </is>
       </c>
       <c r="L58" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">学校の日常の様子にご関心のある方は、通常授業時間中の校内見学にご参加いただけます。</t>
+          <t xml:space="preserve">10年生の保護者の皆様を対象に、DPの科目選択と、お子様の次のステージの学びを計画するためのガイダンスを行います。</t>
         </is>
       </c>
       <c r="M58" t="inlineStr" s="2">
@@ -5681,7 +5681,7 @@
       </c>
       <c r="O58" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-01-22-open-campus.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-01-14-g10-parent-info-session-high-school-subject-choi.webp</t>
         </is>
       </c>
       <c r="P58" t="inlineStr" s="2">
@@ -5708,17 +5708,17 @@
     <row r="59">
       <c r="A59" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-01-23-alumni-talk</t>
+          <t xml:space="preserve">2027-01-22-open-campus</t>
         </is>
       </c>
       <c r="B59" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-01-23</t>
+          <t xml:space="preserve">2027-01-22</t>
         </is>
       </c>
       <c r="C59" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-01-23</t>
+          <t xml:space="preserve">2027-01-22</t>
         </is>
       </c>
       <c r="D59" t="inlineStr" s="3">
@@ -5728,7 +5728,7 @@
       </c>
       <c r="E59" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">High School</t>
+          <t xml:space="preserve">Whole School</t>
         </is>
       </c>
       <c r="F59" t="inlineStr" s="2">
@@ -5748,22 +5748,22 @@
       </c>
       <c r="I59" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Alumni Talk</t>
+          <t xml:space="preserve">Open Campus</t>
         </is>
       </c>
       <c r="J59" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">卒業生トーク</t>
+          <t xml:space="preserve">オープンキャンパス</t>
         </is>
       </c>
       <c r="K59" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Alumni will share their experiences and advice with students, offering insight into life after School and future pathways.</t>
+          <t xml:space="preserve">Any person interested in seeing the daily operation of the school is invited to join a tour of the school during its regular hours.</t>
         </is>
       </c>
       <c r="L59" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">卒業生が自身の経験やアドバイスを生徒に伝え、卒業後の生活や将来の進路について話します。</t>
+          <t xml:space="preserve">学校の日常の様子にご関心のある方は、通常授業時間中の校内見学にご参加いただけます。</t>
         </is>
       </c>
       <c r="M59" t="inlineStr" s="2">
@@ -5778,7 +5778,7 @@
       </c>
       <c r="O59" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-01-23-alumni-talk.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-01-22-open-campus.webp</t>
         </is>
       </c>
       <c r="P59" t="inlineStr" s="2">
@@ -5805,17 +5805,17 @@
     <row r="60">
       <c r="A60" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-01-27-natural-disaster-field-trip</t>
+          <t xml:space="preserve">2027-01-23-alumni-talk</t>
         </is>
       </c>
       <c r="B60" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-01-27</t>
+          <t xml:space="preserve">2027-01-23</t>
         </is>
       </c>
       <c r="C60" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-01-27</t>
+          <t xml:space="preserve">2027-01-23</t>
         </is>
       </c>
       <c r="D60" t="inlineStr" s="3">
@@ -5825,7 +5825,7 @@
       </c>
       <c r="E60" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ELC</t>
+          <t xml:space="preserve">High School</t>
         </is>
       </c>
       <c r="F60" t="inlineStr" s="2">
@@ -5845,22 +5845,22 @@
       </c>
       <c r="I60" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Natural Disaster Field Trip</t>
+          <t xml:space="preserve">Alumni Talk</t>
         </is>
       </c>
       <c r="J60" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">防災校外学習</t>
+          <t xml:space="preserve">卒業生トーク</t>
         </is>
       </c>
       <c r="K60" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students explore disaster preparedness and safety through interactive learning experiences related to natural disasters and emergency response.</t>
+          <t xml:space="preserve">Alumni will share their experiences and advice with students, offering insight into life after School and future pathways.</t>
         </is>
       </c>
       <c r="L60" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">自然災害や緊急時の対応に関する体験型学習を通して、防災と安全について学びます。</t>
+          <t xml:space="preserve">卒業生が自身の経験やアドバイスを生徒に伝え、卒業後の生活や将来の進路について話します。</t>
         </is>
       </c>
       <c r="M60" t="inlineStr" s="2">
@@ -5875,7 +5875,7 @@
       </c>
       <c r="O60" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-01-27-natural-disaster-field-trip.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-01-23-alumni-talk.webp</t>
         </is>
       </c>
       <c r="P60" t="inlineStr" s="2">
@@ -5902,17 +5902,17 @@
     <row r="61">
       <c r="A61" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-01-30-model-united-nations-event-mun</t>
+          <t xml:space="preserve">2027-01-27-natural-disaster-field-trip</t>
         </is>
       </c>
       <c r="B61" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-01-30</t>
+          <t xml:space="preserve">2027-01-27</t>
         </is>
       </c>
       <c r="C61" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-01-30</t>
+          <t xml:space="preserve">2027-01-27</t>
         </is>
       </c>
       <c r="D61" t="inlineStr" s="3">
@@ -5922,7 +5922,7 @@
       </c>
       <c r="E61" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary</t>
+          <t xml:space="preserve">ELC</t>
         </is>
       </c>
       <c r="F61" t="inlineStr" s="2">
@@ -5942,22 +5942,22 @@
       </c>
       <c r="I61" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Model United Nations Event (MUN)</t>
+          <t xml:space="preserve">Natural Disaster Field Trip</t>
         </is>
       </c>
       <c r="J61" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">模擬国連（MUN）</t>
+          <t xml:space="preserve">防災校外学習</t>
         </is>
       </c>
       <c r="K61" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students will participate in Model United Nations, developing public speaking, research, collaboration, and global awareness through discussion of real-world issues.</t>
+          <t xml:space="preserve">Students explore disaster preparedness and safety through interactive learning experiences related to natural disasters and emergency response.</t>
         </is>
       </c>
       <c r="L61" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">模擬国連に参加し、現実の課題について議論することで、スピーチ力、調査力、協働する力、国際的な意識を育みます。</t>
+          <t xml:space="preserve">自然災害や緊急時の対応に関する体験型学習を通して、防災と安全について学びます。</t>
         </is>
       </c>
       <c r="M61" t="inlineStr" s="2">
@@ -5972,7 +5972,7 @@
       </c>
       <c r="O61" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-01-30-model-united-nations-event-mun.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-01-27-natural-disaster-field-trip.webp</t>
         </is>
       </c>
       <c r="P61" t="inlineStr" s="2">
@@ -5999,17 +5999,17 @@
     <row r="62">
       <c r="A62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-02-01-friendly-volleyball-tournament-internal</t>
+          <t xml:space="preserve">2027-01-30-model-united-nations-event-mun</t>
         </is>
       </c>
       <c r="B62" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-02-01</t>
+          <t xml:space="preserve">2027-01-30</t>
         </is>
       </c>
       <c r="C62" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-02-05</t>
+          <t xml:space="preserve">2027-01-30</t>
         </is>
       </c>
       <c r="D62" t="inlineStr" s="3">
@@ -6039,22 +6039,22 @@
       </c>
       <c r="I62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Friendly Volleyball Tournament (Internal)</t>
+          <t xml:space="preserve">Model United Nations Event (MUN)</t>
         </is>
       </c>
       <c r="J62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">校内バレーボール大会</t>
+          <t xml:space="preserve">模擬国連（MUN）</t>
         </is>
       </c>
       <c r="K62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students will take part in a friendly internal volleyball tournament, promoting teamwork, sportsmanship, and school spirit.</t>
+          <t xml:space="preserve">Students will participate in Model United Nations, developing public speaking, research, collaboration, and global awareness through discussion of real-world issues.</t>
         </is>
       </c>
       <c r="L62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">校内バレーボール大会に参加し、チームワーク、スポーツマンシップ、愛校心を育みます。</t>
+          <t xml:space="preserve">模擬国連に参加し、現実の課題について議論することで、スピーチ力、調査力、協働する力、国際的な意識を育みます。</t>
         </is>
       </c>
       <c r="M62" t="inlineStr" s="2">
@@ -6069,7 +6069,7 @@
       </c>
       <c r="O62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-02-01-friendly-volleyball-tournament-internal.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-01-30-model-united-nations-event-mun.webp</t>
         </is>
       </c>
       <c r="P62" t="inlineStr" s="2">
@@ -6096,7 +6096,7 @@
     <row r="63">
       <c r="A63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-02-01-concept-con-language</t>
+          <t xml:space="preserve">2027-02-01-friendly-volleyball-tournament-internal</t>
         </is>
       </c>
       <c r="B63" t="inlineStr" s="3">
@@ -6116,7 +6116,7 @@
       </c>
       <c r="E63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary, ELC</t>
+          <t xml:space="preserve">Secondary</t>
         </is>
       </c>
       <c r="F63" t="inlineStr" s="2">
@@ -6136,22 +6136,22 @@
       </c>
       <c r="I63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Concept Con (Language)</t>
+          <t xml:space="preserve">Friendly Volleyball Tournament (Internal)</t>
         </is>
       </c>
       <c r="J63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">コンセプト・コン（言語）</t>
+          <t xml:space="preserve">校内バレーボール大会</t>
         </is>
       </c>
       <c r="K63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students celebrate language and communication through presentations, performances, and projects that showcase their learning and creativity.</t>
+          <t xml:space="preserve">Students will take part in a friendly internal volleyball tournament, promoting teamwork, sportsmanship, and school spirit.</t>
         </is>
       </c>
       <c r="L63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">学びと創造性を示す発表、パフォーマンス、プロジェクトを通して、言語とコミュニケーションを祝います。</t>
+          <t xml:space="preserve">校内バレーボール大会に参加し、チームワーク、スポーツマンシップ、愛校心を育みます。</t>
         </is>
       </c>
       <c r="M63" t="inlineStr" s="2">
@@ -6166,7 +6166,7 @@
       </c>
       <c r="O63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-02-01-concept-con-language.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-02-01-friendly-volleyball-tournament-internal.webp</t>
         </is>
       </c>
       <c r="P63" t="inlineStr" s="2">
@@ -6193,17 +6193,17 @@
     <row r="64">
       <c r="A64" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-02-18-career-support-second-career-roundtable-and-care</t>
+          <t xml:space="preserve">2027-02-01-concept-con-language</t>
         </is>
       </c>
       <c r="B64" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-02-18</t>
+          <t xml:space="preserve">2027-02-01</t>
         </is>
       </c>
       <c r="C64" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-02-18</t>
+          <t xml:space="preserve">2027-02-05</t>
         </is>
       </c>
       <c r="D64" t="inlineStr" s="3">
@@ -6213,12 +6213,12 @@
       </c>
       <c r="E64" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">High School</t>
+          <t xml:space="preserve">Primary, ELC</t>
         </is>
       </c>
       <c r="F64" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G64" t="inlineStr" s="2">
@@ -6233,22 +6233,22 @@
       </c>
       <c r="I64" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Career Support: Second Career Roundtable and Career Fair</t>
+          <t xml:space="preserve">Concept Con (Language)</t>
         </is>
       </c>
       <c r="J64" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">進路支援：第2回キャリア座談会・キャリアフェア</t>
+          <t xml:space="preserve">コンセプト・コン（言語）</t>
         </is>
       </c>
       <c r="K64" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">An informative event where students and parents can learn about IB university admissions, holistic admissions strategies in Japan and abroad, and explore future academic and career opportunities through discussions with experts and representatives.</t>
+          <t xml:space="preserve">Students celebrate language and communication through presentations, performances, and projects that showcase their learning and creativity.</t>
         </is>
       </c>
       <c r="L64" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">専門家や関係者との対話を通して、生徒と保護者の皆様がIBでの大学入試、国内外の総合型選抜の戦略について学び、将来の進学やキャリアの可能性を探る説明会です。</t>
+          <t xml:space="preserve">学びと創造性を示す発表、パフォーマンス、プロジェクトを通して、言語とコミュニケーションを祝います。</t>
         </is>
       </c>
       <c r="M64" t="inlineStr" s="2">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="O64" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-02-18-career-support-second-career-roundtable-and-care.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-02-01-concept-con-language.webp</t>
         </is>
       </c>
       <c r="P64" t="inlineStr" s="2">
@@ -6290,17 +6290,17 @@
     <row r="65">
       <c r="A65" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-02-19-collective-field-trip</t>
+          <t xml:space="preserve">2027-02-18-career-support-second-career-roundtable-and-care</t>
         </is>
       </c>
       <c r="B65" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-02-19</t>
+          <t xml:space="preserve">2027-02-18</t>
         </is>
       </c>
       <c r="C65" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-02-19</t>
+          <t xml:space="preserve">2027-02-18</t>
         </is>
       </c>
       <c r="D65" t="inlineStr" s="3">
@@ -6310,12 +6310,12 @@
       </c>
       <c r="E65" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary</t>
+          <t xml:space="preserve">High School</t>
         </is>
       </c>
       <c r="F65" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="G65" t="inlineStr" s="2">
@@ -6330,22 +6330,22 @@
       </c>
       <c r="I65" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Collective Field Trip</t>
+          <t xml:space="preserve">Career Support: Second Career Roundtable and Career Fair</t>
         </is>
       </c>
       <c r="J65" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">合同校外学習</t>
+          <t xml:space="preserve">進路支援：第2回キャリア座談会・キャリアフェア</t>
         </is>
       </c>
       <c r="K65" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students participate in an off-campus learning experience that connects classroom learning with real-world exploration and discovery.</t>
+          <t xml:space="preserve">An informative event where students and parents can learn about IB university admissions, holistic admissions strategies in Japan and abroad, and explore future academic and career opportunities through discussions with experts and representatives.</t>
         </is>
       </c>
       <c r="L65" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">校外での学習体験を通して、教室での学びを実社会での探究や発見と結びつけます。</t>
+          <t xml:space="preserve">専門家や関係者との対話を通して、生徒と保護者の皆様がIBでの大学入試、国内外の総合型選抜の戦略について学び、将来の進学やキャリアの可能性を探る説明会です。</t>
         </is>
       </c>
       <c r="M65" t="inlineStr" s="2">
@@ -6360,7 +6360,7 @@
       </c>
       <c r="O65" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-02-19-collective-field-trip.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-02-18-career-support-second-career-roundtable-and-care.webp</t>
         </is>
       </c>
       <c r="P65" t="inlineStr" s="2">
@@ -6387,17 +6387,17 @@
     <row r="66">
       <c r="A66" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-02-22-world-thinking-day</t>
+          <t xml:space="preserve">2027-02-19-collective-field-trip</t>
         </is>
       </c>
       <c r="B66" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-02-22</t>
+          <t xml:space="preserve">2027-02-19</t>
         </is>
       </c>
       <c r="C66" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-02-22</t>
+          <t xml:space="preserve">2027-02-19</t>
         </is>
       </c>
       <c r="D66" t="inlineStr" s="3">
@@ -6407,7 +6407,7 @@
       </c>
       <c r="E66" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary, ELC</t>
+          <t xml:space="preserve">Primary</t>
         </is>
       </c>
       <c r="F66" t="inlineStr" s="2">
@@ -6427,22 +6427,22 @@
       </c>
       <c r="I66" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">World Thinking Day</t>
+          <t xml:space="preserve">Collective Field Trip</t>
         </is>
       </c>
       <c r="J66" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ワールド・シンキング・デー</t>
+          <t xml:space="preserve">合同校外学習</t>
         </is>
       </c>
       <c r="K66" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students learn about cultures, traditions, and global citizenship while celebrating international understanding and connection.</t>
+          <t xml:space="preserve">Students participate in an off-campus learning experience that connects classroom learning with real-world exploration and discovery.</t>
         </is>
       </c>
       <c r="L66" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">国際理解とつながりを祝いながら、さまざまな文化や伝統、地球市民としてのあり方について学びます。</t>
+          <t xml:space="preserve">校外での学習体験を通して、教室での学びを実社会での探究や発見と結びつけます。</t>
         </is>
       </c>
       <c r="M66" t="inlineStr" s="2">
@@ -6457,7 +6457,7 @@
       </c>
       <c r="O66" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-02-22-world-thinking-day.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-02-19-collective-field-trip.webp</t>
         </is>
       </c>
       <c r="P66" t="inlineStr" s="2">
@@ -6484,7 +6484,7 @@
     <row r="67">
       <c r="A67" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-02-22-secondary-sports-day-rehearsal-1</t>
+          <t xml:space="preserve">2027-02-22-world-thinking-day</t>
         </is>
       </c>
       <c r="B67" t="inlineStr" s="3">
@@ -6504,7 +6504,7 @@
       </c>
       <c r="E67" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary</t>
+          <t xml:space="preserve">Primary, ELC</t>
         </is>
       </c>
       <c r="F67" t="inlineStr" s="2">
@@ -6524,22 +6524,22 @@
       </c>
       <c r="I67" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary Sports Day Rehearsal #1</t>
+          <t xml:space="preserve">World Thinking Day</t>
         </is>
       </c>
       <c r="J67" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">中等部運動会リハーサル #1</t>
+          <t xml:space="preserve">ワールド・シンキング・デー</t>
         </is>
       </c>
       <c r="K67" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary students will prepare for Sports Day by practicing event routines, team organization, and activity expectations.</t>
+          <t xml:space="preserve">Students learn about cultures, traditions, and global citizenship while celebrating international understanding and connection.</t>
         </is>
       </c>
       <c r="L67" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">中等部の生徒が、種目の流れ、チーム編成、活動のルールを練習し、運動会に向けて準備します。</t>
+          <t xml:space="preserve">国際理解とつながりを祝いながら、さまざまな文化や伝統、地球市民としてのあり方について学びます。</t>
         </is>
       </c>
       <c r="M67" t="inlineStr" s="2">
@@ -6554,7 +6554,7 @@
       </c>
       <c r="O67" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-02-22-secondary-sports-day-rehearsal-1.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-02-22-world-thinking-day.webp</t>
         </is>
       </c>
       <c r="P67" t="inlineStr" s="2">
@@ -6581,17 +6581,17 @@
     <row r="68">
       <c r="A68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-02-25-primary-sports-day-rehearsal-1</t>
+          <t xml:space="preserve">2027-02-22-secondary-sports-day-rehearsal-1</t>
         </is>
       </c>
       <c r="B68" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-02-25</t>
+          <t xml:space="preserve">2027-02-22</t>
         </is>
       </c>
       <c r="C68" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-02-25</t>
+          <t xml:space="preserve">2027-02-22</t>
         </is>
       </c>
       <c r="D68" t="inlineStr" s="3">
@@ -6601,7 +6601,7 @@
       </c>
       <c r="E68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary</t>
+          <t xml:space="preserve">Secondary</t>
         </is>
       </c>
       <c r="F68" t="inlineStr" s="2">
@@ -6621,22 +6621,22 @@
       </c>
       <c r="I68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary Sports Day Rehearsal #1</t>
+          <t xml:space="preserve">Secondary Sports Day Rehearsal #1</t>
         </is>
       </c>
       <c r="J68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">小学部運動会リハーサル #1</t>
+          <t xml:space="preserve">中等部運動会リハーサル #1</t>
         </is>
       </c>
       <c r="K68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students begin preparing for Sports Day by practicing events, routines, and teamwork activities.</t>
+          <t xml:space="preserve">Secondary students will prepare for Sports Day by practicing event routines, team organization, and activity expectations.</t>
         </is>
       </c>
       <c r="L68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">種目、流れ、チームワークの練習を通して、運動会に向けた準備を始めます。</t>
+          <t xml:space="preserve">中等部の生徒が、種目の流れ、チーム編成、活動のルールを練習し、運動会に向けて準備します。</t>
         </is>
       </c>
       <c r="M68" t="inlineStr" s="2">
@@ -6651,7 +6651,7 @@
       </c>
       <c r="O68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-02-25-primary-sports-day-rehearsal-1.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-02-22-secondary-sports-day-rehearsal-1.webp</t>
         </is>
       </c>
       <c r="P68" t="inlineStr" s="2">
@@ -6678,17 +6678,17 @@
     <row r="69">
       <c r="A69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-02-26-parents-morning-2</t>
+          <t xml:space="preserve">2027-02-25-primary-sports-day-rehearsal-1</t>
         </is>
       </c>
       <c r="B69" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-02-26</t>
+          <t xml:space="preserve">2027-02-25</t>
         </is>
       </c>
       <c r="C69" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-02-26</t>
+          <t xml:space="preserve">2027-02-25</t>
         </is>
       </c>
       <c r="D69" t="inlineStr" s="3">
@@ -6698,12 +6698,12 @@
       </c>
       <c r="E69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary, ELC</t>
+          <t xml:space="preserve">Primary</t>
         </is>
       </c>
       <c r="F69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G69" t="inlineStr" s="2">
@@ -6718,22 +6718,22 @@
       </c>
       <c r="I69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Parents Morning #2</t>
+          <t xml:space="preserve">Primary Sports Day Rehearsal #1</t>
         </is>
       </c>
       <c r="J69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">朝の授業参観 #2</t>
+          <t xml:space="preserve">小学部運動会リハーサル #1</t>
         </is>
       </c>
       <c r="K69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ELC and Primary Parents are invited to come and see the lessons in the morning and experience the morning routines with their child.</t>
+          <t xml:space="preserve">Students begin preparing for Sports Day by practicing events, routines, and teamwork activities.</t>
         </is>
       </c>
       <c r="L69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">幼稚部・小学部の保護者の皆様をお招きし、朝の授業をご参観いただき、お子様と一緒に朝の日課を体験していただきます。</t>
+          <t xml:space="preserve">種目、流れ、チームワークの練習を通して、運動会に向けた準備を始めます。</t>
         </is>
       </c>
       <c r="M69" t="inlineStr" s="2">
@@ -6748,7 +6748,7 @@
       </c>
       <c r="O69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-02-26-parents-morning-2.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-02-25-primary-sports-day-rehearsal-1.webp</t>
         </is>
       </c>
       <c r="P69" t="inlineStr" s="2">
@@ -6775,7 +6775,7 @@
     <row r="70">
       <c r="A70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-02-26-eagle-talks</t>
+          <t xml:space="preserve">2027-02-26-parents-morning-2</t>
         </is>
       </c>
       <c r="B70" t="inlineStr" s="3">
@@ -6815,22 +6815,22 @@
       </c>
       <c r="I70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Eagle Talks</t>
+          <t xml:space="preserve">Parents Morning #2</t>
         </is>
       </c>
       <c r="J70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">イーグル・トーク</t>
+          <t xml:space="preserve">朝の授業参観 #2</t>
         </is>
       </c>
       <c r="K70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students share ideas, experiences, and learning through short presentations designed to build confidence, communication, and leadership skills.</t>
+          <t xml:space="preserve">ELC and Primary Parents are invited to come and see the lessons in the morning and experience the morning routines with their child.</t>
         </is>
       </c>
       <c r="L70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">短いプレゼンテーションを通して考えや経験、学びを共有し、自信、コミュニケーション力、リーダーシップを育みます。</t>
+          <t xml:space="preserve">幼稚部・小学部の保護者の皆様をお招きし、朝の授業をご参観いただき、お子様と一緒に朝の日課を体験していただきます。</t>
         </is>
       </c>
       <c r="M70" t="inlineStr" s="2">
@@ -6845,7 +6845,7 @@
       </c>
       <c r="O70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-02-26-eagle-talks.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-02-26-parents-morning-2.webp</t>
         </is>
       </c>
       <c r="P70" t="inlineStr" s="2">
@@ -6872,17 +6872,17 @@
     <row r="71">
       <c r="A71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-03-04-grade-1-2-musical</t>
+          <t xml:space="preserve">2027-02-26-eagle-talks</t>
         </is>
       </c>
       <c r="B71" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-03-04</t>
+          <t xml:space="preserve">2027-02-26</t>
         </is>
       </c>
       <c r="C71" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-03-05</t>
+          <t xml:space="preserve">2027-02-26</t>
         </is>
       </c>
       <c r="D71" t="inlineStr" s="3">
@@ -6892,7 +6892,7 @@
       </c>
       <c r="E71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary</t>
+          <t xml:space="preserve">Primary, ELC</t>
         </is>
       </c>
       <c r="F71" t="inlineStr" s="2">
@@ -6912,22 +6912,22 @@
       </c>
       <c r="I71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Grade 1, 2 Musical</t>
+          <t xml:space="preserve">Eagle Talks</t>
         </is>
       </c>
       <c r="J71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1・2年生ミュージカル</t>
+          <t xml:space="preserve">イーグル・トーク</t>
         </is>
       </c>
       <c r="K71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students showcase their creativity and confidence through a musical performance featuring songs, acting, and teamwork.</t>
+          <t xml:space="preserve">Students share ideas, experiences, and learning through short presentations designed to build confidence, communication, and leadership skills.</t>
         </is>
       </c>
       <c r="L71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">歌、演技、チームワークによるミュージカルを通して、創造性と自信あふれる姿を披露します。</t>
+          <t xml:space="preserve">短いプレゼンテーションを通して考えや経験、学びを共有し、自信、コミュニケーション力、リーダーシップを育みます。</t>
         </is>
       </c>
       <c r="M71" t="inlineStr" s="2">
@@ -6942,7 +6942,7 @@
       </c>
       <c r="O71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-03-04-grade-1-2-musical.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-02-26-eagle-talks.webp</t>
         </is>
       </c>
       <c r="P71" t="inlineStr" s="2">
@@ -6969,19 +6969,19 @@
     <row r="72">
       <c r="A72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-03-05-higashiyama-zoo-botanical-garden</t>
+          <t xml:space="preserve">2027-03-04-grade-1-2-musical</t>
         </is>
       </c>
       <c r="B72" t="inlineStr" s="3">
         <is>
+          <t xml:space="preserve">2027-03-04</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr" s="3">
+        <is>
           <t xml:space="preserve">2027-03-05</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">2027-03-05</t>
-        </is>
-      </c>
       <c r="D72" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
@@ -6989,12 +6989,12 @@
       </c>
       <c r="E72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary</t>
+          <t xml:space="preserve">Primary</t>
         </is>
       </c>
       <c r="F72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="G72" t="inlineStr" s="2">
@@ -7009,22 +7009,22 @@
       </c>
       <c r="I72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Higashiyama Zoo &amp; Botanical Garden</t>
+          <t xml:space="preserve">Grade 1, 2 Musical</t>
         </is>
       </c>
       <c r="J72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">東山動植物園</t>
+          <t xml:space="preserve">1・2年生ミュージカル</t>
         </is>
       </c>
       <c r="K72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Grade 7 Science students will visit Higashiyama Zoo and Botanical Gardens to support their learning through observation and real-world examples.</t>
+          <t xml:space="preserve">Students showcase their creativity and confidence through a musical performance featuring songs, acting, and teamwork.</t>
         </is>
       </c>
       <c r="L72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">7年生が理科の学習の一環として東山動植物園を訪れ、観察や実物を通して学びを深めます。</t>
+          <t xml:space="preserve">歌、演技、チームワークによるミュージカルを通して、創造性と自信あふれる姿を披露します。</t>
         </is>
       </c>
       <c r="M72" t="inlineStr" s="2">
@@ -7039,7 +7039,7 @@
       </c>
       <c r="O72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-03-05-higashiyama-zoo-botanical-garden.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-03-04-grade-1-2-musical.webp</t>
         </is>
       </c>
       <c r="P72" t="inlineStr" s="2">
@@ -7066,17 +7066,17 @@
     <row r="73">
       <c r="A73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-03-06-sat-test-6</t>
+          <t xml:space="preserve">2027-03-05-higashiyama-zoo-botanical-garden</t>
         </is>
       </c>
       <c r="B73" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-03-06</t>
+          <t xml:space="preserve">2027-03-05</t>
         </is>
       </c>
       <c r="C73" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-03-06</t>
+          <t xml:space="preserve">2027-03-05</t>
         </is>
       </c>
       <c r="D73" t="inlineStr" s="3">
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">High School</t>
+          <t xml:space="preserve">Secondary</t>
         </is>
       </c>
       <c r="F73" t="inlineStr" s="2">
@@ -7106,22 +7106,22 @@
       </c>
       <c r="I73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SAT Test #6</t>
+          <t xml:space="preserve">Higashiyama Zoo &amp; Botanical Garden</t>
         </is>
       </c>
       <c r="J73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SAT試験 第6回</t>
+          <t xml:space="preserve">東山動植物園</t>
         </is>
       </c>
       <c r="K73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">An internationally recognized university entrance exam. Our school is an official SAT test center, and both Enishi students and external students are welcome to take the test on campus.</t>
+          <t xml:space="preserve">Grade 7 Science students will visit Higashiyama Zoo and Botanical Gardens to support their learning through observation and real-world examples.</t>
         </is>
       </c>
       <c r="L73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">国際的に認められた大学入学試験です。本校はSAT公式試験会場であり、本校生徒・外部生徒ともに校内で受験できます。</t>
+          <t xml:space="preserve">7年生が理科の学習の一環として東山動植物園を訪れ、観察や実物を通して学びを深めます。</t>
         </is>
       </c>
       <c r="M73" t="inlineStr" s="2">
@@ -7136,7 +7136,7 @@
       </c>
       <c r="O73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-03-06-sat-test-6.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-03-05-higashiyama-zoo-botanical-garden.webp</t>
         </is>
       </c>
       <c r="P73" t="inlineStr" s="2">
@@ -7163,17 +7163,17 @@
     <row r="74">
       <c r="A74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-03-09-primary-sports-day-rehearsal-2</t>
+          <t xml:space="preserve">2027-03-06-sat-test-6</t>
         </is>
       </c>
       <c r="B74" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-03-09</t>
+          <t xml:space="preserve">2027-03-06</t>
         </is>
       </c>
       <c r="C74" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-03-09</t>
+          <t xml:space="preserve">2027-03-06</t>
         </is>
       </c>
       <c r="D74" t="inlineStr" s="3">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="E74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary</t>
+          <t xml:space="preserve">High School</t>
         </is>
       </c>
       <c r="F74" t="inlineStr" s="2">
@@ -7203,22 +7203,22 @@
       </c>
       <c r="I74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary Sports Day Rehearsal #2</t>
+          <t xml:space="preserve">SAT Test #6</t>
         </is>
       </c>
       <c r="J74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">小学部運動会リハーサル #2</t>
+          <t xml:space="preserve">SAT試験 第6回</t>
         </is>
       </c>
       <c r="K74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students continue building skills and confidence as they prepare for Sports Day events and activities.</t>
+          <t xml:space="preserve">An internationally recognized university entrance exam. Our school is an official SAT test center, and both Enishi students and external students are welcome to take the test on campus.</t>
         </is>
       </c>
       <c r="L74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">運動会の種目や活動に向けて準備を進めながら、技能と自信をさらに高めます。</t>
+          <t xml:space="preserve">国際的に認められた大学入学試験です。本校はSAT公式試験会場であり、本校生徒・外部生徒ともに校内で受験できます。</t>
         </is>
       </c>
       <c r="M74" t="inlineStr" s="2">
@@ -7233,7 +7233,7 @@
       </c>
       <c r="O74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-03-09-primary-sports-day-rehearsal-2.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-03-06-sat-test-6.webp</t>
         </is>
       </c>
       <c r="P74" t="inlineStr" s="2">
@@ -7260,17 +7260,17 @@
     <row r="75">
       <c r="A75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-03-12-secondary-sports-day-rehearsal-2</t>
+          <t xml:space="preserve">2027-03-09-primary-sports-day-rehearsal-2</t>
         </is>
       </c>
       <c r="B75" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-03-12</t>
+          <t xml:space="preserve">2027-03-09</t>
         </is>
       </c>
       <c r="C75" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-03-12</t>
+          <t xml:space="preserve">2027-03-09</t>
         </is>
       </c>
       <c r="D75" t="inlineStr" s="3">
@@ -7280,7 +7280,7 @@
       </c>
       <c r="E75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary</t>
+          <t xml:space="preserve">Primary</t>
         </is>
       </c>
       <c r="F75" t="inlineStr" s="2">
@@ -7300,22 +7300,22 @@
       </c>
       <c r="I75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary Sports Day Rehearsal #2</t>
+          <t xml:space="preserve">Primary Sports Day Rehearsal #2</t>
         </is>
       </c>
       <c r="J75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">中等部運動会リハーサル #2</t>
+          <t xml:space="preserve">小学部運動会リハーサル #2</t>
         </is>
       </c>
       <c r="K75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary students will prepare for Sports Day by practicing event routines, team organization, and activity expectations.</t>
+          <t xml:space="preserve">Students continue building skills and confidence as they prepare for Sports Day events and activities.</t>
         </is>
       </c>
       <c r="L75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">中等部の生徒が、種目の流れ、チーム編成、活動のルールを練習し、運動会に向けて準備します。</t>
+          <t xml:space="preserve">運動会の種目や活動に向けて準備を進めながら、技能と自信をさらに高めます。</t>
         </is>
       </c>
       <c r="M75" t="inlineStr" s="2">
@@ -7330,7 +7330,7 @@
       </c>
       <c r="O75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-03-12-secondary-sports-day-rehearsal-2.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-03-09-primary-sports-day-rehearsal-2.webp</t>
         </is>
       </c>
       <c r="P75" t="inlineStr" s="2">
@@ -7357,17 +7357,17 @@
     <row r="76">
       <c r="A76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-03-18-japanese-culture-day</t>
+          <t xml:space="preserve">2027-03-12-secondary-sports-day-rehearsal-2</t>
         </is>
       </c>
       <c r="B76" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-03-18</t>
+          <t xml:space="preserve">2027-03-12</t>
         </is>
       </c>
       <c r="C76" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-03-18</t>
+          <t xml:space="preserve">2027-03-12</t>
         </is>
       </c>
       <c r="D76" t="inlineStr" s="3">
@@ -7377,12 +7377,12 @@
       </c>
       <c r="E76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Whole School</t>
+          <t xml:space="preserve">Secondary</t>
         </is>
       </c>
       <c r="F76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G76" t="inlineStr" s="2">
@@ -7397,22 +7397,22 @@
       </c>
       <c r="I76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Japanese Culture Day</t>
+          <t xml:space="preserve">Secondary Sports Day Rehearsal #2</t>
         </is>
       </c>
       <c r="J76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">日本文化デー</t>
+          <t xml:space="preserve">中等部運動会リハーサル #2</t>
         </is>
       </c>
       <c r="K76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students will deepen their understanding and appreciation of Japanese culture through a variety of interactive activities with school community.</t>
+          <t xml:space="preserve">Secondary students will prepare for Sports Day by practicing event routines, team organization, and activity expectations.</t>
         </is>
       </c>
       <c r="L76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">学校コミュニティとともにさまざまな体験型の活動に取り組み、日本文化への理解と関心を深めます。</t>
+          <t xml:space="preserve">中等部の生徒が、種目の流れ、チーム編成、活動のルールを練習し、運動会に向けて準備します。</t>
         </is>
       </c>
       <c r="M76" t="inlineStr" s="2">
@@ -7427,7 +7427,7 @@
       </c>
       <c r="O76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-03-18-japanese-culture-day.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-03-12-secondary-sports-day-rehearsal-2.webp</t>
         </is>
       </c>
       <c r="P76" t="inlineStr" s="2">
@@ -7454,17 +7454,17 @@
     <row r="77">
       <c r="A77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-03-19-eagle-bucks-store</t>
+          <t xml:space="preserve">2027-03-18-japanese-culture-day</t>
         </is>
       </c>
       <c r="B77" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-03-19</t>
+          <t xml:space="preserve">2027-03-18</t>
         </is>
       </c>
       <c r="C77" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-03-19</t>
+          <t xml:space="preserve">2027-03-18</t>
         </is>
       </c>
       <c r="D77" t="inlineStr" s="3">
@@ -7474,12 +7474,12 @@
       </c>
       <c r="E77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary, ELC</t>
+          <t xml:space="preserve">Whole School</t>
         </is>
       </c>
       <c r="F77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="G77" t="inlineStr" s="2">
@@ -7494,22 +7494,22 @@
       </c>
       <c r="I77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Eagle Bucks Store</t>
+          <t xml:space="preserve">Japanese Culture Day</t>
         </is>
       </c>
       <c r="J77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">イーグルバックス・ストア</t>
+          <t xml:space="preserve">日本文化デー</t>
         </is>
       </c>
       <c r="K77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students can use their earned Eagle Bucks to purchase rewards and special items. The store reinforces positive behavior, responsibility, and goal-setting.</t>
+          <t xml:space="preserve">Students will deepen their understanding and appreciation of Japanese culture through a variety of interactive activities with school community.</t>
         </is>
       </c>
       <c r="L77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">獲得したイーグルバックスを使って、ごほうびや特別なアイテムと交換できます。前向きな行動、責任感、目標設定を後押しする取り組みです。</t>
+          <t xml:space="preserve">学校コミュニティとともにさまざまな体験型の活動に取り組み、日本文化への理解と関心を深めます。</t>
         </is>
       </c>
       <c r="M77" t="inlineStr" s="2">
@@ -7524,7 +7524,7 @@
       </c>
       <c r="O77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-03-19-eagle-bucks-store.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-03-18-japanese-culture-day.webp</t>
         </is>
       </c>
       <c r="P77" t="inlineStr" s="2">
@@ -7551,7 +7551,7 @@
     <row r="78">
       <c r="A78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-03-19-tea-party-pta-for-all</t>
+          <t xml:space="preserve">2027-03-19-eagle-bucks-store</t>
         </is>
       </c>
       <c r="B78" t="inlineStr" s="3">
@@ -7571,12 +7571,12 @@
       </c>
       <c r="E78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PTA</t>
+          <t xml:space="preserve">Primary, ELC</t>
         </is>
       </c>
       <c r="F78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G78" t="inlineStr" s="2">
@@ -7591,22 +7591,22 @@
       </c>
       <c r="I78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Tea Party / PTA for all</t>
+          <t xml:space="preserve">Eagle Bucks Store</t>
         </is>
       </c>
       <c r="J78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PTAティーパーティー（どなたでも参加できます）</t>
+          <t xml:space="preserve">イーグルバックス・ストア</t>
         </is>
       </c>
       <c r="K78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">A social gathering organized by the PTA and Community Club where staff and students are welcome to enjoy a variety of teas, snacks, and friendly conversation together.</t>
+          <t xml:space="preserve">Students can use their earned Eagle Bucks to purchase rewards and special items. The store reinforces positive behavior, responsibility, and goal-setting.</t>
         </is>
       </c>
       <c r="L78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PTAとコミュニティクラブが主催する交流会です。教職員や生徒も参加でき、さまざまなお茶や軽食、和やかな会話を楽しめます。</t>
+          <t xml:space="preserve">獲得したイーグルバックスを使って、ごほうびや特別なアイテムと交換できます。前向きな行動、責任感、目標設定を後押しする取り組みです。</t>
         </is>
       </c>
       <c r="M78" t="inlineStr" s="2">
@@ -7621,7 +7621,7 @@
       </c>
       <c r="O78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-03-19-tea-party-pta-for-all.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-03-19-eagle-bucks-store.webp</t>
         </is>
       </c>
       <c r="P78" t="inlineStr" s="2">
@@ -7648,7 +7648,7 @@
     <row r="79">
       <c r="A79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-03-19-end-of-term-2-activity-g9-12</t>
+          <t xml:space="preserve">2027-03-19-tea-party-pta-for-all</t>
         </is>
       </c>
       <c r="B79" t="inlineStr" s="3">
@@ -7658,7 +7658,7 @@
       </c>
       <c r="C79" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-03-20</t>
+          <t xml:space="preserve">2027-03-19</t>
         </is>
       </c>
       <c r="D79" t="inlineStr" s="3">
@@ -7668,12 +7668,12 @@
       </c>
       <c r="E79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">High School</t>
+          <t xml:space="preserve">PTA</t>
         </is>
       </c>
       <c r="F79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="G79" t="inlineStr" s="2">
@@ -7688,22 +7688,22 @@
       </c>
       <c r="I79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">End of Term 2 Activity: G9-12</t>
+          <t xml:space="preserve">Tea Party / PTA for all</t>
         </is>
       </c>
       <c r="J79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">第2学期末行事：G9–12</t>
+          <t xml:space="preserve">PTAティーパーティー（どなたでも参加できます）</t>
         </is>
       </c>
       <c r="K79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students will take part in an off-campus day trip activity to celebrate the end of Term 2.</t>
+          <t xml:space="preserve">A social gathering organized by the PTA and Community Club where staff and students are welcome to enjoy a variety of teas, snacks, and friendly conversation together.</t>
         </is>
       </c>
       <c r="L79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">第2学期の終わりを祝い、校外への日帰り活動に参加します。</t>
+          <t xml:space="preserve">PTAとコミュニティクラブが主催する交流会です。教職員や生徒も参加でき、さまざまなお茶や軽食、和やかな会話を楽しめます。</t>
         </is>
       </c>
       <c r="M79" t="inlineStr" s="2">
@@ -7718,7 +7718,7 @@
       </c>
       <c r="O79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-03-19-end-of-term-2-activity-g9-12.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-03-19-tea-party-pta-for-all.webp</t>
         </is>
       </c>
       <c r="P79" t="inlineStr" s="2">
@@ -7745,19 +7745,19 @@
     <row r="80">
       <c r="A80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-03-20-end-of-term-2-activity-g6-8</t>
+          <t xml:space="preserve">2027-03-19-end-of-term-2-activity-g9-12</t>
         </is>
       </c>
       <c r="B80" t="inlineStr" s="3">
         <is>
+          <t xml:space="preserve">2027-03-19</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr" s="3">
+        <is>
           <t xml:space="preserve">2027-03-20</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">2027-03-21</t>
-        </is>
-      </c>
       <c r="D80" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
@@ -7765,7 +7765,7 @@
       </c>
       <c r="E80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary</t>
+          <t xml:space="preserve">High School</t>
         </is>
       </c>
       <c r="F80" t="inlineStr" s="2">
@@ -7785,22 +7785,22 @@
       </c>
       <c r="I80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">End of Term 2 Activity: G6-8</t>
+          <t xml:space="preserve">End of Term 2 Activity: G9-12</t>
         </is>
       </c>
       <c r="J80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">第2学期末行事：G6–8</t>
+          <t xml:space="preserve">第2学期末行事：G9–12</t>
         </is>
       </c>
       <c r="K80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students will take part in an overnight camp at an off-campus camping facility to celebrate the end of Term 2.</t>
+          <t xml:space="preserve">Students will take part in an off-campus day trip activity to celebrate the end of Term 2.</t>
         </is>
       </c>
       <c r="L80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">第2学期の終わりを祝い、校外のキャンプ施設での一泊キャンプに参加します。</t>
+          <t xml:space="preserve">第2学期の終わりを祝い、校外への日帰り活動に参加します。</t>
         </is>
       </c>
       <c r="M80" t="inlineStr" s="2">
@@ -7815,7 +7815,7 @@
       </c>
       <c r="O80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-03-20-end-of-term-2-activity-g6-8.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-03-19-end-of-term-2-activity-g9-12.webp</t>
         </is>
       </c>
       <c r="P80" t="inlineStr" s="2">
@@ -7842,17 +7842,17 @@
     <row r="81">
       <c r="A81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-03-30-parent-teacher-conferences</t>
+          <t xml:space="preserve">2027-03-20-end-of-term-2-activity-g6-8</t>
         </is>
       </c>
       <c r="B81" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-03-30</t>
+          <t xml:space="preserve">2027-03-20</t>
         </is>
       </c>
       <c r="C81" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-03-30</t>
+          <t xml:space="preserve">2027-03-21</t>
         </is>
       </c>
       <c r="D81" t="inlineStr" s="3">
@@ -7862,17 +7862,17 @@
       </c>
       <c r="E81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Whole School</t>
+          <t xml:space="preserve">Secondary</t>
         </is>
       </c>
       <c r="F81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H81" t="inlineStr" s="2">
@@ -7882,22 +7882,22 @@
       </c>
       <c r="I81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Parent Teacher Conferences</t>
+          <t xml:space="preserve">End of Term 2 Activity: G6-8</t>
         </is>
       </c>
       <c r="J81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">保護者面談</t>
+          <t xml:space="preserve">第2学期末行事：G6–8</t>
         </is>
       </c>
       <c r="K81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Parents meet one-on-one with each teacher to discuss their child's progress, strengths, and next steps. The school campus is closed to students on this day.</t>
+          <t xml:space="preserve">Students will take part in an overnight camp at an off-campus camping facility to celebrate the end of Term 2.</t>
         </is>
       </c>
       <c r="L81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">保護者の皆様が各担当教員と個別に面談し、お子様の成長、強み、今後の課題についてお話しします。当日、生徒は登校しません。</t>
+          <t xml:space="preserve">第2学期の終わりを祝い、校外のキャンプ施設での一泊キャンプに参加します。</t>
         </is>
       </c>
       <c r="M81" t="inlineStr" s="2">
@@ -7912,7 +7912,7 @@
       </c>
       <c r="O81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-03-30-parent-teacher-conferences.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-03-20-end-of-term-2-activity-g6-8.webp</t>
         </is>
       </c>
       <c r="P81" t="inlineStr" s="2">
@@ -7939,17 +7939,17 @@
     <row r="82">
       <c r="A82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-03-31-secondary-sports-day-rehearsal-3</t>
+          <t xml:space="preserve">2027-03-30-parent-teacher-conferences</t>
         </is>
       </c>
       <c r="B82" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-03-31</t>
+          <t xml:space="preserve">2027-03-30</t>
         </is>
       </c>
       <c r="C82" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-03-31</t>
+          <t xml:space="preserve">2027-03-30</t>
         </is>
       </c>
       <c r="D82" t="inlineStr" s="3">
@@ -7959,17 +7959,17 @@
       </c>
       <c r="E82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary</t>
+          <t xml:space="preserve">Whole School</t>
         </is>
       </c>
       <c r="F82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="G82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="H82" t="inlineStr" s="2">
@@ -7979,22 +7979,22 @@
       </c>
       <c r="I82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary Sports Day Rehearsal #3</t>
+          <t xml:space="preserve">Parent Teacher Conferences</t>
         </is>
       </c>
       <c r="J82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">中等部運動会リハーサル #3</t>
+          <t xml:space="preserve">保護者面談</t>
         </is>
       </c>
       <c r="K82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary students will prepare for Sports Day by practicing event routines, team organization, and activity expectations.</t>
+          <t xml:space="preserve">Parents meet one-on-one with each teacher to discuss their child's progress, strengths, and next steps. The school campus is closed to students on this day.</t>
         </is>
       </c>
       <c r="L82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">中等部の生徒が、種目の流れ、チーム編成、活動のルールを練習し、運動会に向けて準備します。</t>
+          <t xml:space="preserve">保護者の皆様が各担当教員と個別に面談し、お子様の成長、強み、今後の課題についてお話しします。当日、生徒は登校しません。</t>
         </is>
       </c>
       <c r="M82" t="inlineStr" s="2">
@@ -8009,7 +8009,7 @@
       </c>
       <c r="O82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-03-31-secondary-sports-day-rehearsal-3.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-03-30-parent-teacher-conferences.webp</t>
         </is>
       </c>
       <c r="P82" t="inlineStr" s="2">
@@ -8036,17 +8036,17 @@
     <row r="83">
       <c r="A83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-04-01-primary-sports-day-rehearsal-3</t>
+          <t xml:space="preserve">2027-03-31-secondary-sports-day-rehearsal-3</t>
         </is>
       </c>
       <c r="B83" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-04-01</t>
+          <t xml:space="preserve">2027-03-31</t>
         </is>
       </c>
       <c r="C83" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-04-01</t>
+          <t xml:space="preserve">2027-03-31</t>
         </is>
       </c>
       <c r="D83" t="inlineStr" s="3">
@@ -8056,7 +8056,7 @@
       </c>
       <c r="E83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary</t>
+          <t xml:space="preserve">Secondary</t>
         </is>
       </c>
       <c r="F83" t="inlineStr" s="2">
@@ -8076,22 +8076,22 @@
       </c>
       <c r="I83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary Sports Day Rehearsal #3</t>
+          <t xml:space="preserve">Secondary Sports Day Rehearsal #3</t>
         </is>
       </c>
       <c r="J83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">小学部運動会リハーサル #3</t>
+          <t xml:space="preserve">中等部運動会リハーサル #3</t>
         </is>
       </c>
       <c r="K83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">The final rehearsal provides students with an opportunity to practice events and ensure they are ready for Sports Day.</t>
+          <t xml:space="preserve">Secondary students will prepare for Sports Day by practicing event routines, team organization, and activity expectations.</t>
         </is>
       </c>
       <c r="L83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">最終リハーサルで各種目を練習し、運動会当日に向けて準備を整えます。</t>
+          <t xml:space="preserve">中等部の生徒が、種目の流れ、チーム編成、活動のルールを練習し、運動会に向けて準備します。</t>
         </is>
       </c>
       <c r="M83" t="inlineStr" s="2">
@@ -8106,7 +8106,7 @@
       </c>
       <c r="O83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-04-01-primary-sports-day-rehearsal-3.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-03-31-secondary-sports-day-rehearsal-3.webp</t>
         </is>
       </c>
       <c r="P83" t="inlineStr" s="2">
@@ -8133,17 +8133,17 @@
     <row r="84">
       <c r="A84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-04-03-sports-day</t>
+          <t xml:space="preserve">2027-04-01-primary-sports-day-rehearsal-3</t>
         </is>
       </c>
       <c r="B84" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-04-03</t>
+          <t xml:space="preserve">2027-04-01</t>
         </is>
       </c>
       <c r="C84" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-04-03</t>
+          <t xml:space="preserve">2027-04-01</t>
         </is>
       </c>
       <c r="D84" t="inlineStr" s="3">
@@ -8153,12 +8153,12 @@
       </c>
       <c r="E84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary</t>
+          <t xml:space="preserve">Primary</t>
         </is>
       </c>
       <c r="F84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G84" t="inlineStr" s="2">
@@ -8173,22 +8173,22 @@
       </c>
       <c r="I84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sports Day</t>
+          <t xml:space="preserve">Primary Sports Day Rehearsal #3</t>
         </is>
       </c>
       <c r="J84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">運動会</t>
+          <t xml:space="preserve">小学部運動会リハーサル #3</t>
         </is>
       </c>
       <c r="K84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students will take part in Sports Day activities, participating in team games, athletic challenges, and school spirit events.</t>
+          <t xml:space="preserve">The final rehearsal provides students with an opportunity to practice events and ensure they are ready for Sports Day.</t>
         </is>
       </c>
       <c r="L84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">運動会に参加し、チームゲーム、運動競技、応援などの行事に取り組みます。</t>
+          <t xml:space="preserve">最終リハーサルで各種目を練習し、運動会当日に向けて準備を整えます。</t>
         </is>
       </c>
       <c r="M84" t="inlineStr" s="2">
@@ -8203,7 +8203,7 @@
       </c>
       <c r="O84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-04-03-sports-day.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-04-01-primary-sports-day-rehearsal-3.webp</t>
         </is>
       </c>
       <c r="P84" t="inlineStr" s="2">
@@ -8230,7 +8230,7 @@
     <row r="85">
       <c r="A85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-04-03-primary-sports-day-2027</t>
+          <t xml:space="preserve">2027-04-03-sports-day</t>
         </is>
       </c>
       <c r="B85" t="inlineStr" s="3">
@@ -8250,7 +8250,7 @@
       </c>
       <c r="E85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary</t>
+          <t xml:space="preserve">Secondary</t>
         </is>
       </c>
       <c r="F85" t="inlineStr" s="2">
@@ -8270,22 +8270,22 @@
       </c>
       <c r="I85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary Sports Day 2027</t>
+          <t xml:space="preserve">Sports Day</t>
         </is>
       </c>
       <c r="J85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">小学部運動会 2027</t>
+          <t xml:space="preserve">運動会</t>
         </is>
       </c>
       <c r="K85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students participate in a day of fun, fitness, and friendly competition while demonstrating teamwork, perseverance, and sportsmanship.</t>
+          <t xml:space="preserve">Students will take part in Sports Day activities, participating in team games, athletic challenges, and school spirit events.</t>
         </is>
       </c>
       <c r="L85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">チームワーク、粘り強さ、スポーツマンシップを発揮しながら、楽しく体を動かし、仲間と競い合う一日を過ごします。</t>
+          <t xml:space="preserve">運動会に参加し、チームゲーム、運動競技、応援などの行事に取り組みます。</t>
         </is>
       </c>
       <c r="M85" t="inlineStr" s="2">
@@ -8300,7 +8300,7 @@
       </c>
       <c r="O85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-04-03-primary-sports-day-2027.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-04-03-sports-day.webp</t>
         </is>
       </c>
       <c r="P85" t="inlineStr" s="2">
@@ -8327,17 +8327,17 @@
     <row r="86">
       <c r="A86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-04-15-world-art-day</t>
+          <t xml:space="preserve">2027-04-03-primary-sports-day-2027</t>
         </is>
       </c>
       <c r="B86" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-04-15</t>
+          <t xml:space="preserve">2027-04-03</t>
         </is>
       </c>
       <c r="C86" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-04-15</t>
+          <t xml:space="preserve">2027-04-03</t>
         </is>
       </c>
       <c r="D86" t="inlineStr" s="3">
@@ -8347,7 +8347,7 @@
       </c>
       <c r="E86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary, ELC</t>
+          <t xml:space="preserve">Primary</t>
         </is>
       </c>
       <c r="F86" t="inlineStr" s="2">
@@ -8367,22 +8367,22 @@
       </c>
       <c r="I86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">World Art Day</t>
+          <t xml:space="preserve">Primary Sports Day 2027</t>
         </is>
       </c>
       <c r="J86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ワールド・アート・デー</t>
+          <t xml:space="preserve">小学部運動会 2027</t>
         </is>
       </c>
       <c r="K86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students celebrate creativity through art activities, exhibitions, and opportunities to explore different artistic styles and cultures.</t>
+          <t xml:space="preserve">Students participate in a day of fun, fitness, and friendly competition while demonstrating teamwork, perseverance, and sportsmanship.</t>
         </is>
       </c>
       <c r="L86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">アート活動や展示を通して創造性を祝い、さまざまな芸術様式や文化に触れます。</t>
+          <t xml:space="preserve">チームワーク、粘り強さ、スポーツマンシップを発揮しながら、楽しく体を動かし、仲間と競い合う一日を過ごします。</t>
         </is>
       </c>
       <c r="M86" t="inlineStr" s="2">
@@ -8397,7 +8397,7 @@
       </c>
       <c r="O86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-04-15-world-art-day.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-04-03-primary-sports-day-2027.webp</t>
         </is>
       </c>
       <c r="P86" t="inlineStr" s="2">
@@ -8424,17 +8424,17 @@
     <row r="87">
       <c r="A87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-04-16-foundation-field-trip</t>
+          <t xml:space="preserve">2027-04-15-world-art-day</t>
         </is>
       </c>
       <c r="B87" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-04-16</t>
+          <t xml:space="preserve">2027-04-15</t>
         </is>
       </c>
       <c r="C87" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-04-16</t>
+          <t xml:space="preserve">2027-04-15</t>
         </is>
       </c>
       <c r="D87" t="inlineStr" s="3">
@@ -8444,7 +8444,7 @@
       </c>
       <c r="E87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary</t>
+          <t xml:space="preserve">Primary, ELC</t>
         </is>
       </c>
       <c r="F87" t="inlineStr" s="2">
@@ -8464,22 +8464,22 @@
       </c>
       <c r="I87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Foundation Field Trip</t>
+          <t xml:space="preserve">World Art Day</t>
         </is>
       </c>
       <c r="J87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ファウンデーション校外学習</t>
+          <t xml:space="preserve">ワールド・アート・デー</t>
         </is>
       </c>
       <c r="K87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Our youngest learners will enjoy an age-appropriate educational excursion that supports classroom learning through hands-on experiences.</t>
+          <t xml:space="preserve">Students celebrate creativity through art activities, exhibitions, and opportunities to explore different artistic styles and cultures.</t>
         </is>
       </c>
       <c r="L87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">年少の子どもたちが、年齢に合った校外学習に出かけ、体験を通して教室での学びを深めます。</t>
+          <t xml:space="preserve">アート活動や展示を通して創造性を祝い、さまざまな芸術様式や文化に触れます。</t>
         </is>
       </c>
       <c r="M87" t="inlineStr" s="2">
@@ -8494,7 +8494,7 @@
       </c>
       <c r="O87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-04-16-foundation-field-trip.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-04-15-world-art-day.webp</t>
         </is>
       </c>
       <c r="P87" t="inlineStr" s="2">
@@ -8521,17 +8521,17 @@
     <row r="88">
       <c r="A88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-04-21-hackathon-hour-of-code</t>
+          <t xml:space="preserve">2027-04-16-foundation-field-trip</t>
         </is>
       </c>
       <c r="B88" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-04-21</t>
+          <t xml:space="preserve">2027-04-16</t>
         </is>
       </c>
       <c r="C88" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-04-21</t>
+          <t xml:space="preserve">2027-04-16</t>
         </is>
       </c>
       <c r="D88" t="inlineStr" s="3">
@@ -8541,12 +8541,12 @@
       </c>
       <c r="E88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary</t>
+          <t xml:space="preserve">Primary</t>
         </is>
       </c>
       <c r="F88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="G88" t="inlineStr" s="2">
@@ -8561,22 +8561,22 @@
       </c>
       <c r="I88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Hackathon (Hour of Code)</t>
+          <t xml:space="preserve">Foundation Field Trip</t>
         </is>
       </c>
       <c r="J88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ハッカソン（Hour of Code）</t>
+          <t xml:space="preserve">ファウンデーション校外学習</t>
         </is>
       </c>
       <c r="K88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students will take part in an engaging Hour of Code challenge, using creativity and problem-solving skills to build simple coding projects. This event encourages computational thinking, teamwork, and confidence in technology in a fun and supportive environment.</t>
+          <t xml:space="preserve">Our youngest learners will enjoy an age-appropriate educational excursion that supports classroom learning through hands-on experiences.</t>
         </is>
       </c>
       <c r="L88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Hour of Codeチャレンジに参加し、創造性と問題解決力を生かして簡単なプログラミング作品を作ります。楽しく支え合う環境の中で、コンピュテーショナル・シンキング、チームワーク、テクノロジーへの自信を育みます。</t>
+          <t xml:space="preserve">年少の子どもたちが、年齢に合った校外学習に出かけ、体験を通して教室での学びを深めます。</t>
         </is>
       </c>
       <c r="M88" t="inlineStr" s="2">
@@ -8591,7 +8591,7 @@
       </c>
       <c r="O88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-04-21-hackathon-hour-of-code.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-04-16-foundation-field-trip.webp</t>
         </is>
       </c>
       <c r="P88" t="inlineStr" s="2">
@@ -8618,17 +8618,17 @@
     <row r="89">
       <c r="A89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-04-22-biology-ia-prep-field-trip-shore-ecosystem</t>
+          <t xml:space="preserve">2027-04-21-hackathon-hour-of-code</t>
         </is>
       </c>
       <c r="B89" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-04-22</t>
+          <t xml:space="preserve">2027-04-21</t>
         </is>
       </c>
       <c r="C89" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-04-22</t>
+          <t xml:space="preserve">2027-04-21</t>
         </is>
       </c>
       <c r="D89" t="inlineStr" s="3">
@@ -8638,7 +8638,7 @@
       </c>
       <c r="E89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">High School</t>
+          <t xml:space="preserve">Secondary</t>
         </is>
       </c>
       <c r="F89" t="inlineStr" s="2">
@@ -8658,22 +8658,22 @@
       </c>
       <c r="I89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Biology IA Prep. Field Trip: Shore Ecosystem</t>
+          <t xml:space="preserve">Hackathon (Hour of Code)</t>
         </is>
       </c>
       <c r="J89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">生物IA準備校外学習：海岸生態系調査</t>
+          <t xml:space="preserve">ハッカソン（Hour of Code）</t>
         </is>
       </c>
       <c r="K89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Grade 11 and 12 Biology students will visit a shore ecosystem to prepare for their Biology Internal Assessment by collecting fieldwork data and practicing research methods.</t>
+          <t xml:space="preserve">Students will take part in an engaging Hour of Code challenge, using creativity and problem-solving skills to build simple coding projects. This event encourages computational thinking, teamwork, and confidence in technology in a fun and supportive environment.</t>
         </is>
       </c>
       <c r="L89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">11・12年生の生物履修者が海岸の生態系を訪れ、フィールドワークでのデータ収集や研究手法の練習を通して、生物の内部評価（IA）に向けた準備を行います。</t>
+          <t xml:space="preserve">Hour of Codeチャレンジに参加し、創造性と問題解決力を生かして簡単なプログラミング作品を作ります。楽しく支え合う環境の中で、コンピュテーショナル・シンキング、チームワーク、テクノロジーへの自信を育みます。</t>
         </is>
       </c>
       <c r="M89" t="inlineStr" s="2">
@@ -8688,7 +8688,7 @@
       </c>
       <c r="O89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-04-22-biology-ia-prep-field-trip-shore-ecosystem.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-04-21-hackathon-hour-of-code.webp</t>
         </is>
       </c>
       <c r="P89" t="inlineStr" s="2">
@@ -8715,17 +8715,17 @@
     <row r="90">
       <c r="A90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-04-23-g12-celebration</t>
+          <t xml:space="preserve">2027-04-22-biology-ia-prep-field-trip-shore-ecosystem</t>
         </is>
       </c>
       <c r="B90" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-04-23</t>
+          <t xml:space="preserve">2027-04-22</t>
         </is>
       </c>
       <c r="C90" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-04-23</t>
+          <t xml:space="preserve">2027-04-22</t>
         </is>
       </c>
       <c r="D90" t="inlineStr" s="3">
@@ -8755,22 +8755,22 @@
       </c>
       <c r="I90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">G12 Celebration</t>
+          <t xml:space="preserve">Biology IA Prep. Field Trip: Shore Ecosystem</t>
         </is>
       </c>
       <c r="J90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">G12修了記念イベント</t>
+          <t xml:space="preserve">生物IA準備校外学習：海岸生態系調査</t>
         </is>
       </c>
       <c r="K90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Grade 12 students will take part in a Graduation Walk as the school community celebrates them ahead of graduation.</t>
+          <t xml:space="preserve">Grade 11 and 12 Biology students will visit a shore ecosystem to prepare for their Biology Internal Assessment by collecting fieldwork data and practicing research methods.</t>
         </is>
       </c>
       <c r="L90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">卒業を前に、12年生がグラデュエーション・ウォークに参加し、学校コミュニティ全体でお祝いします。</t>
+          <t xml:space="preserve">11・12年生の生物履修者が海岸の生態系を訪れ、フィールドワークでのデータ収集や研究手法の練習を通して、生物の内部評価（IA）に向けた準備を行います。</t>
         </is>
       </c>
       <c r="M90" t="inlineStr" s="2">
@@ -8785,7 +8785,7 @@
       </c>
       <c r="O90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-04-23-g12-celebration.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-04-22-biology-ia-prep-field-trip-shore-ecosystem.webp</t>
         </is>
       </c>
       <c r="P90" t="inlineStr" s="2">
@@ -8812,17 +8812,17 @@
     <row r="91">
       <c r="A91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-04-26-grade-4-5-camping-trip</t>
+          <t xml:space="preserve">2027-04-23-g12-celebration</t>
         </is>
       </c>
       <c r="B91" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-04-26</t>
+          <t xml:space="preserve">2027-04-23</t>
         </is>
       </c>
       <c r="C91" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-04-27</t>
+          <t xml:space="preserve">2027-04-23</t>
         </is>
       </c>
       <c r="D91" t="inlineStr" s="3">
@@ -8832,7 +8832,7 @@
       </c>
       <c r="E91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary</t>
+          <t xml:space="preserve">High School</t>
         </is>
       </c>
       <c r="F91" t="inlineStr" s="2">
@@ -8852,22 +8852,22 @@
       </c>
       <c r="I91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Grade 4, 5 Camping Trip</t>
+          <t xml:space="preserve">G12 Celebration</t>
         </is>
       </c>
       <c r="J91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">4・5年生キャンプ</t>
+          <t xml:space="preserve">G12修了記念イベント</t>
         </is>
       </c>
       <c r="K91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students enjoy an outdoor learning experience that promotes independence, teamwork, resilience, and a connection with nature.</t>
+          <t xml:space="preserve">Grade 12 students will take part in a Graduation Walk as the school community celebrates them ahead of graduation.</t>
         </is>
       </c>
       <c r="L91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">自立心、チームワーク、たくましさ、自然とのつながりを育む野外学習を楽しみます。</t>
+          <t xml:space="preserve">卒業を前に、12年生がグラデュエーション・ウォークに参加し、学校コミュニティ全体でお祝いします。</t>
         </is>
       </c>
       <c r="M91" t="inlineStr" s="2">
@@ -8882,7 +8882,7 @@
       </c>
       <c r="O91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-04-26-grade-4-5-camping-trip.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-04-23-g12-celebration.webp</t>
         </is>
       </c>
       <c r="P91" t="inlineStr" s="2">
@@ -8909,19 +8909,19 @@
     <row r="92">
       <c r="A92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-04-27-choir-and-orchestra-concert</t>
+          <t xml:space="preserve">2027-04-26-grade-4-5-camping-trip</t>
         </is>
       </c>
       <c r="B92" t="inlineStr" s="3">
         <is>
+          <t xml:space="preserve">2027-04-26</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr" s="3">
+        <is>
           <t xml:space="preserve">2027-04-27</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">2027-04-27</t>
-        </is>
-      </c>
       <c r="D92" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
@@ -8929,12 +8929,12 @@
       </c>
       <c r="E92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary</t>
+          <t xml:space="preserve">Primary</t>
         </is>
       </c>
       <c r="F92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G92" t="inlineStr" s="2">
@@ -8949,22 +8949,22 @@
       </c>
       <c r="I92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Choir and Orchestra Concert</t>
+          <t xml:space="preserve">Grade 4, 5 Camping Trip</t>
         </is>
       </c>
       <c r="J92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">合唱・オーケストラコンサート</t>
+          <t xml:space="preserve">4・5年生キャンプ</t>
         </is>
       </c>
       <c r="K92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Choir class and orchestra club will perform the music repertoire they have been rehearsing for an audience of family, peers and teachers.</t>
+          <t xml:space="preserve">Students enjoy an outdoor learning experience that promotes independence, teamwork, resilience, and a connection with nature.</t>
         </is>
       </c>
       <c r="L92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">合唱クラスとオーケストラクラブが、練習を重ねてきた曲目をご家族、友人、教員の前で演奏します。</t>
+          <t xml:space="preserve">自立心、チームワーク、たくましさ、自然とのつながりを育む野外学習を楽しみます。</t>
         </is>
       </c>
       <c r="M92" t="inlineStr" s="2">
@@ -8979,7 +8979,7 @@
       </c>
       <c r="O92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-04-27-choir-and-orchestra-concert.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-04-26-grade-4-5-camping-trip.webp</t>
         </is>
       </c>
       <c r="P92" t="inlineStr" s="2">
@@ -9006,17 +9006,17 @@
     <row r="93">
       <c r="A93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-04-30-science-fair</t>
+          <t xml:space="preserve">2027-04-27-choir-and-orchestra-concert</t>
         </is>
       </c>
       <c r="B93" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-04-30</t>
+          <t xml:space="preserve">2027-04-27</t>
         </is>
       </c>
       <c r="C93" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-04-30</t>
+          <t xml:space="preserve">2027-04-27</t>
         </is>
       </c>
       <c r="D93" t="inlineStr" s="3">
@@ -9046,22 +9046,22 @@
       </c>
       <c r="I93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Science Fair</t>
+          <t xml:space="preserve">Choir and Orchestra Concert</t>
         </is>
       </c>
       <c r="J93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">サイエンスフェア</t>
+          <t xml:space="preserve">合唱・オーケストラコンサート</t>
         </is>
       </c>
       <c r="K93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students will share their science projects and investigations with the school community, showcasing their research, creativity, and scientific thinking.</t>
+          <t xml:space="preserve">Choir class and orchestra club will perform the music repertoire they have been rehearsing for an audience of family, peers and teachers.</t>
         </is>
       </c>
       <c r="L93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">理科のプロジェクトや探究の成果を学校コミュニティに発表し、研究、創造性、科学的思考を披露します。</t>
+          <t xml:space="preserve">合唱クラスとオーケストラクラブが、練習を重ねてきた曲目をご家族、友人、教員の前で演奏します。</t>
         </is>
       </c>
       <c r="M93" t="inlineStr" s="2">
@@ -9076,7 +9076,7 @@
       </c>
       <c r="O93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-04-30-science-fair.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-04-27-choir-and-orchestra-concert.webp</t>
         </is>
       </c>
       <c r="P93" t="inlineStr" s="2">
@@ -9103,17 +9103,17 @@
     <row r="94">
       <c r="A94" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-05-17-friendly-basketball-tournament-internal</t>
+          <t xml:space="preserve">2027-04-30-science-fair</t>
         </is>
       </c>
       <c r="B94" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-05-17</t>
+          <t xml:space="preserve">2027-04-30</t>
         </is>
       </c>
       <c r="C94" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-05-21</t>
+          <t xml:space="preserve">2027-04-30</t>
         </is>
       </c>
       <c r="D94" t="inlineStr" s="3">
@@ -9128,7 +9128,7 @@
       </c>
       <c r="F94" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="G94" t="inlineStr" s="2">
@@ -9143,22 +9143,22 @@
       </c>
       <c r="I94" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Friendly Basketball Tournament (Internal)</t>
+          <t xml:space="preserve">Science Fair</t>
         </is>
       </c>
       <c r="J94" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">校内バスケットボール大会</t>
+          <t xml:space="preserve">サイエンスフェア</t>
         </is>
       </c>
       <c r="K94" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students will take part in a friendly internal basketball tournament, promoting teamwork, sportsmanship, and school spirit.</t>
+          <t xml:space="preserve">Students will share their science projects and investigations with the school community, showcasing their research, creativity, and scientific thinking.</t>
         </is>
       </c>
       <c r="L94" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">校内バスケットボール大会に参加し、チームワーク、スポーツマンシップ、愛校心を育みます。</t>
+          <t xml:space="preserve">理科のプロジェクトや探究の成果を学校コミュニティに発表し、研究、創造性、科学的思考を披露します。</t>
         </is>
       </c>
       <c r="M94" t="inlineStr" s="2">
@@ -9173,7 +9173,7 @@
       </c>
       <c r="O94" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-05-17-friendly-basketball-tournament-internal.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-04-30-science-fair.webp</t>
         </is>
       </c>
       <c r="P94" t="inlineStr" s="2">
@@ -9200,17 +9200,17 @@
     <row r="95">
       <c r="A95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-05-19-entrepreneurs-day</t>
+          <t xml:space="preserve">2027-05-17-friendly-basketball-tournament-internal</t>
         </is>
       </c>
       <c r="B95" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-05-19</t>
+          <t xml:space="preserve">2027-05-17</t>
         </is>
       </c>
       <c r="C95" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-05-20</t>
+          <t xml:space="preserve">2027-05-21</t>
         </is>
       </c>
       <c r="D95" t="inlineStr" s="3">
@@ -9220,12 +9220,12 @@
       </c>
       <c r="E95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary, ELC</t>
+          <t xml:space="preserve">Secondary</t>
         </is>
       </c>
       <c r="F95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G95" t="inlineStr" s="2">
@@ -9240,22 +9240,22 @@
       </c>
       <c r="I95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Entrepreneurs Day</t>
+          <t xml:space="preserve">Friendly Basketball Tournament (Internal)</t>
         </is>
       </c>
       <c r="J95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">アントレプレナーシップ・デー</t>
+          <t xml:space="preserve">校内バスケットボール大会</t>
         </is>
       </c>
       <c r="K95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students develop and showcase business ideas while learning about creativity, financial literacy, problem-solving, and entrepreneurship.</t>
+          <t xml:space="preserve">Students will take part in a friendly internal basketball tournament, promoting teamwork, sportsmanship, and school spirit.</t>
         </is>
       </c>
       <c r="L95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">創造性、金融リテラシー、問題解決、起業家精神について学びながら、ビジネスのアイデアを考え、発表します。</t>
+          <t xml:space="preserve">校内バスケットボール大会に参加し、チームワーク、スポーツマンシップ、愛校心を育みます。</t>
         </is>
       </c>
       <c r="M95" t="inlineStr" s="2">
@@ -9270,7 +9270,7 @@
       </c>
       <c r="O95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-05-19-entrepreneurs-day.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-05-17-friendly-basketball-tournament-internal.webp</t>
         </is>
       </c>
       <c r="P95" t="inlineStr" s="2">
@@ -9297,17 +9297,17 @@
     <row r="96">
       <c r="A96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-05-21-collective-field-trip</t>
+          <t xml:space="preserve">2027-05-19-entrepreneurs-day</t>
         </is>
       </c>
       <c r="B96" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-05-21</t>
+          <t xml:space="preserve">2027-05-19</t>
         </is>
       </c>
       <c r="C96" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-05-21</t>
+          <t xml:space="preserve">2027-05-20</t>
         </is>
       </c>
       <c r="D96" t="inlineStr" s="3">
@@ -9322,7 +9322,7 @@
       </c>
       <c r="F96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="G96" t="inlineStr" s="2">
@@ -9337,22 +9337,22 @@
       </c>
       <c r="I96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Collective Field Trip</t>
+          <t xml:space="preserve">Entrepreneurs Day</t>
         </is>
       </c>
       <c r="J96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">合同校外学習</t>
+          <t xml:space="preserve">アントレプレナーシップ・デー</t>
         </is>
       </c>
       <c r="K96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students participate in a shared educational experience that promotes collaboration, inquiry, and real-world learning.</t>
+          <t xml:space="preserve">Students develop and showcase business ideas while learning about creativity, financial literacy, problem-solving, and entrepreneurship.</t>
         </is>
       </c>
       <c r="L96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">協働、探究、実社会での学びを促す合同の学習体験に参加します。</t>
+          <t xml:space="preserve">創造性、金融リテラシー、問題解決、起業家精神について学びながら、ビジネスのアイデアを考え、発表します。</t>
         </is>
       </c>
       <c r="M96" t="inlineStr" s="2">
@@ -9367,7 +9367,7 @@
       </c>
       <c r="O96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-05-21-collective-field-trip.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-05-19-entrepreneurs-day.webp</t>
         </is>
       </c>
       <c r="P96" t="inlineStr" s="2">
@@ -9394,17 +9394,17 @@
     <row r="97">
       <c r="A97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-05-22-saturday-school-last-day-event</t>
+          <t xml:space="preserve">2027-05-21-collective-field-trip</t>
         </is>
       </c>
       <c r="B97" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-05-22</t>
+          <t xml:space="preserve">2027-05-21</t>
         </is>
       </c>
       <c r="C97" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-05-22</t>
+          <t xml:space="preserve">2027-05-21</t>
         </is>
       </c>
       <c r="D97" t="inlineStr" s="3">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="E97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary</t>
+          <t xml:space="preserve">Primary, ELC</t>
         </is>
       </c>
       <c r="F97" t="inlineStr" s="2">
@@ -9434,22 +9434,22 @@
       </c>
       <c r="I97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Saturday School Last Day Event</t>
+          <t xml:space="preserve">Collective Field Trip</t>
         </is>
       </c>
       <c r="J97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">土曜校最終日イベント</t>
+          <t xml:space="preserve">合同校外学習</t>
         </is>
       </c>
       <c r="K97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students will take part in a relaxed final Saturday School session, with leisure activities at school to celebrate the last day.</t>
+          <t xml:space="preserve">Students participate in a shared educational experience that promotes collaboration, inquiry, and real-world learning.</t>
         </is>
       </c>
       <c r="L97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">土曜校の最終日を、校内でのレクリエーション活動とともにリラックスして過ごし、お祝いします。</t>
+          <t xml:space="preserve">協働、探究、実社会での学びを促す合同の学習体験に参加します。</t>
         </is>
       </c>
       <c r="M97" t="inlineStr" s="2">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="O97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-05-22-saturday-school-last-day-event.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-05-21-collective-field-trip.webp</t>
         </is>
       </c>
       <c r="P97" t="inlineStr" s="2">
@@ -9491,17 +9491,17 @@
     <row r="98">
       <c r="A98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-05-24-concept-con-future-focus</t>
+          <t xml:space="preserve">2027-05-22-saturday-school-last-day-event</t>
         </is>
       </c>
       <c r="B98" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-05-24</t>
+          <t xml:space="preserve">2027-05-22</t>
         </is>
       </c>
       <c r="C98" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-05-28</t>
+          <t xml:space="preserve">2027-05-22</t>
         </is>
       </c>
       <c r="D98" t="inlineStr" s="3">
@@ -9511,7 +9511,7 @@
       </c>
       <c r="E98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary, ELC</t>
+          <t xml:space="preserve">Secondary</t>
         </is>
       </c>
       <c r="F98" t="inlineStr" s="2">
@@ -9531,22 +9531,22 @@
       </c>
       <c r="I98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Concept Con (Future Focus)</t>
+          <t xml:space="preserve">Saturday School Last Day Event</t>
         </is>
       </c>
       <c r="J98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">コンセプト・コン（未来を考える）</t>
+          <t xml:space="preserve">土曜校最終日イベント</t>
         </is>
       </c>
       <c r="K98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students investigate future possibilities, innovations, and solutions to real-world challenges through inquiry-based projects and presentations.</t>
+          <t xml:space="preserve">Students will take part in a relaxed final Saturday School session, with leisure activities at school to celebrate the last day.</t>
         </is>
       </c>
       <c r="L98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">探究型のプロジェクトや発表を通して、未来の可能性、イノベーション、現実の課題の解決策について考えます。</t>
+          <t xml:space="preserve">土曜校の最終日を、校内でのレクリエーション活動とともにリラックスして過ごし、お祝いします。</t>
         </is>
       </c>
       <c r="M98" t="inlineStr" s="2">
@@ -9561,7 +9561,7 @@
       </c>
       <c r="O98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-05-24-concept-con-future-focus.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-05-22-saturday-school-last-day-event.webp</t>
         </is>
       </c>
       <c r="P98" t="inlineStr" s="2">
@@ -9588,17 +9588,17 @@
     <row r="99">
       <c r="A99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-05-28-g12-graduation-with-performances</t>
+          <t xml:space="preserve">2027-05-24-concept-con-future-focus</t>
         </is>
       </c>
       <c r="B99" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-05-29</t>
+          <t xml:space="preserve">2027-05-24</t>
         </is>
       </c>
       <c r="C99" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-05-29</t>
+          <t xml:space="preserve">2027-05-28</t>
         </is>
       </c>
       <c r="D99" t="inlineStr" s="3">
@@ -9608,12 +9608,12 @@
       </c>
       <c r="E99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">High School</t>
+          <t xml:space="preserve">Primary, ELC</t>
         </is>
       </c>
       <c r="F99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G99" t="inlineStr" s="2">
@@ -9623,27 +9623,27 @@
       </c>
       <c r="H99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">changed</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">G12 Graduation with Performances</t>
+          <t xml:space="preserve">Concept Con (Future Focus)</t>
         </is>
       </c>
       <c r="J99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">G12卒業式・記念パフォーマンス</t>
+          <t xml:space="preserve">コンセプト・コン（未来を考える）</t>
         </is>
       </c>
       <c r="K99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Grade 12 students will celebrate their graduation with a formal ceremony featuring student performances and the wider school community.</t>
+          <t xml:space="preserve">Students investigate future possibilities, innovations, and solutions to real-world challenges through inquiry-based projects and presentations.</t>
         </is>
       </c>
       <c r="L99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">12年生が、生徒によるパフォーマンスを交えた式典で、学校コミュニティ全体とともに卒業を祝います。</t>
+          <t xml:space="preserve">探究型のプロジェクトや発表を通して、未来の可能性、イノベーション、現実の課題の解決策について考えます。</t>
         </is>
       </c>
       <c r="M99" t="inlineStr" s="2">
@@ -9658,7 +9658,7 @@
       </c>
       <c r="O99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-05-28-g12-graduation-with-performances.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-05-24-concept-con-future-focus.webp</t>
         </is>
       </c>
       <c r="P99" t="inlineStr" s="2">
@@ -9685,17 +9685,17 @@
     <row r="100">
       <c r="A100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-06-03-celebration-of-learning-prep</t>
+          <t xml:space="preserve">2027-05-28-g12-graduation-with-performances</t>
         </is>
       </c>
       <c r="B100" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-06-03</t>
+          <t xml:space="preserve">2027-05-29</t>
         </is>
       </c>
       <c r="C100" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-06-03</t>
+          <t xml:space="preserve">2027-05-29</t>
         </is>
       </c>
       <c r="D100" t="inlineStr" s="3">
@@ -9705,12 +9705,12 @@
       </c>
       <c r="E100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Whole School</t>
+          <t xml:space="preserve">High School</t>
         </is>
       </c>
       <c r="F100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="G100" t="inlineStr" s="2">
@@ -9720,27 +9720,27 @@
       </c>
       <c r="H100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">changed</t>
         </is>
       </c>
       <c r="I100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Celebration of Learning Prep</t>
+          <t xml:space="preserve">G12 Graduation with Performances</t>
         </is>
       </c>
       <c r="J100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">学びの発表会準備</t>
+          <t xml:space="preserve">G12卒業式・記念パフォーマンス</t>
         </is>
       </c>
       <c r="K100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students help prepare the school for the Celebration of Learning by organizing learning spaces, setting up displays, arranging materials, and ensuring classrooms and common areas are ready to welcome visitors. This preparation helps create an engaging and welcoming environment for families and guests.</t>
+          <t xml:space="preserve">Grade 12 students will celebrate their graduation with a formal ceremony featuring student performances and the wider school community.</t>
         </is>
       </c>
       <c r="L100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">学びの発表会に向けて、学習スペースの整理、展示の設営、資料の準備を行い、教室や共用エリアで来場者をお迎えできるよう整えます。ご家族やお客様にとって魅力的で温かな空間づくりにつながります。</t>
+          <t xml:space="preserve">12年生が、生徒によるパフォーマンスを交えた式典で、学校コミュニティ全体とともに卒業を祝います。</t>
         </is>
       </c>
       <c r="M100" t="inlineStr" s="2">
@@ -9755,7 +9755,7 @@
       </c>
       <c r="O100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-06-03-celebration-of-learning-prep.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-05-28-g12-graduation-with-performances.webp</t>
         </is>
       </c>
       <c r="P100" t="inlineStr" s="2">
@@ -9782,7 +9782,7 @@
     <row r="101">
       <c r="A101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-06-03-ukulele-concert</t>
+          <t xml:space="preserve">2027-06-03-celebration-of-learning-prep</t>
         </is>
       </c>
       <c r="B101" t="inlineStr" s="3">
@@ -9792,7 +9792,7 @@
       </c>
       <c r="C101" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-06-04</t>
+          <t xml:space="preserve">2027-06-03</t>
         </is>
       </c>
       <c r="D101" t="inlineStr" s="3">
@@ -9802,12 +9802,12 @@
       </c>
       <c r="E101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary</t>
+          <t xml:space="preserve">Whole School</t>
         </is>
       </c>
       <c r="F101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G101" t="inlineStr" s="2">
@@ -9822,22 +9822,22 @@
       </c>
       <c r="I101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ukulele Concert</t>
+          <t xml:space="preserve">Celebration of Learning Prep</t>
         </is>
       </c>
       <c r="J101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ウクレレコンサート</t>
+          <t xml:space="preserve">学びの発表会準備</t>
         </is>
       </c>
       <c r="K101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students perform musical pieces they have learned throughout the year, demonstrating their growth, confidence, and musical skills.</t>
+          <t xml:space="preserve">Students help prepare the school for the Celebration of Learning by organizing learning spaces, setting up displays, arranging materials, and ensuring classrooms and common areas are ready to welcome visitors. This preparation helps create an engaging and welcoming environment for families and guests.</t>
         </is>
       </c>
       <c r="L101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">一年を通して学んだ曲を演奏し、成長、自信、音楽の技能を披露します。</t>
+          <t xml:space="preserve">学びの発表会に向けて、学習スペースの整理、展示の設営、資料の準備を行い、教室や共用エリアで来場者をお迎えできるよう整えます。ご家族やお客様にとって魅力的で温かな空間づくりにつながります。</t>
         </is>
       </c>
       <c r="M101" t="inlineStr" s="2">
@@ -9852,7 +9852,7 @@
       </c>
       <c r="O101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-06-03-ukulele-concert.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-06-03-celebration-of-learning-prep.webp</t>
         </is>
       </c>
       <c r="P101" t="inlineStr" s="2">
@@ -9879,19 +9879,19 @@
     <row r="102">
       <c r="A102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-06-04-celebration-of-learning</t>
+          <t xml:space="preserve">2027-06-03-ukulele-concert</t>
         </is>
       </c>
       <c r="B102" t="inlineStr" s="3">
         <is>
+          <t xml:space="preserve">2027-06-03</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr" s="3">
+        <is>
           <t xml:space="preserve">2027-06-04</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve">2027-06-04</t>
-        </is>
-      </c>
       <c r="D102" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve"/>
@@ -9899,7 +9899,7 @@
       </c>
       <c r="E102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Whole School</t>
+          <t xml:space="preserve">Primary</t>
         </is>
       </c>
       <c r="F102" t="inlineStr" s="2">
@@ -9919,22 +9919,22 @@
       </c>
       <c r="I102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Celebration of Learning</t>
+          <t xml:space="preserve">Ukulele Concert</t>
         </is>
       </c>
       <c r="J102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">学びの発表会</t>
+          <t xml:space="preserve">ウクレレコンサート</t>
         </is>
       </c>
       <c r="K102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">The school community will celebrate learning as students share projects and exhibitions, including PYPX, MYPX, CAS, EE, TOK and Foundation to 4 projects.</t>
+          <t xml:space="preserve">Students perform musical pieces they have learned throughout the year, demonstrating their growth, confidence, and musical skills.</t>
         </is>
       </c>
       <c r="L102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PYPX、MYPX、CAS、EE、TOK、ファウンデーション～4年生のプロジェクトなど、生徒の作品や展示を通して学校コミュニティ全体で学びを祝います。</t>
+          <t xml:space="preserve">一年を通して学んだ曲を演奏し、成長、自信、音楽の技能を披露します。</t>
         </is>
       </c>
       <c r="M102" t="inlineStr" s="2">
@@ -9949,7 +9949,7 @@
       </c>
       <c r="O102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-06-04-celebration-of-learning.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-06-03-ukulele-concert.webp</t>
         </is>
       </c>
       <c r="P102" t="inlineStr" s="2">
@@ -9976,17 +9976,17 @@
     <row r="103">
       <c r="A103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-06-05-sat-test-7</t>
+          <t xml:space="preserve">2027-06-04-celebration-of-learning</t>
         </is>
       </c>
       <c r="B103" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-06-05</t>
+          <t xml:space="preserve">2027-06-04</t>
         </is>
       </c>
       <c r="C103" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-06-05</t>
+          <t xml:space="preserve">2027-06-04</t>
         </is>
       </c>
       <c r="D103" t="inlineStr" s="3">
@@ -9996,12 +9996,12 @@
       </c>
       <c r="E103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">High School</t>
+          <t xml:space="preserve">Whole School</t>
         </is>
       </c>
       <c r="F103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="G103" t="inlineStr" s="2">
@@ -10016,22 +10016,22 @@
       </c>
       <c r="I103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SAT Test #7</t>
+          <t xml:space="preserve">Celebration of Learning</t>
         </is>
       </c>
       <c r="J103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SAT試験 第7回</t>
+          <t xml:space="preserve">学びの発表会</t>
         </is>
       </c>
       <c r="K103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">An internationally recognized university entrance exam. Our school is an official SAT test center, and both Enishi students and external students are welcome to take the test on campus.</t>
+          <t xml:space="preserve">The school community will celebrate learning as students share projects and exhibitions, including PYPX, MYPX, CAS, EE, TOK and Foundation to 4 projects.</t>
         </is>
       </c>
       <c r="L103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">国際的に認められた大学入学試験です。本校はSAT公式試験会場であり、本校生徒・外部生徒ともに校内で受験できます。</t>
+          <t xml:space="preserve">PYPX、MYPX、CAS、EE、TOK、ファウンデーション～4年生のプロジェクトなど、生徒の作品や展示を通して学校コミュニティ全体で学びを祝います。</t>
         </is>
       </c>
       <c r="M103" t="inlineStr" s="2">
@@ -10046,7 +10046,7 @@
       </c>
       <c r="O103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-06-05-sat-test-7.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-06-04-celebration-of-learning.webp</t>
         </is>
       </c>
       <c r="P103" t="inlineStr" s="2">
@@ -10073,17 +10073,17 @@
     <row r="104">
       <c r="A104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-06-17-eagle-bucks-store</t>
+          <t xml:space="preserve">2027-06-05-sat-test-7</t>
         </is>
       </c>
       <c r="B104" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-06-17</t>
+          <t xml:space="preserve">2027-06-05</t>
         </is>
       </c>
       <c r="C104" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-06-17</t>
+          <t xml:space="preserve">2027-06-05</t>
         </is>
       </c>
       <c r="D104" t="inlineStr" s="3">
@@ -10093,7 +10093,7 @@
       </c>
       <c r="E104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary, ELC</t>
+          <t xml:space="preserve">High School</t>
         </is>
       </c>
       <c r="F104" t="inlineStr" s="2">
@@ -10113,22 +10113,22 @@
       </c>
       <c r="I104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Eagle Bucks Store</t>
+          <t xml:space="preserve">SAT Test #7</t>
         </is>
       </c>
       <c r="J104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">イーグルバックス・ストア</t>
+          <t xml:space="preserve">SAT試験 第7回</t>
         </is>
       </c>
       <c r="K104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students can use their earned Eagle Bucks to purchase rewards and special items. The store reinforces positive behavior, responsibility, and goal-setting.</t>
+          <t xml:space="preserve">An internationally recognized university entrance exam. Our school is an official SAT test center, and both Enishi students and external students are welcome to take the test on campus.</t>
         </is>
       </c>
       <c r="L104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">獲得したイーグルバックスを使って、ごほうびや特別なアイテムと交換できます。前向きな行動、責任感、目標設定を後押しする取り組みです。</t>
+          <t xml:space="preserve">国際的に認められた大学入学試験です。本校はSAT公式試験会場であり、本校生徒・外部生徒ともに校内で受験できます。</t>
         </is>
       </c>
       <c r="M104" t="inlineStr" s="2">
@@ -10143,7 +10143,7 @@
       </c>
       <c r="O104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-06-17-eagle-bucks-store.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-06-05-sat-test-7.webp</t>
         </is>
       </c>
       <c r="P104" t="inlineStr" s="2">
@@ -10170,17 +10170,17 @@
     <row r="105">
       <c r="A105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-06-18-kindergarten-and-grade-5-graduation</t>
+          <t xml:space="preserve">2027-06-17-eagle-bucks-store</t>
         </is>
       </c>
       <c r="B105" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-06-18</t>
+          <t xml:space="preserve">2027-06-17</t>
         </is>
       </c>
       <c r="C105" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-06-18</t>
+          <t xml:space="preserve">2027-06-17</t>
         </is>
       </c>
       <c r="D105" t="inlineStr" s="3">
@@ -10195,7 +10195,7 @@
       </c>
       <c r="F105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G105" t="inlineStr" s="2">
@@ -10210,22 +10210,22 @@
       </c>
       <c r="I105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Kindergarten and Grade 5 Graduation</t>
+          <t xml:space="preserve">Eagle Bucks Store</t>
         </is>
       </c>
       <c r="J105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">幼稚部・5年生卒業式</t>
+          <t xml:space="preserve">イーグルバックス・ストア</t>
         </is>
       </c>
       <c r="K105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students participate in graduation ceremonies to celebrate important milestones in their educational journey. The events recognize student growth, achievements, and readiness for the next stage of learning while bringing together families, staff, and the school community in celebration.</t>
+          <t xml:space="preserve">Students can use their earned Eagle Bucks to purchase rewards and special items. The store reinforces positive behavior, responsibility, and goal-setting.</t>
         </is>
       </c>
       <c r="L105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">学びの歩みにおける大切な節目を祝う卒業式に参加します。生徒の成長と成果、そして次のステージへの準備が整ったことを、ご家族、教職員、学校コミュニティが一堂に会して祝福します。</t>
+          <t xml:space="preserve">獲得したイーグルバックスを使って、ごほうびや特別なアイテムと交換できます。前向きな行動、責任感、目標設定を後押しする取り組みです。</t>
         </is>
       </c>
       <c r="M105" t="inlineStr" s="2">
@@ -10240,7 +10240,7 @@
       </c>
       <c r="O105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-06-18-kindergarten-and-grade-5-graduation.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-06-17-eagle-bucks-store.webp</t>
         </is>
       </c>
       <c r="P105" t="inlineStr" s="2">
@@ -10267,7 +10267,7 @@
     <row r="106">
       <c r="A106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-06-18-primary-elc-year-end-performance</t>
+          <t xml:space="preserve">2027-06-18-kindergarten-and-grade-5-graduation</t>
         </is>
       </c>
       <c r="B106" t="inlineStr" s="3">
@@ -10307,22 +10307,22 @@
       </c>
       <c r="I106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary &amp; ELC Year End Performance</t>
+          <t xml:space="preserve">Kindergarten and Grade 5 Graduation</t>
         </is>
       </c>
       <c r="J106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">小学部・幼稚部年度末発表会</t>
+          <t xml:space="preserve">幼稚部・5年生卒業式</t>
         </is>
       </c>
       <c r="K106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students participate in music, dance, drama, and other performance activities to showcase their learning, creativity, and talents. These performances provide an opportunity to celebrate the school year and share achievements with families and the school community.</t>
+          <t xml:space="preserve">Students participate in graduation ceremonies to celebrate important milestones in their educational journey. The events recognize student growth, achievements, and readiness for the next stage of learning while bringing together families, staff, and the school community in celebration.</t>
         </is>
       </c>
       <c r="L106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">音楽、ダンス、演劇などのパフォーマンスを通して、学び、創造性、才能を披露します。一年の締めくくりを祝い、その成果をご家族や学校コミュニティと分かち合う機会です。</t>
+          <t xml:space="preserve">学びの歩みにおける大切な節目を祝う卒業式に参加します。生徒の成長と成果、そして次のステージへの準備が整ったことを、ご家族、教職員、学校コミュニティが一堂に会して祝福します。</t>
         </is>
       </c>
       <c r="M106" t="inlineStr" s="2">
@@ -10337,7 +10337,7 @@
       </c>
       <c r="O106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-06-18-primary-elc-year-end-performance.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-06-18-kindergarten-and-grade-5-graduation.webp</t>
         </is>
       </c>
       <c r="P106" t="inlineStr" s="2">
@@ -10364,17 +10364,17 @@
     <row r="107">
       <c r="A107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-06-19-end-of-term-3-activity-g6-10</t>
+          <t xml:space="preserve">2027-06-18-primary-elc-year-end-performance</t>
         </is>
       </c>
       <c r="B107" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-06-19</t>
+          <t xml:space="preserve">2027-06-18</t>
         </is>
       </c>
       <c r="C107" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-06-19</t>
+          <t xml:space="preserve">2027-06-18</t>
         </is>
       </c>
       <c r="D107" t="inlineStr" s="3">
@@ -10384,12 +10384,12 @@
       </c>
       <c r="E107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary</t>
+          <t xml:space="preserve">Primary, ELC</t>
         </is>
       </c>
       <c r="F107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="G107" t="inlineStr" s="2">
@@ -10404,22 +10404,22 @@
       </c>
       <c r="I107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">End of Term 3 Activity: G6-10</t>
+          <t xml:space="preserve">Primary &amp; ELC Year End Performance</t>
         </is>
       </c>
       <c r="J107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">第3学期末行事：G6–10</t>
+          <t xml:space="preserve">小学部・幼稚部年度末発表会</t>
         </is>
       </c>
       <c r="K107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Students will take part in an off-campus day trip outside Nagoya to celebrate the end of Term 3.</t>
+          <t xml:space="preserve">Students participate in music, dance, drama, and other performance activities to showcase their learning, creativity, and talents. These performances provide an opportunity to celebrate the school year and share achievements with families and the school community.</t>
         </is>
       </c>
       <c r="L107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">第3学期の終わりを祝い、名古屋近郊への日帰り校外活動に参加します。</t>
+          <t xml:space="preserve">音楽、ダンス、演劇などのパフォーマンスを通して、学び、創造性、才能を披露します。一年の締めくくりを祝い、その成果をご家族や学校コミュニティと分かち合う機会です。</t>
         </is>
       </c>
       <c r="M107" t="inlineStr" s="2">
@@ -10434,7 +10434,7 @@
       </c>
       <c r="O107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-06-19-end-of-term-3-activity-g6-10.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-06-18-primary-elc-year-end-performance.webp</t>
         </is>
       </c>
       <c r="P107" t="inlineStr" s="2">
@@ -10461,17 +10461,17 @@
     <row r="108">
       <c r="A108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-06-22-parent-teacher-conferences</t>
+          <t xml:space="preserve">2027-06-19-end-of-term-3-activity-g6-10</t>
         </is>
       </c>
       <c r="B108" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-06-22</t>
+          <t xml:space="preserve">2027-06-19</t>
         </is>
       </c>
       <c r="C108" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-06-23</t>
+          <t xml:space="preserve">2027-06-19</t>
         </is>
       </c>
       <c r="D108" t="inlineStr" s="3">
@@ -10481,17 +10481,17 @@
       </c>
       <c r="E108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Whole School</t>
+          <t xml:space="preserve">Secondary</t>
         </is>
       </c>
       <c r="F108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H108" t="inlineStr" s="2">
@@ -10501,22 +10501,22 @@
       </c>
       <c r="I108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Parent Teacher Conferences</t>
+          <t xml:space="preserve">End of Term 3 Activity: G6-10</t>
         </is>
       </c>
       <c r="J108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">保護者面談</t>
+          <t xml:space="preserve">第3学期末行事：G6–10</t>
         </is>
       </c>
       <c r="K108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Parents meet one-on-one with each teacher to discuss their child's progress, strengths, and next steps. The school campus is closed to students on these days.</t>
+          <t xml:space="preserve">Students will take part in an off-campus day trip outside Nagoya to celebrate the end of Term 3.</t>
         </is>
       </c>
       <c r="L108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">保護者の皆様が各担当教員と個別に面談し、お子様の成長、強み、今後の課題についてお話しします。期間中、生徒は登校しません。</t>
+          <t xml:space="preserve">第3学期の終わりを祝い、名古屋近郊への日帰り校外活動に参加します。</t>
         </is>
       </c>
       <c r="M108" t="inlineStr" s="2">
@@ -10531,7 +10531,7 @@
       </c>
       <c r="O108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-06-22-parent-teacher-conferences.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-06-19-end-of-term-3-activity-g6-10.webp</t>
         </is>
       </c>
       <c r="P108" t="inlineStr" s="2">
@@ -10558,17 +10558,17 @@
     <row r="109">
       <c r="A109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2027-06-28-summer-school</t>
+          <t xml:space="preserve">2027-06-22-parent-teacher-conferences</t>
         </is>
       </c>
       <c r="B109" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-06-28</t>
+          <t xml:space="preserve">2027-06-22</t>
         </is>
       </c>
       <c r="C109" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-07-18</t>
+          <t xml:space="preserve">2027-06-23</t>
         </is>
       </c>
       <c r="D109" t="inlineStr" s="3">
@@ -10583,12 +10583,12 @@
       </c>
       <c r="F109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="G109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="H109" t="inlineStr" s="2">
@@ -10598,22 +10598,22 @@
       </c>
       <c r="I109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Summer School</t>
+          <t xml:space="preserve">Parent Teacher Conferences</t>
         </is>
       </c>
       <c r="J109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">サマースクール</t>
+          <t xml:space="preserve">保護者面談</t>
         </is>
       </c>
       <c r="K109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Participate in fun English style summer camps that challenge students and help foster friendships and connections with others.</t>
+          <t xml:space="preserve">Parents meet one-on-one with each teacher to discuss their child's progress, strengths, and next steps. The school campus is closed to students on these days.</t>
         </is>
       </c>
       <c r="L109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">英語で楽しく過ごすサマーキャンプに参加し、新たなことに挑戦しながら友情や人とのつながりを育みます。</t>
+          <t xml:space="preserve">保護者の皆様が各担当教員と個別に面談し、お子様の成長、強み、今後の課題についてお話しします。期間中、生徒は登校しません。</t>
         </is>
       </c>
       <c r="M109" t="inlineStr" s="2">
@@ -10628,7 +10628,7 @@
       </c>
       <c r="O109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2027-06-28-summer-school.webp</t>
+          <t xml:space="preserve">compass/images/events/2027-06-22-parent-teacher-conferences.webp</t>
         </is>
       </c>
       <c r="P109" t="inlineStr" s="2">
@@ -10655,95 +10655,192 @@
     <row r="110">
       <c r="A110" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">2027-06-28-summer-school</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">2027-06-28</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve">2027-07-18</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Whole School</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Summer School</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">サマースクール</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Participate in fun English style summer camps that challenge students and help foster friendships and connections with others.</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">英語で楽しく過ごすサマーキャンプに参加し、新たなことに挑戦しながら友情や人とのつながりを育みます。</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">compass/images/events/2027-06-28-summer-school.webp</t>
+        </is>
+      </c>
+      <c r="P110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="Q110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">2027-07-20-summer-school</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr" s="3">
+      <c r="B111" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-07-20</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr" s="3">
+      <c r="C111" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">2027-07-24</t>
         </is>
       </c>
-      <c r="D110" t="inlineStr" s="3">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E110" t="inlineStr" s="2">
+      <c r="D111" t="inlineStr" s="3">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Whole School</t>
         </is>
       </c>
-      <c r="F110" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G110" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H110" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="I110" t="inlineStr" s="2">
+      <c r="F111" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Summer School</t>
         </is>
       </c>
-      <c r="J110" t="inlineStr" s="2">
+      <c r="J111" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">サマースクール</t>
         </is>
       </c>
-      <c r="K110" t="inlineStr" s="2">
+      <c r="K111" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Participate in fun English style summer camps that challenge students and help foster friendships and connections with others.</t>
         </is>
       </c>
-      <c r="L110" t="inlineStr" s="2">
+      <c r="L111" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">英語で楽しく過ごすサマーキャンプに参加し、新たなことに挑戦しながら友情や人とのつながりを育みます。</t>
         </is>
       </c>
-      <c r="M110" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N110" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="O110" t="inlineStr" s="2">
+      <c r="M111" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N111" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O111" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">compass/images/events/2027-06-28-summer-school.webp</t>
         </is>
       </c>
-      <c r="P110" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="Q110" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="R110" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="S110" t="inlineStr" s="2">
+      <c r="P111" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="Q111" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R111" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S111" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -11068,7 +11165,7 @@
       </c>
       <c r="B12" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2027-01-08</t>
+          <t xml:space="preserve">2027-01-07</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="2">

</xml_diff>

<commit_message>
Move Nagoya University laboratory visit to 20 Oct (was 23 Oct)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/admin/EIS-Compass-events.xlsx
+++ b/admin/EIS-Compass-events.xlsx
@@ -2604,17 +2604,17 @@
     <row r="27">
       <c r="A27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2026-10-21-college-fair</t>
+          <t xml:space="preserve">2026-10-23-nagoya-university-biology-laboratory-visit</t>
         </is>
       </c>
       <c r="B27" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-10-21</t>
+          <t xml:space="preserve">2026-10-20</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-10-21</t>
+          <t xml:space="preserve">2026-10-20</t>
         </is>
       </c>
       <c r="D27" t="inlineStr" s="3">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="F27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G27" t="inlineStr" s="2">
@@ -2639,27 +2639,27 @@
       </c>
       <c r="H27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">changed</t>
         </is>
       </c>
       <c r="I27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">College Fair</t>
+          <t xml:space="preserve">Nagoya University Biology Laboratory Visit</t>
         </is>
       </c>
       <c r="J27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">大学進学フェア</t>
+          <t xml:space="preserve">名古屋大学 生物学研究室訪問</t>
         </is>
       </c>
       <c r="K27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">A special event where representatives from several international and Japanese universities visit our school to introduce their programs and admission opportunities. The fair is open to all students and parents, and students from other international schools in the area are also invited to attend.</t>
+          <t xml:space="preserve">Grade 11 and 12 Biology students will visit Nagoya University for a guided laboratory experience, connecting classroom learning with real-world scientific research.</t>
         </is>
       </c>
       <c r="L27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">国内外の複数の大学の担当者が来校し、各大学のプログラムや入学機会を紹介する特別イベントです。全生徒・保護者が参加でき、近隣のインターナショナルスクールの生徒もご招待しています。</t>
+          <t xml:space="preserve">11・12年生の生物履修者が名古屋大学を訪問し、研究室での体験を通して授業での学びと実際の科学研究を結びつけます。</t>
         </is>
       </c>
       <c r="M27" t="inlineStr" s="2">
@@ -2674,7 +2674,7 @@
       </c>
       <c r="O27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2026-10-21-college-fair.webp</t>
+          <t xml:space="preserve">compass/images/events/2026-10-23-nagoya-university-biology-laboratory-visit.webp</t>
         </is>
       </c>
       <c r="P27" t="inlineStr" s="2">
@@ -2701,17 +2701,17 @@
     <row r="28">
       <c r="A28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2026-10-23-nagoya-university-biology-laboratory-visit</t>
+          <t xml:space="preserve">2026-10-21-college-fair</t>
         </is>
       </c>
       <c r="B28" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-10-23</t>
+          <t xml:space="preserve">2026-10-21</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">2026-10-23</t>
+          <t xml:space="preserve">2026-10-21</t>
         </is>
       </c>
       <c r="D28" t="inlineStr" s="3">
@@ -2726,7 +2726,7 @@
       </c>
       <c r="F28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="G28" t="inlineStr" s="2">
@@ -2741,22 +2741,22 @@
       </c>
       <c r="I28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Nagoya University Biology Laboratory Visit</t>
+          <t xml:space="preserve">College Fair</t>
         </is>
       </c>
       <c r="J28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">名古屋大学 生物学研究室訪問</t>
+          <t xml:space="preserve">大学進学フェア</t>
         </is>
       </c>
       <c r="K28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Grade 11 and 12 Biology students will visit Nagoya University for a guided laboratory experience, connecting classroom learning with real-world scientific research.</t>
+          <t xml:space="preserve">A special event where representatives from several international and Japanese universities visit our school to introduce their programs and admission opportunities. The fair is open to all students and parents, and students from other international schools in the area are also invited to attend.</t>
         </is>
       </c>
       <c r="L28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">11・12年生の生物履修者が名古屋大学を訪問し、研究室での体験を通して授業での学びと実際の科学研究を結びつけます。</t>
+          <t xml:space="preserve">国内外の複数の大学の担当者が来校し、各大学のプログラムや入学機会を紹介する特別イベントです。全生徒・保護者が参加でき、近隣のインターナショナルスクールの生徒もご招待しています。</t>
         </is>
       </c>
       <c r="M28" t="inlineStr" s="2">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="O28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">compass/images/events/2026-10-23-nagoya-university-biology-laboratory-visit.webp</t>
+          <t xml:space="preserve">compass/images/events/2026-10-21-college-fair.webp</t>
         </is>
       </c>
       <c r="P28" t="inlineStr" s="2">

</xml_diff>

<commit_message>
Update 24 Nov event: ELC & Primary Art Showcase
New title, parent viewing 13:10-14:45 (event 13:05-15:15), School Gym,
participants ELC to Grade 5, full EN/JA description from the parent
announcement (student voting, no stickers for parents).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/admin/EIS-Compass-events.xlsx
+++ b/admin/EIS-Compass-events.xlsx
@@ -4700,7 +4700,7 @@
       </c>
       <c r="D44" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">13:10-14:55</t>
+          <t xml:space="preserve">13:10-14:45</t>
         </is>
       </c>
       <c r="E44" t="inlineStr" s="2">
@@ -4710,12 +4710,12 @@
       </c>
       <c r="F44" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ELC to Grade 5</t>
         </is>
       </c>
       <c r="G44" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">幼稚部〜小学5年生</t>
         </is>
       </c>
       <c r="H44" t="inlineStr" s="2">
@@ -4735,27 +4735,27 @@
       </c>
       <c r="K44" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Gallery Day: ELC &amp; Primary Art Showcase</t>
+          <t xml:space="preserve">ELC &amp; Primary Art Showcase</t>
         </is>
       </c>
       <c r="L44" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ギャラリーデー：幼稚部・小学部アート展</t>
+          <t xml:space="preserve">幼稚部・小学部アート展</t>
         </is>
       </c>
       <c r="M44" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ELC and Primary students display the artwork they have created with the visual arts teacher. Parents are welcome to view the gallery from 13:10 to 14:55. Students vote for their favourite artworks, and the winners for each grade are announced.</t>
+          <t xml:space="preserve">Enishi’s first-ever Art Showcase! Students from ELC through Grade 5 exhibit the artwork they created during Term 1. Walk through the gallery at your own pace, appreciate the artworks, and feel free to ask students about their creative process and inspiration. Parent viewing: 13:10–14:45 (event 13:05–15:15). Students will vote for their favourite artwork from other grade levels, and one outstanding artwork from each grade will receive a set of art-supply prizes. Voting is for students only — parents and guardians are welcome to enjoy all the artwork, but please do not place voting stickers on any artwork.</t>
         </is>
       </c>
       <c r="N44" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">幼稚部・小学部の児童が美術の授業で制作した作品を展示します。保護者の皆さまは13:10～14:55にご鑑賞いただけます。児童による投票を行い、学年ごとの受賞作品を発表します。</t>
+          <t xml:space="preserve">本校初のアート展を開催します！幼稚部から小学5年生までの子どもたちが、1学期に制作した作品を展示します。会場内はご自身のペースで自由にご覧いただけます。作品をじっくり鑑賞しながら、制作の過程や着想について、ぜひ子どもたちにお尋ねください。保護者鑑賞時間：13:10～14:45（開催時間 13:05～15:15）。子どもたちは他学年の作品の中からお気に入りの作品に投票し、各学年から優秀作品を1点ずつ選出して、受賞者には画材セットを贈呈します。投票は子どもたちのみを対象としています。保護者の皆様もぜひすべての作品をお楽しみください。ただし、作品に投票用シールを貼ることはご遠慮ください。</t>
         </is>
       </c>
       <c r="O44" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Gym</t>
+          <t xml:space="preserve">School Gym</t>
         </is>
       </c>
       <c r="P44" t="inlineStr" s="2">

</xml_diff>

<commit_message>
Add IMF brochure links (English and Japanese)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/admin/EIS-Compass-events.xlsx
+++ b/admin/EIS-Compass-events.xlsx
@@ -3486,12 +3486,12 @@
       </c>
       <c r="R32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Event brochure (English) | イベントパンフレット（英語） | https://drive.google.com/file/d/1iK0N-LadmFzOjYjQr4HX23_EzAvgl_oC/view?usp=sharing</t>
         </is>
       </c>
       <c r="S32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Event brochure (Japanese) | イベントパンフレット（日本語） | https://drive.google.com/file/d/19MKvjdYx80BMoxM6uG35rMK8YX3sWpXI/view?usp=sharing</t>
         </is>
       </c>
       <c r="T32" t="inlineStr" s="2">

</xml_diff>

<commit_message>
IMF: full programme, 9:45-13:50
Gates 9:45, booths 10:00-13:00, Haunted House 10:00-12:00, costume
parade, food trucks, final gym event 13:00-13:50, supervision rule
(EN/JA).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/admin/EIS-Compass-events.xlsx
+++ b/admin/EIS-Compass-events.xlsx
@@ -3416,7 +3416,7 @@
       </c>
       <c r="D32" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">10:00-14:00</t>
+          <t xml:space="preserve">9:45-13:50</t>
         </is>
       </c>
       <c r="E32" t="inlineStr" s="2">
@@ -3461,22 +3461,22 @@
       </c>
       <c r="M32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">This year’s theme is “Festivals and Holidays Around the World”. A Saturday family event celebrating traditions, cultures, stories, arts, music and celebrations from around the world, with student activities, cultural displays, performances, arts and crafts, and interactive booths. Clean-up runs from 14:00 to 15:00, and community members are welcome to help. ELC and Primary students must attend with a parent or guardian and may not be dropped off. School buses will not operate. More details will be shared soon.</t>
+          <t xml:space="preserve">This year’s theme is “Festivals and Holidays Around the World” — a celebration of the many traditions, celebrations and cultures in our school community. Gates open at 9:45 and the festival begins at 10:00. From 10:00 to 13:00, teachers and students run three booth sessions with games, crafts, cultural activities and hands-on experiences from around the world. The Haunted House is open from 10:00 to 12:00, and there will be a costume parade: students may wear traditional or cultural clothing, an outfit representing a festival or holiday, or a Halloween costume (dressing up is optional — regular clothes are very welcome). Food trucks and food prepared and sold by school parents will be available. From 13:00 to 13:50, everyone moves to the gym for the final event with games and dances. Please note that IMF is not a normal school day: ELC and Primary students must be accompanied and supervised by a parent or guardian throughout their visit and may not be dropped off and collected later. School buses will not operate.</t>
         </is>
       </c>
       <c r="N32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">今年のテーマは「世界の祭りと祝日」です。世界各地の伝統、文化、物語、芸術、音楽、お祝いを紹介する、土曜日のご家族参加型イベントです。児童・生徒の活動、文化展示、パフォーマンス、工作、体験型ブースをお楽しみいただけます。午後2時～3時に片付けを行います（学校コミュニティの皆さまのご協力も歓迎します）。幼稚部・小学部の児童は必ず保護者同伴でご参加ください（お子さまだけを送り届けることはできません）。当日はスクールバスの運行はありません。詳細は近日中にお知らせします。</t>
+          <t xml:space="preserve">今年のテーマは「世界の祝日とお祭り」です。学校コミュニティのさまざまな伝統、行事、文化をみんなで楽しくお祝いする一日です。9:45開門、10:00にフェスティバルが始まります。10:00～13:00には、教職員や生徒によるゲーム、クラフト、文化体験など、世界各地にちなんだ体験型ブースセッションを3回行います。お化け屋敷は10:00～12:00。仮装パレードでは、伝統衣装や民族衣装、祝日やお祭りを表す衣装、ハロウィンの仮装で参加できます（仮装は自由参加です。普段着での参加ももちろん歓迎します）。フードトラックの出店や、保護者の皆様による食べ物の販売もあります。13:00～13:50は体育館に移動し、ゲームやダンスの最終イベントを行います。IMFは通常の登校日ではありません。幼稚部・小学部の児童は、参加している間、必ず保護者または付き添いの大人と一緒に行動してください。お子様だけを学校に送り、後からお迎えに来ることはできません。当日はスクールバスの運行はありません。</t>
         </is>
       </c>
       <c r="O32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Enishi International School</t>
         </is>
       </c>
       <c r="P32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">エニシインターナショナルスクール</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr" s="2">

</xml_diff>